<commit_message>
PolyKybd: store real icon codepoints in lang_lut.xlsx (canonical de-PUA)
Update the 40 UI-icon rows in the named_glyphs sheet so column B holds the
real SMP codepoint (e.g. PRIVATE_WORLD E310 -> 1F310) instead of the legacy
BMP-PUA address. Edited surgically at the worksheet-XML level (only the
named_glyphs sheet) so the latin_sup_ex formula caches that cog reads stay
byte-identical; the C/D calc columns are recomputed to match.

With column B now canonical, the named_glyphs cog drops the +0x11000 PUA
remap and reads B directly. Generated named_glyphs.h is byte-identical, and
lang_lut.c / uni.h regenerate unchanged.

https://claude.ai/code/session_014g2hQRQQkpo5EEX3pPwM3o
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -24392,16 +24392,18 @@
       <c r="A749" s="7" t="s">
         <v>925</v>
       </c>
-      <c r="B749" s="8" t="s">
-        <v>926</v>
+      <c r="B749" s="8" t="inlineStr">
+        <is>
+          <t>1F300</t>
+        </is>
       </c>
       <c r="C749" s="7" t="n">
         <f aca="false">HEX2DEC(B749)</f>
-        <v>58112</v>
+        <v>127744</v>
       </c>
       <c r="D749" s="9" t="str">
         <f aca="false">DEC2HEX(C749,4)</f>
-        <v>E300</v>
+        <v>1F300</v>
       </c>
       <c r="E749" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C749)</f>
@@ -24409,7 +24411,7 @@
       </c>
       <c r="F749" s="7" t="n">
         <f aca="false">C749-C748</f>
-        <v>45572</v>
+        <v>115204</v>
       </c>
       <c r="G749" s="16" t="s">
         <v>927</v>
@@ -24419,16 +24421,18 @@
       <c r="A750" s="7" t="s">
         <v>928</v>
       </c>
-      <c r="B750" s="8" t="s">
-        <v>929</v>
+      <c r="B750" s="8" t="inlineStr">
+        <is>
+          <t>1F310</t>
+        </is>
       </c>
       <c r="C750" s="7" t="n">
         <f aca="false">HEX2DEC(B750)</f>
-        <v>58128</v>
+        <v>127760</v>
       </c>
       <c r="D750" s="9" t="str">
         <f aca="false">DEC2HEX(C750,4)</f>
-        <v>E310</v>
+        <v>1F310</v>
       </c>
       <c r="E750" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C750)</f>
@@ -24444,16 +24448,18 @@
       <c r="A751" s="7" t="s">
         <v>930</v>
       </c>
-      <c r="B751" s="8" t="s">
-        <v>931</v>
+      <c r="B751" s="8" t="inlineStr">
+        <is>
+          <t>1F311</t>
+        </is>
       </c>
       <c r="C751" s="7" t="n">
         <f aca="false">HEX2DEC(B751)</f>
-        <v>58129</v>
+        <v>127761</v>
       </c>
       <c r="D751" s="9" t="str">
         <f aca="false">DEC2HEX(C751,4)</f>
-        <v>E311</v>
+        <v>1F311</v>
       </c>
       <c r="E751" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C751)</f>
@@ -24469,16 +24475,18 @@
       <c r="A752" s="7" t="s">
         <v>932</v>
       </c>
-      <c r="B752" s="8" t="s">
-        <v>933</v>
+      <c r="B752" s="8" t="inlineStr">
+        <is>
+          <t>1F315</t>
+        </is>
       </c>
       <c r="C752" s="7" t="n">
         <f aca="false">HEX2DEC(B752)</f>
-        <v>58133</v>
+        <v>127765</v>
       </c>
       <c r="D752" s="9" t="str">
         <f aca="false">DEC2HEX(C752,4)</f>
-        <v>E315</v>
+        <v>1F315</v>
       </c>
       <c r="E752" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C752)</f>
@@ -24494,16 +24502,18 @@
       <c r="A753" s="7" t="s">
         <v>934</v>
       </c>
-      <c r="B753" s="8" t="s">
-        <v>935</v>
+      <c r="B753" s="8" t="inlineStr">
+        <is>
+          <t>1F316</t>
+        </is>
       </c>
       <c r="C753" s="7" t="n">
         <f aca="false">HEX2DEC(B753)</f>
-        <v>58134</v>
+        <v>127766</v>
       </c>
       <c r="D753" s="9" t="str">
         <f aca="false">DEC2HEX(C753,4)</f>
-        <v>E316</v>
+        <v>1F316</v>
       </c>
       <c r="E753" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C753)</f>
@@ -24519,16 +24529,18 @@
       <c r="A754" s="7" t="s">
         <v>936</v>
       </c>
-      <c r="B754" s="8" t="s">
-        <v>937</v>
+      <c r="B754" s="8" t="inlineStr">
+        <is>
+          <t>1F317</t>
+        </is>
       </c>
       <c r="C754" s="7" t="n">
         <f aca="false">HEX2DEC(B754)</f>
-        <v>58135</v>
+        <v>127767</v>
       </c>
       <c r="D754" s="9" t="str">
         <f aca="false">DEC2HEX(C754,4)</f>
-        <v>E317</v>
+        <v>1F317</v>
       </c>
       <c r="E754" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C754)</f>
@@ -24544,16 +24556,18 @@
       <c r="A755" s="7" t="s">
         <v>938</v>
       </c>
-      <c r="B755" s="8" t="s">
-        <v>939</v>
+      <c r="B755" s="8" t="inlineStr">
+        <is>
+          <t>1F318</t>
+        </is>
       </c>
       <c r="C755" s="7" t="n">
         <f aca="false">HEX2DEC(B755)</f>
-        <v>58136</v>
+        <v>127768</v>
       </c>
       <c r="D755" s="9" t="str">
         <f aca="false">DEC2HEX(C755,4)</f>
-        <v>E318</v>
+        <v>1F318</v>
       </c>
       <c r="E755" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C755)</f>
@@ -24569,16 +24583,18 @@
       <c r="A756" s="7" t="s">
         <v>940</v>
       </c>
-      <c r="B756" s="8" t="s">
-        <v>941</v>
+      <c r="B756" s="8" t="inlineStr">
+        <is>
+          <t>1F3E0</t>
+        </is>
       </c>
       <c r="C756" s="7" t="n">
         <f aca="false">HEX2DEC(B756)</f>
-        <v>58336</v>
+        <v>127968</v>
       </c>
       <c r="D756" s="9" t="str">
         <f aca="false">DEC2HEX(C756,4)</f>
-        <v>E3E0</v>
+        <v>1F3E0</v>
       </c>
       <c r="E756" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C756)</f>
@@ -24594,16 +24610,18 @@
       <c r="A757" s="7" t="s">
         <v>942</v>
       </c>
-      <c r="B757" s="8" t="s">
-        <v>943</v>
+      <c r="B757" s="8" t="inlineStr">
+        <is>
+          <t>1F410</t>
+        </is>
       </c>
       <c r="C757" s="7" t="n">
         <f aca="false">HEX2DEC(B757)</f>
-        <v>58384</v>
+        <v>128016</v>
       </c>
       <c r="D757" s="9" t="str">
         <f aca="false">DEC2HEX(C757,4)</f>
-        <v>E410</v>
+        <v>1F410</v>
       </c>
       <c r="E757" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C757)</f>
@@ -24619,16 +24637,18 @@
       <c r="A758" s="7" t="s">
         <v>944</v>
       </c>
-      <c r="B758" s="8" t="s">
-        <v>945</v>
+      <c r="B758" s="8" t="inlineStr">
+        <is>
+          <t>1F4A1</t>
+        </is>
       </c>
       <c r="C758" s="7" t="n">
         <f aca="false">HEX2DEC(B758)</f>
-        <v>58529</v>
+        <v>128161</v>
       </c>
       <c r="D758" s="9" t="str">
         <f aca="false">DEC2HEX(C758,4)</f>
-        <v>E4A1</v>
+        <v>1F4A1</v>
       </c>
       <c r="E758" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C758)</f>
@@ -24644,16 +24664,18 @@
       <c r="A759" s="7" t="s">
         <v>946</v>
       </c>
-      <c r="B759" s="8" t="s">
-        <v>947</v>
+      <c r="B759" s="8" t="inlineStr">
+        <is>
+          <t>1F4AB</t>
+        </is>
       </c>
       <c r="C759" s="7" t="n">
         <f aca="false">HEX2DEC(B759)</f>
-        <v>58539</v>
+        <v>128171</v>
       </c>
       <c r="D759" s="9" t="str">
         <f aca="false">DEC2HEX(C759,4)</f>
-        <v>E4AB</v>
+        <v>1F4AB</v>
       </c>
       <c r="E759" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C759)</f>
@@ -24669,16 +24691,18 @@
       <c r="A760" s="7" t="s">
         <v>948</v>
       </c>
-      <c r="B760" s="11" t="s">
-        <v>949</v>
+      <c r="B760" s="11" t="inlineStr">
+        <is>
+          <t>1F4C2</t>
+        </is>
       </c>
       <c r="C760" s="7" t="n">
         <f aca="false">HEX2DEC(B760)</f>
-        <v>58562</v>
+        <v>128194</v>
       </c>
       <c r="D760" s="9" t="str">
         <f aca="false">DEC2HEX(C760,4)</f>
-        <v>E4C2</v>
+        <v>1F4C2</v>
       </c>
       <c r="E760" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C760)</f>
@@ -24694,16 +24718,18 @@
       <c r="A761" s="7" t="s">
         <v>950</v>
       </c>
-      <c r="B761" s="11" t="s">
-        <v>951</v>
+      <c r="B761" s="11" t="inlineStr">
+        <is>
+          <t>1F4CB</t>
+        </is>
       </c>
       <c r="C761" s="7" t="n">
         <f aca="false">HEX2DEC(B761)</f>
-        <v>58571</v>
+        <v>128203</v>
       </c>
       <c r="D761" s="9" t="str">
         <f aca="false">DEC2HEX(C761,4)</f>
-        <v>E4CB</v>
+        <v>1F4CB</v>
       </c>
       <c r="E761" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C761)</f>
@@ -24719,16 +24745,18 @@
       <c r="A762" s="7" t="s">
         <v>952</v>
       </c>
-      <c r="B762" s="8" t="s">
-        <v>953</v>
+      <c r="B762" s="8" t="inlineStr">
+        <is>
+          <t>1F4DD</t>
+        </is>
       </c>
       <c r="C762" s="7" t="n">
         <f aca="false">HEX2DEC(B762)</f>
-        <v>58589</v>
+        <v>128221</v>
       </c>
       <c r="D762" s="9" t="str">
         <f aca="false">DEC2HEX(C762,4)</f>
-        <v>E4DD</v>
+        <v>1F4DD</v>
       </c>
       <c r="E762" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C762)</f>
@@ -24744,16 +24772,18 @@
       <c r="A763" s="7" t="s">
         <v>954</v>
       </c>
-      <c r="B763" s="11" t="s">
-        <v>955</v>
+      <c r="B763" s="11" t="inlineStr">
+        <is>
+          <t>1F50E</t>
+        </is>
       </c>
       <c r="C763" s="7" t="n">
         <f aca="false">HEX2DEC(B763)</f>
-        <v>58638</v>
+        <v>128270</v>
       </c>
       <c r="D763" s="9" t="str">
         <f aca="false">DEC2HEX(C763,4)</f>
-        <v>E50E</v>
+        <v>1F50E</v>
       </c>
       <c r="E763" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C763)</f>
@@ -24769,16 +24799,18 @@
       <c r="A764" s="7" t="s">
         <v>956</v>
       </c>
-      <c r="B764" s="8" t="s">
-        <v>957</v>
+      <c r="B764" s="8" t="inlineStr">
+        <is>
+          <t>1F512</t>
+        </is>
       </c>
       <c r="C764" s="7" t="n">
         <f aca="false">HEX2DEC(B764)</f>
-        <v>58642</v>
+        <v>128274</v>
       </c>
       <c r="D764" s="9" t="str">
         <f aca="false">DEC2HEX(C764,4)</f>
-        <v>E512</v>
+        <v>1F512</v>
       </c>
       <c r="E764" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C764)</f>
@@ -24794,16 +24826,18 @@
       <c r="A765" s="7" t="s">
         <v>958</v>
       </c>
-      <c r="B765" s="8" t="s">
-        <v>959</v>
+      <c r="B765" s="8" t="inlineStr">
+        <is>
+          <t>1F527</t>
+        </is>
       </c>
       <c r="C765" s="7" t="n">
         <f aca="false">HEX2DEC(B765)</f>
-        <v>58663</v>
+        <v>128295</v>
       </c>
       <c r="D765" s="9" t="str">
         <f aca="false">DEC2HEX(C765,4)</f>
-        <v>E527</v>
+        <v>1F527</v>
       </c>
       <c r="E765" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C765)</f>
@@ -24819,16 +24853,18 @@
       <c r="A766" s="7" t="s">
         <v>960</v>
       </c>
-      <c r="B766" s="11" t="s">
-        <v>961</v>
+      <c r="B766" s="11" t="inlineStr">
+        <is>
+          <t>1F568</t>
+        </is>
       </c>
       <c r="C766" s="7" t="n">
         <f aca="false">HEX2DEC(B766)</f>
-        <v>58728</v>
+        <v>128360</v>
       </c>
       <c r="D766" s="9" t="str">
         <f aca="false">DEC2HEX(C766,4)</f>
-        <v>E568</v>
+        <v>1F568</v>
       </c>
       <c r="E766" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C766)</f>
@@ -24844,16 +24880,18 @@
       <c r="A767" s="7" t="s">
         <v>962</v>
       </c>
-      <c r="B767" s="8" t="s">
-        <v>963</v>
+      <c r="B767" s="8" t="inlineStr">
+        <is>
+          <t>1F569</t>
+        </is>
       </c>
       <c r="C767" s="7" t="n">
         <f aca="false">HEX2DEC(B767)</f>
-        <v>58729</v>
+        <v>128361</v>
       </c>
       <c r="D767" s="9" t="str">
         <f aca="false">DEC2HEX(C767,4)</f>
-        <v>E569</v>
+        <v>1F569</v>
       </c>
       <c r="E767" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C767)</f>
@@ -24869,16 +24907,18 @@
       <c r="A768" s="7" t="s">
         <v>964</v>
       </c>
-      <c r="B768" s="8" t="s">
-        <v>965</v>
+      <c r="B768" s="8" t="inlineStr">
+        <is>
+          <t>1F56A</t>
+        </is>
       </c>
       <c r="C768" s="7" t="n">
         <f aca="false">HEX2DEC(B768)</f>
-        <v>58730</v>
+        <v>128362</v>
       </c>
       <c r="D768" s="9" t="str">
         <f aca="false">DEC2HEX(C768,4)</f>
-        <v>E56A</v>
+        <v>1F56A</v>
       </c>
       <c r="E768" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C768)</f>
@@ -24894,16 +24934,18 @@
       <c r="A769" s="7" t="s">
         <v>966</v>
       </c>
-      <c r="B769" s="8" t="s">
-        <v>967</v>
+      <c r="B769" s="8" t="inlineStr">
+        <is>
+          <t>1F5A9</t>
+        </is>
       </c>
       <c r="C769" s="7" t="n">
         <f aca="false">HEX2DEC(B769)</f>
-        <v>58793</v>
+        <v>128425</v>
       </c>
       <c r="D769" s="9" t="str">
         <f aca="false">DEC2HEX(C769,4)</f>
-        <v>E5A9</v>
+        <v>1F5A9</v>
       </c>
       <c r="E769" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C769)</f>
@@ -24919,16 +24961,18 @@
       <c r="A770" s="7" t="s">
         <v>968</v>
       </c>
-      <c r="B770" s="8" t="s">
-        <v>969</v>
+      <c r="B770" s="8" t="inlineStr">
+        <is>
+          <t>1F5AB</t>
+        </is>
       </c>
       <c r="C770" s="7" t="n">
         <f aca="false">HEX2DEC(B770)</f>
-        <v>58795</v>
+        <v>128427</v>
       </c>
       <c r="D770" s="9" t="str">
         <f aca="false">DEC2HEX(C770,4)</f>
-        <v>E5AB</v>
+        <v>1F5AB</v>
       </c>
       <c r="E770" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C770)</f>
@@ -24944,16 +24988,18 @@
       <c r="A771" s="7" t="s">
         <v>970</v>
       </c>
-      <c r="B771" s="11" t="s">
-        <v>971</v>
+      <c r="B771" s="11" t="inlineStr">
+        <is>
+          <t>1F5B3</t>
+        </is>
       </c>
       <c r="C771" s="7" t="n">
         <f aca="false">HEX2DEC(B771)</f>
-        <v>58803</v>
+        <v>128435</v>
       </c>
       <c r="D771" s="9" t="str">
         <f aca="false">DEC2HEX(C771,4)</f>
-        <v>E5B3</v>
+        <v>1F5B3</v>
       </c>
       <c r="E771" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C771)</f>
@@ -24969,16 +25015,18 @@
       <c r="A772" s="7" t="s">
         <v>972</v>
       </c>
-      <c r="B772" s="8" t="s">
-        <v>973</v>
+      <c r="B772" s="8" t="inlineStr">
+        <is>
+          <t>1F5B4</t>
+        </is>
       </c>
       <c r="C772" s="7" t="n">
         <f aca="false">HEX2DEC(B772)</f>
-        <v>58804</v>
+        <v>128436</v>
       </c>
       <c r="D772" s="9" t="str">
         <f aca="false">DEC2HEX(C772,4)</f>
-        <v>E5B4</v>
+        <v>1F5B4</v>
       </c>
       <c r="E772" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C772)</f>
@@ -24994,16 +25042,18 @@
       <c r="A773" s="7" t="s">
         <v>974</v>
       </c>
-      <c r="B773" s="8" t="s">
-        <v>975</v>
+      <c r="B773" s="8" t="inlineStr">
+        <is>
+          <t>1F5B5</t>
+        </is>
       </c>
       <c r="C773" s="7" t="n">
         <f aca="false">HEX2DEC(B773)</f>
-        <v>58805</v>
+        <v>128437</v>
       </c>
       <c r="D773" s="9" t="str">
         <f aca="false">DEC2HEX(C773,4)</f>
-        <v>E5B5</v>
+        <v>1F5B5</v>
       </c>
       <c r="E773" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C773)</f>
@@ -25019,16 +25069,18 @@
       <c r="A774" s="7" t="s">
         <v>976</v>
       </c>
-      <c r="B774" s="8" t="s">
-        <v>977</v>
+      <c r="B774" s="8" t="inlineStr">
+        <is>
+          <t>1F5B6</t>
+        </is>
       </c>
       <c r="C774" s="7" t="n">
         <f aca="false">HEX2DEC(B774)</f>
-        <v>58806</v>
+        <v>128438</v>
       </c>
       <c r="D774" s="9" t="str">
         <f aca="false">DEC2HEX(C774,4)</f>
-        <v>E5B6</v>
+        <v>1F5B6</v>
       </c>
       <c r="E774" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C774)</f>
@@ -25044,16 +25096,18 @@
       <c r="A775" s="7" t="s">
         <v>978</v>
       </c>
-      <c r="B775" s="8" t="s">
-        <v>979</v>
+      <c r="B775" s="8" t="inlineStr">
+        <is>
+          <t>1F5B7</t>
+        </is>
       </c>
       <c r="C775" s="7" t="n">
         <f aca="false">HEX2DEC(B775)</f>
-        <v>58807</v>
+        <v>128439</v>
       </c>
       <c r="D775" s="9" t="str">
         <f aca="false">DEC2HEX(C775,4)</f>
-        <v>E5B7</v>
+        <v>1F5B7</v>
       </c>
       <c r="E775" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C775)</f>
@@ -25069,16 +25123,18 @@
       <c r="A776" s="7" t="s">
         <v>980</v>
       </c>
-      <c r="B776" s="8" t="s">
-        <v>981</v>
+      <c r="B776" s="8" t="inlineStr">
+        <is>
+          <t>1F5B8</t>
+        </is>
       </c>
       <c r="C776" s="7" t="n">
         <f aca="false">HEX2DEC(B776)</f>
-        <v>58808</v>
+        <v>128440</v>
       </c>
       <c r="D776" s="9" t="str">
         <f aca="false">DEC2HEX(C776,4)</f>
-        <v>E5B8</v>
+        <v>1F5B8</v>
       </c>
       <c r="E776" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C776)</f>
@@ -25094,16 +25150,18 @@
       <c r="A777" s="7" t="s">
         <v>982</v>
       </c>
-      <c r="B777" s="8" t="s">
-        <v>983</v>
+      <c r="B777" s="8" t="inlineStr">
+        <is>
+          <t>1F5B9</t>
+        </is>
       </c>
       <c r="C777" s="7" t="n">
         <f aca="false">HEX2DEC(B777)</f>
-        <v>58809</v>
+        <v>128441</v>
       </c>
       <c r="D777" s="9" t="str">
         <f aca="false">DEC2HEX(C777,4)</f>
-        <v>E5B9</v>
+        <v>1F5B9</v>
       </c>
       <c r="E777" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C777)</f>
@@ -25119,16 +25177,18 @@
       <c r="A778" s="7" t="s">
         <v>984</v>
       </c>
-      <c r="B778" s="8" t="s">
-        <v>985</v>
+      <c r="B778" s="8" t="inlineStr">
+        <is>
+          <t>1F5BA</t>
+        </is>
       </c>
       <c r="C778" s="7" t="n">
         <f aca="false">HEX2DEC(B778)</f>
-        <v>58810</v>
+        <v>128442</v>
       </c>
       <c r="D778" s="9" t="str">
         <f aca="false">DEC2HEX(C778,4)</f>
-        <v>E5BA</v>
+        <v>1F5BA</v>
       </c>
       <c r="E778" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C778)</f>
@@ -25144,16 +25204,18 @@
       <c r="A779" s="7" t="s">
         <v>986</v>
       </c>
-      <c r="B779" s="8" t="s">
-        <v>987</v>
+      <c r="B779" s="8" t="inlineStr">
+        <is>
+          <t>1F5BB</t>
+        </is>
       </c>
       <c r="C779" s="7" t="n">
         <f aca="false">HEX2DEC(B779)</f>
-        <v>58811</v>
+        <v>128443</v>
       </c>
       <c r="D779" s="9" t="str">
         <f aca="false">DEC2HEX(C779,4)</f>
-        <v>E5BB</v>
+        <v>1F5BB</v>
       </c>
       <c r="E779" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C779)</f>
@@ -25169,16 +25231,18 @@
       <c r="A780" s="7" t="s">
         <v>988</v>
       </c>
-      <c r="B780" s="8" t="s">
-        <v>989</v>
+      <c r="B780" s="8" t="inlineStr">
+        <is>
+          <t>1F5BC</t>
+        </is>
       </c>
       <c r="C780" s="7" t="n">
         <f aca="false">HEX2DEC(B780)</f>
-        <v>58812</v>
+        <v>128444</v>
       </c>
       <c r="D780" s="9" t="str">
         <f aca="false">DEC2HEX(C780,4)</f>
-        <v>E5BC</v>
+        <v>1F5BC</v>
       </c>
       <c r="E780" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C780)</f>
@@ -25194,16 +25258,18 @@
       <c r="A781" s="7" t="s">
         <v>990</v>
       </c>
-      <c r="B781" s="11" t="s">
-        <v>991</v>
+      <c r="B781" s="11" t="inlineStr">
+        <is>
+          <t>1F5CA</t>
+        </is>
       </c>
       <c r="C781" s="7" t="n">
         <f aca="false">HEX2DEC(B781)</f>
-        <v>58826</v>
+        <v>128458</v>
       </c>
       <c r="D781" s="9" t="str">
         <f aca="false">DEC2HEX(C781,4)</f>
-        <v>E5CA</v>
+        <v>1F5CA</v>
       </c>
       <c r="E781" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C781)</f>
@@ -25219,16 +25285,18 @@
       <c r="A782" s="7" t="s">
         <v>992</v>
       </c>
-      <c r="B782" s="11" t="s">
-        <v>993</v>
+      <c r="B782" s="11" t="inlineStr">
+        <is>
+          <t>1F5D5</t>
+        </is>
       </c>
       <c r="C782" s="7" t="n">
         <f aca="false">HEX2DEC(B782)</f>
-        <v>58837</v>
+        <v>128469</v>
       </c>
       <c r="D782" s="9" t="str">
         <f aca="false">DEC2HEX(C782,4)</f>
-        <v>E5D5</v>
+        <v>1F5D5</v>
       </c>
       <c r="E782" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C782)</f>
@@ -25244,16 +25312,18 @@
       <c r="A783" s="7" t="s">
         <v>994</v>
       </c>
-      <c r="B783" s="8" t="s">
-        <v>995</v>
+      <c r="B783" s="8" t="inlineStr">
+        <is>
+          <t>1F5D6</t>
+        </is>
       </c>
       <c r="C783" s="7" t="n">
         <f aca="false">HEX2DEC(B783)</f>
-        <v>58838</v>
+        <v>128470</v>
       </c>
       <c r="D783" s="9" t="str">
         <f aca="false">DEC2HEX(C783,4)</f>
-        <v>E5D6</v>
+        <v>1F5D6</v>
       </c>
       <c r="E783" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C783)</f>
@@ -25269,16 +25339,18 @@
       <c r="A784" s="7" t="s">
         <v>996</v>
       </c>
-      <c r="B784" s="11" t="s">
-        <v>997</v>
+      <c r="B784" s="11" t="inlineStr">
+        <is>
+          <t>1F5D7</t>
+        </is>
       </c>
       <c r="C784" s="7" t="n">
         <f aca="false">HEX2DEC(B784)</f>
-        <v>58839</v>
+        <v>128471</v>
       </c>
       <c r="D784" s="9" t="str">
         <f aca="false">DEC2HEX(C784,4)</f>
-        <v>E5D7</v>
+        <v>1F5D7</v>
       </c>
       <c r="E784" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C784)</f>
@@ -25294,16 +25366,18 @@
       <c r="A785" s="7" t="s">
         <v>998</v>
       </c>
-      <c r="B785" s="8" t="s">
-        <v>999</v>
+      <c r="B785" s="8" t="inlineStr">
+        <is>
+          <t>1F5D8</t>
+        </is>
       </c>
       <c r="C785" s="7" t="n">
         <f aca="false">HEX2DEC(B785)</f>
-        <v>58840</v>
+        <v>128472</v>
       </c>
       <c r="D785" s="9" t="str">
         <f aca="false">DEC2HEX(C785,4)</f>
-        <v>E5D8</v>
+        <v>1F5D8</v>
       </c>
       <c r="E785" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C785)</f>
@@ -25319,16 +25393,18 @@
       <c r="A786" s="7" t="s">
         <v>1000</v>
       </c>
-      <c r="B786" s="11" t="s">
-        <v>1001</v>
+      <c r="B786" s="11" t="inlineStr">
+        <is>
+          <t>1F5D9</t>
+        </is>
       </c>
       <c r="C786" s="7" t="n">
         <f aca="false">HEX2DEC(B786)</f>
-        <v>58841</v>
+        <v>128473</v>
       </c>
       <c r="D786" s="9" t="str">
         <f aca="false">DEC2HEX(C786,4)</f>
-        <v>E5D9</v>
+        <v>1F5D9</v>
       </c>
       <c r="E786" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C786)</f>
@@ -25344,16 +25420,18 @@
       <c r="A787" s="7" t="s">
         <v>1002</v>
       </c>
-      <c r="B787" s="8" t="s">
-        <v>1003</v>
+      <c r="B787" s="8" t="inlineStr">
+        <is>
+          <t>1F5DA</t>
+        </is>
       </c>
       <c r="C787" s="7" t="n">
         <f aca="false">HEX2DEC(B787)</f>
-        <v>58842</v>
+        <v>128474</v>
       </c>
       <c r="D787" s="9" t="str">
         <f aca="false">DEC2HEX(C787,4)</f>
-        <v>E5DA</v>
+        <v>1F5DA</v>
       </c>
       <c r="E787" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C787)</f>
@@ -25369,16 +25447,18 @@
       <c r="A788" s="7" t="s">
         <v>1004</v>
       </c>
-      <c r="B788" s="11" t="s">
-        <v>1005</v>
+      <c r="B788" s="11" t="inlineStr">
+        <is>
+          <t>1F5DB</t>
+        </is>
       </c>
       <c r="C788" s="7" t="n">
         <f aca="false">HEX2DEC(B788)</f>
-        <v>58843</v>
+        <v>128475</v>
       </c>
       <c r="D788" s="9" t="str">
         <f aca="false">DEC2HEX(C788,4)</f>
-        <v>E5DB</v>
+        <v>1F5DB</v>
       </c>
       <c r="E788" s="10" t="str">
         <f aca="false">_xlfn.UNICHAR(C788)</f>

</xml_diff>

<commit_message>
polykybd: add Croatian (hr) keyboard layout + future-variant notes
First layout of the language-expansion batch. Croatian is the ex-Yugoslav Latin
QWERTZ (Gajica) and the fold parent for Bosnian/Montenegrin/Slovenian (handled
host-side). Added via a surgical key_lut-sheet edit that preserves every formula
cache in lang_lut.xlsx (verified: all 27 existing languages regenerate
byte-identically apart from cs-CZ gaining a trailing comma). lang_lut.c/.h
regenerated with cog; HR appended to gen-lang-fonts.sh COUNTRIES (flag_fonts.h
regen deferred to the end of the batch). FUTURE_LANGUAGES.md: documented the
regional variants (latam/ch/be/gb/ca-fr) that need their own entries, not folds.

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -30588,7 +30588,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:DE79"/>
+  <dimension ref="A1:DI79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -30843,6 +30843,11 @@
       <c r="DE1" s="63" t="n">
         <v>1029</v>
       </c>
+      <c r="DF1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hr-HR</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -31173,6 +31178,11 @@
       <c r="DE3" s="115" t="s">
         <v>1137</v>
       </c>
+      <c r="DI3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -31708,6 +31718,11 @@
       <c r="DE6" s="115" t="s">
         <v>682</v>
       </c>
+      <c r="DI6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
     </row>
     <row r="7" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="93" t="s">
@@ -31871,6 +31886,11 @@
       <c r="DE7" s="115" t="s">
         <v>1154</v>
       </c>
+      <c r="DI7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -32032,6 +32052,11 @@
       <c r="DE8" s="115" t="s">
         <v>1145</v>
       </c>
+      <c r="DI8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -33203,6 +33228,11 @@
       <c r="DE15" s="115" t="s">
         <v>1185</v>
       </c>
+      <c r="DI15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">}</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -33722,6 +33752,11 @@
       <c r="DE18" s="115" t="s">
         <v>16</v>
       </c>
+      <c r="DI18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BACKSLASH</t>
+        </is>
+      </c>
     </row>
     <row r="19" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="93" t="s">
@@ -34551,6 +34586,11 @@
       <c r="DE23" s="115" t="s">
         <v>1195</v>
       </c>
+      <c r="DI23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -34727,6 +34767,11 @@
       <c r="DD24" s="115"/>
       <c r="DE24" s="115" t="s">
         <v>1224</v>
+      </c>
+      <c r="DI24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|</t>
+        </is>
       </c>
     </row>
     <row r="25" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35072,6 +35117,16 @@
       </c>
       <c r="DD26" s="115"/>
       <c r="DE26" s="115"/>
+      <c r="DF26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z</t>
+        </is>
+      </c>
+      <c r="DG26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Z</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -35255,6 +35310,16 @@
       </c>
       <c r="DD27" s="115"/>
       <c r="DE27" s="115"/>
+      <c r="DF27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y</t>
+        </is>
+      </c>
+      <c r="DG27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -35533,6 +35598,22 @@
       </c>
       <c r="DE28" s="115" t="s">
         <v>198</v>
+      </c>
+      <c r="DF28">
+        <v>1</v>
+      </c>
+      <c r="DG28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="DH28">
+        <v>1</v>
+      </c>
+      <c r="DI28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_TILDE</t>
+        </is>
       </c>
     </row>
     <row r="29" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35829,6 +35910,22 @@
       <c r="DE29" s="115" t="s">
         <v>1241</v>
       </c>
+      <c r="DF29">
+        <v>2</v>
+      </c>
+      <c r="DG29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"</t>
+        </is>
+      </c>
+      <c r="DH29">
+        <v>2</v>
+      </c>
+      <c r="DI29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_CARON</t>
+        </is>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -36126,6 +36223,22 @@
       <c r="DE30" s="115" t="s">
         <v>1245</v>
       </c>
+      <c r="DF30">
+        <v>3</v>
+      </c>
+      <c r="DG30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="DH30">
+        <v>3</v>
+      </c>
+      <c r="DI30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -36423,6 +36536,22 @@
       <c r="DE31" s="115" t="s">
         <v>190</v>
       </c>
+      <c r="DF31">
+        <v>4</v>
+      </c>
+      <c r="DG31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="DH31">
+        <v>4</v>
+      </c>
+      <c r="DI31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_BREVE</t>
+        </is>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -36720,6 +36849,22 @@
       <c r="DE32" s="115" t="s">
         <v>194</v>
       </c>
+      <c r="DF32">
+        <v>5</v>
+      </c>
+      <c r="DG32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="DH32">
+        <v>5</v>
+      </c>
+      <c r="DI32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_RING</t>
+        </is>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -37005,6 +37150,22 @@
       <c r="DE33" s="127" t="s">
         <v>196</v>
       </c>
+      <c r="DF33">
+        <v>6</v>
+      </c>
+      <c r="DG33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="DH33">
+        <v>6</v>
+      </c>
+      <c r="DI33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_OGONEK</t>
+        </is>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -37299,6 +37460,22 @@
       </c>
       <c r="DE34" s="115" t="s">
         <v>1268</v>
+      </c>
+      <c r="DF34">
+        <v>7</v>
+      </c>
+      <c r="DG34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="DH34">
+        <v>7</v>
+      </c>
+      <c r="DI34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
+        </is>
       </c>
     </row>
     <row r="35" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37595,6 +37772,22 @@
       <c r="DE35" s="127" t="s">
         <v>192</v>
       </c>
+      <c r="DF35">
+        <v>8</v>
+      </c>
+      <c r="DG35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="DH35">
+        <v>8</v>
+      </c>
+      <c r="DI35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_DOT_ACCENT</t>
+        </is>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -37890,6 +38083,22 @@
       <c r="DE36" s="127" t="s">
         <v>80</v>
       </c>
+      <c r="DF36">
+        <v>9</v>
+      </c>
+      <c r="DG36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="DH36">
+        <v>9</v>
+      </c>
+      <c r="DI36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -38182,6 +38391,26 @@
       </c>
       <c r="DE37" s="127" t="s">
         <v>200</v>
+      </c>
+      <c r="DF37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DG37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="DH37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DI37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_HUNGARUMLAUT</t>
+        </is>
       </c>
     </row>
     <row r="38" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39023,6 +39252,26 @@
       <c r="DE43" s="127" t="s">
         <v>59</v>
       </c>
+      <c r="DF43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="DG43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="DH43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="DI43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIAERESIS</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -39302,6 +39551,26 @@
       <c r="DE44" s="115" t="s">
         <v>1295</v>
       </c>
+      <c r="DF44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="DG44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="DH44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="DI44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEDILLA</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -39573,6 +39842,16 @@
       <c r="DE45" s="127" t="s">
         <v>163</v>
       </c>
+      <c r="DF45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
+      <c r="DG45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0160</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -39849,6 +40128,16 @@
       </c>
       <c r="DE46" s="115" t="s">
         <v>1311</v>
+      </c>
+      <c r="DF46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0111</t>
+        </is>
+      </c>
+      <c r="DG46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0110</t>
+        </is>
       </c>
     </row>
     <row r="47" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40252,6 +40541,16 @@
       <c r="DC48" s="115"/>
       <c r="DD48" s="115"/>
       <c r="DE48" s="115"/>
+      <c r="DF48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017E</t>
+        </is>
+      </c>
+      <c r="DG48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017D</t>
+        </is>
+      </c>
     </row>
     <row r="49" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="93" t="s">
@@ -40506,6 +40805,16 @@
       </c>
       <c r="DE49" s="115" t="s">
         <v>1249</v>
+      </c>
+      <c r="DF49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010D</t>
+        </is>
+      </c>
+      <c r="DG49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010C</t>
+        </is>
       </c>
     </row>
     <row r="50" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40766,6 +41075,16 @@
       <c r="DE50" s="115" t="s">
         <v>135</v>
       </c>
+      <c r="DF50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0107</t>
+        </is>
+      </c>
+      <c r="DG50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0106</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -41033,6 +41352,21 @@
         <v>1197</v>
       </c>
       <c r="DE51" s="115"/>
+      <c r="DF51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEDILLA</t>
+        </is>
+      </c>
+      <c r="DG51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIAERESIS</t>
+        </is>
+      </c>
+      <c r="DH51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEDILLA</t>
+        </is>
+      </c>
     </row>
     <row r="52" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="93" t="s">
@@ -42037,6 +42371,26 @@
         <v>16</v>
       </c>
       <c r="DE55" s="171"/>
+      <c r="DF55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DG55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="DH55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DI55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|</t>
+        </is>
+      </c>
     </row>
     <row r="56" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="141" t="s">
@@ -42250,6 +42604,14 @@
       <c r="DE56" s="171" t="n">
         <v>48</v>
       </c>
+      <c r="DG56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DI56">
+        <v>52</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -42463,6 +42825,14 @@
       <c r="DE57" s="171" t="n">
         <v>12</v>
       </c>
+      <c r="DG57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DI57">
+        <v>12</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -42676,6 +43046,12 @@
       <c r="DE58" s="171" t="n">
         <v>50</v>
       </c>
+      <c r="DG58">
+        <v>30</v>
+      </c>
+      <c r="DI58">
+        <v>52</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -42889,6 +43265,12 @@
       <c r="DE59" s="171" t="n">
         <v>12</v>
       </c>
+      <c r="DG59">
+        <v>0</v>
+      </c>
+      <c r="DI59">
+        <v>12</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -43102,6 +43484,12 @@
       <c r="DE60" s="171" t="n">
         <v>48</v>
       </c>
+      <c r="DG60">
+        <v>30</v>
+      </c>
+      <c r="DI60">
+        <v>52</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -43313,6 +43701,12 @@
       </c>
       <c r="DD61" s="171"/>
       <c r="DE61" s="171" t="n">
+        <v>12</v>
+      </c>
+      <c r="DG61">
+        <v>0</v>
+      </c>
+      <c r="DI61">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: add Slovak, Lithuanian, Latvian, Estonian, Brazilian Portuguese layouts
Phase 1 of the language batch - the five remaining no-new-glyph Latin layouts,
added via the cache-preserving key_lut surgical editor (all existing languages
regenerate byte-identically; hr-HR only gains trailing commas as the new columns
follow it). Letters + main symbols + safe AltGr (EUR, dead-key row); uncertain
AltGr left empty per review-after policy. Country codes appended to
gen-lang-fonts.sh COUNTRIES (flag_fonts.h regen deferred to batch end).

  sk-SK Slovak (CSN QWERTZ)        lt-LT Lithuanian (letters on number row)
  lv-LV Latvian (US base + AltGr)  et-EE Estonian (Nordic + o-tilde)
  pt-BR Brazilian Portuguese (ABNT2: c-cedilla + dead keys)

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -30588,7 +30588,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:DI79"/>
+  <dimension ref="A1:EC79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -30848,6 +30848,31 @@
           <t xml:space="preserve">hr-HR</t>
         </is>
       </c>
+      <c r="DJ1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sk-SK</t>
+        </is>
+      </c>
+      <c r="DN1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lt-LT</t>
+        </is>
+      </c>
+      <c r="DR1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lv-LV</t>
+        </is>
+      </c>
+      <c r="DV1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">et-EE</t>
+        </is>
+      </c>
+      <c r="DZ1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pt-BR</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -31015,6 +31040,11 @@
       <c r="DC2" s="90"/>
       <c r="DD2" s="90"/>
       <c r="DE2" s="91"/>
+      <c r="DU2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0101</t>
+        </is>
+      </c>
     </row>
     <row r="3" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="93" t="s">
@@ -31352,6 +31382,11 @@
       <c r="DE4" s="127" t="s">
         <v>1141</v>
       </c>
+      <c r="DU4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010D</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -31723,6 +31758,31 @@
           <t xml:space="preserve">EURO_SIGN</t>
         </is>
       </c>
+      <c r="DM6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
+      <c r="DQ6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
+      <c r="DU6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0113</t>
+        </is>
+      </c>
+      <c r="DY6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
+      <c r="EC6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
     </row>
     <row r="7" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="93" t="s">
@@ -32057,6 +32117,11 @@
           <t xml:space="preserve">]</t>
         </is>
       </c>
+      <c r="DU8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0123</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -32389,6 +32454,11 @@
       <c r="DE10" s="115" t="s">
         <v>116</v>
       </c>
+      <c r="DU10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_012B</t>
+        </is>
+      </c>
     </row>
     <row r="11" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="93" t="s">
@@ -32717,6 +32787,11 @@
       <c r="DE12" s="115" t="s">
         <v>1170</v>
       </c>
+      <c r="DU12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0137</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -32882,6 +32957,11 @@
       <c r="DE13" s="115" t="s">
         <v>1174</v>
       </c>
+      <c r="DU13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_013C</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -33233,6 +33313,11 @@
           <t xml:space="preserve">}</t>
         </is>
       </c>
+      <c r="DU15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0146</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -34093,6 +34178,16 @@
       <c r="DE20" s="127" t="s">
         <v>1207</v>
       </c>
+      <c r="DU20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
+      <c r="DY20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
     </row>
     <row r="21" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="93" t="s">
@@ -34421,6 +34516,11 @@
       <c r="DE22" s="115" t="s">
         <v>682</v>
       </c>
+      <c r="DU22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_016B</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -35127,6 +35227,16 @@
           <t xml:space="preserve">Z</t>
         </is>
       </c>
+      <c r="DJ26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z</t>
+        </is>
+      </c>
+      <c r="DK26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Z</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -35320,6 +35430,26 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
+      <c r="DJ27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y</t>
+        </is>
+      </c>
+      <c r="DK27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="DU27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017E</t>
+        </is>
+      </c>
+      <c r="DY27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017E</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -35614,6 +35744,46 @@
         <is>
           <t xml:space="preserve">MOD_TILDE</t>
         </is>
+      </c>
+      <c r="DJ28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="DK28">
+        <v>1</v>
+      </c>
+      <c r="DL28">
+        <v>1</v>
+      </c>
+      <c r="DM28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_TILDE</t>
+        </is>
+      </c>
+      <c r="DN28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0105</t>
+        </is>
+      </c>
+      <c r="DO28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0104</t>
+        </is>
+      </c>
+      <c r="DQ28">
+        <v>1</v>
+      </c>
+      <c r="DV28">
+        <v>1</v>
+      </c>
+      <c r="DW28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="DX28">
+        <v>1</v>
       </c>
     </row>
     <row r="29" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35926,6 +36096,51 @@
           <t xml:space="preserve">MOD_CARON</t>
         </is>
       </c>
+      <c r="DJ29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_013E</t>
+        </is>
+      </c>
+      <c r="DK29">
+        <v>2</v>
+      </c>
+      <c r="DL29">
+        <v>2</v>
+      </c>
+      <c r="DM29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_CARON</t>
+        </is>
+      </c>
+      <c r="DN29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010D</t>
+        </is>
+      </c>
+      <c r="DO29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010C</t>
+        </is>
+      </c>
+      <c r="DQ29">
+        <v>2</v>
+      </c>
+      <c r="DV29">
+        <v>2</v>
+      </c>
+      <c r="DW29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"</t>
+        </is>
+      </c>
+      <c r="DX29">
+        <v>2</v>
+      </c>
+      <c r="DY29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@</t>
+        </is>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -36239,6 +36454,51 @@
           <t xml:space="preserve">^</t>
         </is>
       </c>
+      <c r="DJ30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
+      <c r="DK30">
+        <v>3</v>
+      </c>
+      <c r="DL30">
+        <v>3</v>
+      </c>
+      <c r="DM30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="DN30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0119</t>
+        </is>
+      </c>
+      <c r="DO30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0118</t>
+        </is>
+      </c>
+      <c r="DQ30">
+        <v>3</v>
+      </c>
+      <c r="DV30">
+        <v>3</v>
+      </c>
+      <c r="DW30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="DX30">
+        <v>3</v>
+      </c>
+      <c r="DY30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POUND_SIGN</t>
+        </is>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -36552,6 +36812,51 @@
           <t xml:space="preserve">MOD_BREVE</t>
         </is>
       </c>
+      <c r="DJ31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_010D</t>
+        </is>
+      </c>
+      <c r="DK31">
+        <v>4</v>
+      </c>
+      <c r="DL31">
+        <v>4</v>
+      </c>
+      <c r="DM31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_BREVE</t>
+        </is>
+      </c>
+      <c r="DN31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0117</t>
+        </is>
+      </c>
+      <c r="DO31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0116</t>
+        </is>
+      </c>
+      <c r="DQ31">
+        <v>4</v>
+      </c>
+      <c r="DV31">
+        <v>4</v>
+      </c>
+      <c r="DW31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CURRENCY_SIGN</t>
+        </is>
+      </c>
+      <c r="DX31">
+        <v>4</v>
+      </c>
+      <c r="DY31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -36865,6 +37170,46 @@
           <t xml:space="preserve">MOD_RING</t>
         </is>
       </c>
+      <c r="DJ32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0165</t>
+        </is>
+      </c>
+      <c r="DK32">
+        <v>5</v>
+      </c>
+      <c r="DL32">
+        <v>5</v>
+      </c>
+      <c r="DM32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_RING</t>
+        </is>
+      </c>
+      <c r="DN32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_012F</t>
+        </is>
+      </c>
+      <c r="DO32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_012E</t>
+        </is>
+      </c>
+      <c r="DQ32">
+        <v>5</v>
+      </c>
+      <c r="DV32">
+        <v>5</v>
+      </c>
+      <c r="DW32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="DX32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -37166,6 +37511,46 @@
           <t xml:space="preserve">MOD_OGONEK</t>
         </is>
       </c>
+      <c r="DJ33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017E</t>
+        </is>
+      </c>
+      <c r="DK33">
+        <v>6</v>
+      </c>
+      <c r="DL33">
+        <v>6</v>
+      </c>
+      <c r="DM33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_OGONEK</t>
+        </is>
+      </c>
+      <c r="DN33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
+      <c r="DO33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0160</t>
+        </is>
+      </c>
+      <c r="DQ33">
+        <v>6</v>
+      </c>
+      <c r="DV33">
+        <v>6</v>
+      </c>
+      <c r="DW33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="DX33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -37477,6 +37862,51 @@
           <t xml:space="preserve">`</t>
         </is>
       </c>
+      <c r="DJ34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00FD</t>
+        </is>
+      </c>
+      <c r="DK34">
+        <v>7</v>
+      </c>
+      <c r="DL34">
+        <v>7</v>
+      </c>
+      <c r="DM34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
+        </is>
+      </c>
+      <c r="DN34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0173</t>
+        </is>
+      </c>
+      <c r="DO34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0172</t>
+        </is>
+      </c>
+      <c r="DQ34">
+        <v>7</v>
+      </c>
+      <c r="DV34">
+        <v>7</v>
+      </c>
+      <c r="DW34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="DX34">
+        <v>7</v>
+      </c>
+      <c r="DY34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{</t>
+        </is>
+      </c>
     </row>
     <row r="35" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="93" t="s">
@@ -37788,6 +38218,51 @@
           <t xml:space="preserve">MOD_DOT_ACCENT</t>
         </is>
       </c>
+      <c r="DJ35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E1</t>
+        </is>
+      </c>
+      <c r="DK35">
+        <v>8</v>
+      </c>
+      <c r="DL35">
+        <v>8</v>
+      </c>
+      <c r="DM35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_DOT_ACCENT</t>
+        </is>
+      </c>
+      <c r="DN35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_016B</t>
+        </is>
+      </c>
+      <c r="DO35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_016A</t>
+        </is>
+      </c>
+      <c r="DQ35">
+        <v>8</v>
+      </c>
+      <c r="DV35">
+        <v>8</v>
+      </c>
+      <c r="DW35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="DX35">
+        <v>8</v>
+      </c>
+      <c r="DY35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -38099,6 +38574,49 @@
           <t xml:space="preserve">ACUTE_ACCENT</t>
         </is>
       </c>
+      <c r="DJ36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00ED</t>
+        </is>
+      </c>
+      <c r="DK36">
+        <v>9</v>
+      </c>
+      <c r="DL36">
+        <v>9</v>
+      </c>
+      <c r="DM36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
+      <c r="DN36">
+        <v>9</v>
+      </c>
+      <c r="DO36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="DP36">
+        <v>9</v>
+      </c>
+      <c r="DV36">
+        <v>9</v>
+      </c>
+      <c r="DW36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="DX36">
+        <v>9</v>
+      </c>
+      <c r="DY36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -38410,6 +38928,61 @@
       <c r="DI37" t="inlineStr">
         <is>
           <t xml:space="preserve">MOD_HUNGARUMLAUT</t>
+        </is>
+      </c>
+      <c r="DJ37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E9</t>
+        </is>
+      </c>
+      <c r="DK37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DL37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DM37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_HUNGARUMLAUT</t>
+        </is>
+      </c>
+      <c r="DN37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DO37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="DP37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DV37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DW37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="DX37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="DY37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">}</t>
         </is>
       </c>
     </row>
@@ -39272,6 +39845,56 @@
           <t xml:space="preserve">DIAERESIS</t>
         </is>
       </c>
+      <c r="DJ43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="DK43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="DL43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="DN43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="DO43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_</t>
+        </is>
+      </c>
+      <c r="DP43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="DV43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="DW43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="DX43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="DY43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BACKSLASH</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -39571,6 +40194,46 @@
           <t xml:space="preserve">CEDILLA</t>
         </is>
       </c>
+      <c r="DJ44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
+      <c r="DK44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOD_CARON</t>
+        </is>
+      </c>
+      <c r="DL44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
+      <c r="DN44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017E</t>
+        </is>
+      </c>
+      <c r="DO44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_017D</t>
+        </is>
+      </c>
+      <c r="DV44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
+      <c r="DW44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
+        </is>
+      </c>
+      <c r="DX44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -39852,6 +40515,46 @@
           <t xml:space="preserve">LATIN_0160</t>
         </is>
       </c>
+      <c r="DJ45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00FA</t>
+        </is>
+      </c>
+      <c r="DK45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="DL45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00FA</t>
+        </is>
+      </c>
+      <c r="DV45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00FC</t>
+        </is>
+      </c>
+      <c r="DW45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00DC</t>
+        </is>
+      </c>
+      <c r="DZ45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
+      <c r="EA45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
+        </is>
+      </c>
+      <c r="EB45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACUTE_ACCENT</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -40139,6 +40842,46 @@
           <t xml:space="preserve">LATIN_0110</t>
         </is>
       </c>
+      <c r="DJ46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E4</t>
+        </is>
+      </c>
+      <c r="DK46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="DL46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E4</t>
+        </is>
+      </c>
+      <c r="DV46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00F5</t>
+        </is>
+      </c>
+      <c r="DW46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00D5</t>
+        </is>
+      </c>
+      <c r="DZ46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
+      <c r="EA46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{</t>
+        </is>
+      </c>
+      <c r="EB46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
     </row>
     <row r="47" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="93" t="s">
@@ -40405,6 +41148,21 @@
       </c>
       <c r="DE47" s="127" t="s">
         <v>51</v>
+      </c>
+      <c r="DZ47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
+      <c r="EA47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">}</t>
+        </is>
+      </c>
+      <c r="EB47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
       </c>
     </row>
     <row r="48" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40551,6 +41309,36 @@
           <t xml:space="preserve">LATIN_017D</t>
         </is>
       </c>
+      <c r="DJ48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0148</t>
+        </is>
+      </c>
+      <c r="DK48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="DL48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_0148</t>
+        </is>
+      </c>
+      <c r="DV48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="DW48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="DX48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
     </row>
     <row r="49" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="93" t="s">
@@ -40814,6 +41602,41 @@
       <c r="DG49" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_010C</t>
+        </is>
+      </c>
+      <c r="DJ49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00F4</t>
+        </is>
+      </c>
+      <c r="DK49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"</t>
+        </is>
+      </c>
+      <c r="DL49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00F4</t>
+        </is>
+      </c>
+      <c r="DV49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00F6</t>
+        </is>
+      </c>
+      <c r="DW49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00D6</t>
+        </is>
+      </c>
+      <c r="DZ49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E7</t>
+        </is>
+      </c>
+      <c r="EA49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00C7</t>
         </is>
       </c>
     </row>
@@ -41085,6 +41908,46 @@
           <t xml:space="preserve">LATIN_0106</t>
         </is>
       </c>
+      <c r="DJ50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTION</t>
+        </is>
+      </c>
+      <c r="DK50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="DL50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SECTION</t>
+        </is>
+      </c>
+      <c r="DV50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00E4</t>
+        </is>
+      </c>
+      <c r="DW50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LATIN_00C4</t>
+        </is>
+      </c>
+      <c r="DZ50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~</t>
+        </is>
+      </c>
+      <c r="EA50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="EB50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -41365,6 +42228,21 @@
       <c r="DH51" t="inlineStr">
         <is>
           <t xml:space="preserve">CEDILLA</t>
+        </is>
+      </c>
+      <c r="DJ51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">;</t>
+        </is>
+      </c>
+      <c r="DK51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEGREE</t>
+        </is>
+      </c>
+      <c r="DL51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">;</t>
         </is>
       </c>
     </row>
@@ -42391,6 +43269,41 @@
           <t xml:space="preserve">|</t>
         </is>
       </c>
+      <c r="DJ55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DK55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="DL55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DV55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DW55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="DX55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="DY55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|</t>
+        </is>
+      </c>
     </row>
     <row r="56" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="141" t="s">
@@ -42612,6 +43525,46 @@
       <c r="DI56">
         <v>52</v>
       </c>
+      <c r="DK56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DM56">
+        <v>52</v>
+      </c>
+      <c r="DO56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DQ56">
+        <v>52</v>
+      </c>
+      <c r="DS56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DU56">
+        <v>52</v>
+      </c>
+      <c r="DW56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DY56">
+        <v>52</v>
+      </c>
+      <c r="EA56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EC56">
+        <v>52</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -42833,6 +43786,46 @@
       <c r="DI57">
         <v>12</v>
       </c>
+      <c r="DK57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DM57">
+        <v>12</v>
+      </c>
+      <c r="DO57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DQ57">
+        <v>12</v>
+      </c>
+      <c r="DS57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DU57">
+        <v>12</v>
+      </c>
+      <c r="DW57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="DY57">
+        <v>12</v>
+      </c>
+      <c r="EA57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EC57">
+        <v>12</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -43052,6 +44045,36 @@
       <c r="DI58">
         <v>52</v>
       </c>
+      <c r="DK58">
+        <v>30</v>
+      </c>
+      <c r="DM58">
+        <v>52</v>
+      </c>
+      <c r="DO58">
+        <v>30</v>
+      </c>
+      <c r="DQ58">
+        <v>52</v>
+      </c>
+      <c r="DS58">
+        <v>30</v>
+      </c>
+      <c r="DU58">
+        <v>52</v>
+      </c>
+      <c r="DW58">
+        <v>30</v>
+      </c>
+      <c r="DY58">
+        <v>52</v>
+      </c>
+      <c r="EA58">
+        <v>30</v>
+      </c>
+      <c r="EC58">
+        <v>52</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -43271,6 +44294,36 @@
       <c r="DI59">
         <v>12</v>
       </c>
+      <c r="DK59">
+        <v>0</v>
+      </c>
+      <c r="DM59">
+        <v>12</v>
+      </c>
+      <c r="DO59">
+        <v>0</v>
+      </c>
+      <c r="DQ59">
+        <v>12</v>
+      </c>
+      <c r="DS59">
+        <v>0</v>
+      </c>
+      <c r="DU59">
+        <v>12</v>
+      </c>
+      <c r="DW59">
+        <v>0</v>
+      </c>
+      <c r="DY59">
+        <v>12</v>
+      </c>
+      <c r="EA59">
+        <v>0</v>
+      </c>
+      <c r="EC59">
+        <v>12</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -43490,6 +44543,36 @@
       <c r="DI60">
         <v>52</v>
       </c>
+      <c r="DK60">
+        <v>30</v>
+      </c>
+      <c r="DM60">
+        <v>52</v>
+      </c>
+      <c r="DO60">
+        <v>30</v>
+      </c>
+      <c r="DQ60">
+        <v>52</v>
+      </c>
+      <c r="DS60">
+        <v>30</v>
+      </c>
+      <c r="DU60">
+        <v>52</v>
+      </c>
+      <c r="DW60">
+        <v>30</v>
+      </c>
+      <c r="DY60">
+        <v>52</v>
+      </c>
+      <c r="EA60">
+        <v>30</v>
+      </c>
+      <c r="EC60">
+        <v>52</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -43707,6 +44790,36 @@
         <v>0</v>
       </c>
       <c r="DI61">
+        <v>12</v>
+      </c>
+      <c r="DK61">
+        <v>0</v>
+      </c>
+      <c r="DM61">
+        <v>12</v>
+      </c>
+      <c r="DO61">
+        <v>0</v>
+      </c>
+      <c r="DQ61">
+        <v>12</v>
+      </c>
+      <c r="DS61">
+        <v>0</v>
+      </c>
+      <c r="DU61">
+        <v>12</v>
+      </c>
+      <c r="DW61">
+        <v>0</v>
+      </c>
+      <c r="DY61">
+        <v>12</v>
+      </c>
+      <c r="EA61">
+        <v>0</v>
+      </c>
+      <c r="EC61">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: add Serbian-Cyrillic and Macedonian layouts + Cyrillic glyphs
Phase 2 (Cyrillic). Added 18 South-Slavic Cyrillic glyphs (ђћljnjdž ѓќѕ ј, both
cases) to the named_glyphs sheet (rows 956-973, surgical/cache-safe) and
regenerated named_glyphs.h; their codepoints (U+0402-045F) already fall inside
the compiled _Cyrillic_ font strike (0x401-0x46b), so no font regen is needed.

  sr-RS Serbian (Cyrillic) - JUS layout
  mk-MK Macedonian          - with Ѓ Ќ Ѕ

Both Cyrillic layouts NEED a hardware-review pass on exact key positions (built
from the published standard). Mongolian deferred: its 35-letter MNS layout has
number-row placements I want to verify before committing. All 33 existing
languages regenerate byte-identically (pt-BR only gains trailing commas).

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -29387,128 +29387,272 @@
       <c r="I955" s="15"/>
     </row>
     <row r="956" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A956" s="12"/>
-      <c r="B956" s="15"/>
+      <c r="A956" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DJE</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t xml:space="preserve">402</t>
+        </is>
+      </c>
       <c r="D956" s="9"/>
       <c r="E956" s="10"/>
       <c r="F956" s="1"/>
       <c r="H956" s="7"/>
     </row>
     <row r="957" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A957" s="7"/>
-      <c r="B957" s="7"/>
+      <c r="A957" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DJE</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t xml:space="preserve">452</t>
+        </is>
+      </c>
       <c r="C957" s="7"/>
       <c r="D957" s="7"/>
       <c r="E957" s="7"/>
     </row>
     <row r="958" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A958" s="7"/>
-      <c r="B958" s="7"/>
+      <c r="A958" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TSHE</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40B</t>
+        </is>
+      </c>
       <c r="C958" s="7"/>
       <c r="D958" s="7"/>
       <c r="E958" s="7"/>
     </row>
     <row r="959" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A959" s="7"/>
-      <c r="B959" s="7"/>
+      <c r="A959" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TSHE</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45B</t>
+        </is>
+      </c>
       <c r="C959" s="7"/>
       <c r="D959" s="7"/>
       <c r="E959" s="7"/>
     </row>
     <row r="960" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A960" s="7"/>
-      <c r="B960" s="7"/>
+      <c r="A960" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_LJE</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t xml:space="preserve">409</t>
+        </is>
+      </c>
       <c r="C960" s="7"/>
       <c r="D960" s="7"/>
       <c r="E960" s="7"/>
     </row>
     <row r="961" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A961" s="7"/>
-      <c r="B961" s="7"/>
+      <c r="A961" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_LJE</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t xml:space="preserve">459</t>
+        </is>
+      </c>
       <c r="C961" s="7"/>
       <c r="D961" s="7"/>
       <c r="E961" s="7"/>
     </row>
     <row r="962" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A962" s="7"/>
-      <c r="B962" s="7"/>
+      <c r="A962" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_NJE</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40A</t>
+        </is>
+      </c>
       <c r="C962" s="7"/>
       <c r="D962" s="7"/>
       <c r="E962" s="7"/>
     </row>
     <row r="963" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A963" s="7"/>
-      <c r="B963" s="7"/>
+      <c r="A963" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_NJE</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45A</t>
+        </is>
+      </c>
       <c r="C963" s="7"/>
       <c r="D963" s="7"/>
       <c r="E963" s="7"/>
     </row>
     <row r="964" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A964" s="7"/>
-      <c r="B964" s="7"/>
+      <c r="A964" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZHE</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40F</t>
+        </is>
+      </c>
       <c r="C964" s="7"/>
       <c r="D964" s="7"/>
       <c r="E964" s="7"/>
     </row>
     <row r="965" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A965" s="7"/>
-      <c r="B965" s="7"/>
+      <c r="A965" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZHE</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45F</t>
+        </is>
+      </c>
       <c r="C965" s="7"/>
       <c r="D965" s="7"/>
       <c r="E965" s="7"/>
     </row>
     <row r="966" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A966" s="7"/>
-      <c r="B966" s="7"/>
+      <c r="A966" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_JE</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t xml:space="preserve">408</t>
+        </is>
+      </c>
       <c r="C966" s="7"/>
       <c r="D966" s="7"/>
       <c r="E966" s="7"/>
     </row>
     <row r="967" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A967" s="7"/>
-      <c r="B967" s="7"/>
+      <c r="A967" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_JE</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t xml:space="preserve">458</t>
+        </is>
+      </c>
       <c r="C967" s="7"/>
       <c r="D967" s="7"/>
       <c r="E967" s="7"/>
     </row>
     <row r="968" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A968" s="7"/>
-      <c r="B968" s="7"/>
+      <c r="A968" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_GJE</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403</t>
+        </is>
+      </c>
       <c r="C968" s="7"/>
       <c r="D968" s="7"/>
       <c r="E968" s="7"/>
     </row>
     <row r="969" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A969" s="7"/>
-      <c r="B969" s="7"/>
+      <c r="A969" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_GJE</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t xml:space="preserve">453</t>
+        </is>
+      </c>
       <c r="C969" s="7"/>
       <c r="D969" s="7"/>
       <c r="E969" s="7"/>
     </row>
     <row r="970" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A970" s="7"/>
-      <c r="B970" s="7"/>
+      <c r="A970" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_KJE</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40C</t>
+        </is>
+      </c>
       <c r="C970" s="7"/>
       <c r="D970" s="7"/>
       <c r="E970" s="7"/>
     </row>
     <row r="971" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A971" s="7"/>
-      <c r="B971" s="7"/>
+      <c r="A971" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_KJE</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45C</t>
+        </is>
+      </c>
       <c r="C971" s="7"/>
       <c r="D971" s="7"/>
       <c r="E971" s="7"/>
     </row>
     <row r="972" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A972" s="7"/>
-      <c r="B972" s="7"/>
+      <c r="A972" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZE</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t xml:space="preserve">405</t>
+        </is>
+      </c>
       <c r="C972" s="7"/>
       <c r="D972" s="7"/>
       <c r="E972" s="7"/>
     </row>
     <row r="973" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A973" s="7"/>
-      <c r="B973" s="7"/>
+      <c r="A973" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZE</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t xml:space="preserve">455</t>
+        </is>
+      </c>
       <c r="C973" s="7"/>
       <c r="D973" s="7"/>
       <c r="E973" s="7"/>
@@ -30588,7 +30732,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:EC79"/>
+  <dimension ref="A1:EK79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -30873,6 +31017,16 @@
           <t xml:space="preserve">pt-BR</t>
         </is>
       </c>
+      <c r="ED1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sr-RS</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mk-MK</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -31043,6 +31197,26 @@
       <c r="DU2" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_0101</t>
+        </is>
+      </c>
+      <c r="ED2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_A</t>
+        </is>
+      </c>
+      <c r="EE2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_A</t>
+        </is>
+      </c>
+      <c r="EH2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_A</t>
+        </is>
+      </c>
+      <c r="EI2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_A</t>
         </is>
       </c>
     </row>
@@ -31213,6 +31387,26 @@
           <t xml:space="preserve">{</t>
         </is>
       </c>
+      <c r="ED3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_BE</t>
+        </is>
+      </c>
+      <c r="EE3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_BE</t>
+        </is>
+      </c>
+      <c r="EH3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_BE</t>
+        </is>
+      </c>
+      <c r="EI3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_BE</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -31387,6 +31581,26 @@
           <t xml:space="preserve">LATIN_010D</t>
         </is>
       </c>
+      <c r="ED4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TSE</t>
+        </is>
+      </c>
+      <c r="EE4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TSE</t>
+        </is>
+      </c>
+      <c r="EH4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TSE</t>
+        </is>
+      </c>
+      <c r="EI4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TSE</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -31556,6 +31770,26 @@
       <c r="DE5" s="115" t="s">
         <v>1146</v>
       </c>
+      <c r="ED5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DE</t>
+        </is>
+      </c>
+      <c r="EE5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DE</t>
+        </is>
+      </c>
+      <c r="EH5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DE</t>
+        </is>
+      </c>
+      <c r="EI5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DE</t>
+        </is>
+      </c>
     </row>
     <row r="6" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="93" t="s">
@@ -31781,6 +32015,26 @@
       <c r="EC6" t="inlineStr">
         <is>
           <t xml:space="preserve">EURO_SIGN</t>
+        </is>
+      </c>
+      <c r="ED6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_IE</t>
+        </is>
+      </c>
+      <c r="EE6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_IE</t>
+        </is>
+      </c>
+      <c r="EH6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_IE</t>
+        </is>
+      </c>
+      <c r="EI6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_IE</t>
         </is>
       </c>
     </row>
@@ -31951,6 +32205,26 @@
           <t xml:space="preserve">[</t>
         </is>
       </c>
+      <c r="ED7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EF</t>
+        </is>
+      </c>
+      <c r="EE7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EF</t>
+        </is>
+      </c>
+      <c r="EH7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EF</t>
+        </is>
+      </c>
+      <c r="EI7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EF</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -32122,6 +32396,26 @@
           <t xml:space="preserve">LATIN_0123</t>
         </is>
       </c>
+      <c r="ED8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_GHE</t>
+        </is>
+      </c>
+      <c r="EE8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_GHE</t>
+        </is>
+      </c>
+      <c r="EH8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_GHE</t>
+        </is>
+      </c>
+      <c r="EI8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_GHE</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -32283,6 +32577,26 @@
       <c r="DC9" s="115"/>
       <c r="DD9" s="115"/>
       <c r="DE9" s="115"/>
+      <c r="ED9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_HA</t>
+        </is>
+      </c>
+      <c r="EE9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_HA</t>
+        </is>
+      </c>
+      <c r="EH9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_HA</t>
+        </is>
+      </c>
+      <c r="EI9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_HA</t>
+        </is>
+      </c>
     </row>
     <row r="10" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="93" t="s">
@@ -32457,6 +32771,26 @@
       <c r="DU10" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_012B</t>
+        </is>
+      </c>
+      <c r="ED10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_I</t>
+        </is>
+      </c>
+      <c r="EE10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_I</t>
+        </is>
+      </c>
+      <c r="EH10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_I</t>
+        </is>
+      </c>
+      <c r="EI10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_I</t>
         </is>
       </c>
     </row>
@@ -32624,6 +32958,26 @@
       <c r="DE11" s="127" t="s">
         <v>151</v>
       </c>
+      <c r="ED11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_JE</t>
+        </is>
+      </c>
+      <c r="EE11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_JE</t>
+        </is>
+      </c>
+      <c r="EH11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_JE</t>
+        </is>
+      </c>
+      <c r="EI11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_JE</t>
+        </is>
+      </c>
     </row>
     <row r="12" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
@@ -32792,6 +33146,26 @@
           <t xml:space="preserve">LATIN_0137</t>
         </is>
       </c>
+      <c r="ED12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_KA</t>
+        </is>
+      </c>
+      <c r="EE12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_KA</t>
+        </is>
+      </c>
+      <c r="EH12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_KA</t>
+        </is>
+      </c>
+      <c r="EI12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_KA</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -32962,6 +33336,26 @@
           <t xml:space="preserve">LATIN_013C</t>
         </is>
       </c>
+      <c r="ED13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EL</t>
+        </is>
+      </c>
+      <c r="EE13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EL</t>
+        </is>
+      </c>
+      <c r="EH13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EL</t>
+        </is>
+      </c>
+      <c r="EI13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EL</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -33142,6 +33536,26 @@
       <c r="DD14" s="115"/>
       <c r="DE14" s="115" t="s">
         <v>1181</v>
+      </c>
+      <c r="ED14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EM</t>
+        </is>
+      </c>
+      <c r="EE14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EM</t>
+        </is>
+      </c>
+      <c r="EH14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EM</t>
+        </is>
+      </c>
+      <c r="EI14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EM</t>
+        </is>
       </c>
     </row>
     <row r="15" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33318,6 +33732,26 @@
           <t xml:space="preserve">LATIN_0146</t>
         </is>
       </c>
+      <c r="ED15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EN</t>
+        </is>
+      </c>
+      <c r="EE15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EN</t>
+        </is>
+      </c>
+      <c r="EH15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EN</t>
+        </is>
+      </c>
+      <c r="EI15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EN</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -33483,6 +33917,26 @@
       <c r="DC16" s="115"/>
       <c r="DD16" s="115"/>
       <c r="DE16" s="115"/>
+      <c r="ED16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_O</t>
+        </is>
+      </c>
+      <c r="EE16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_O</t>
+        </is>
+      </c>
+      <c r="EH16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_O</t>
+        </is>
+      </c>
+      <c r="EI16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_O</t>
+        </is>
+      </c>
     </row>
     <row r="17" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
@@ -33648,6 +34102,26 @@
       <c r="DC17" s="115"/>
       <c r="DD17" s="115"/>
       <c r="DE17" s="127"/>
+      <c r="ED17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_PE</t>
+        </is>
+      </c>
+      <c r="EE17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_PE</t>
+        </is>
+      </c>
+      <c r="EH17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_PE</t>
+        </is>
+      </c>
+      <c r="EI17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_PE</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="93" t="s">
@@ -33840,6 +34314,26 @@
       <c r="DI18" t="inlineStr">
         <is>
           <t xml:space="preserve">BACKSLASH</t>
+        </is>
+      </c>
+      <c r="ED18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_LJE</t>
+        </is>
+      </c>
+      <c r="EE18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_LJE</t>
+        </is>
+      </c>
+      <c r="EH18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_LJE</t>
+        </is>
+      </c>
+      <c r="EI18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_LJE</t>
         </is>
       </c>
     </row>
@@ -34011,6 +34505,26 @@
       <c r="DC19" s="115"/>
       <c r="DD19" s="115"/>
       <c r="DE19" s="115"/>
+      <c r="ED19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ER</t>
+        </is>
+      </c>
+      <c r="EE19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ER</t>
+        </is>
+      </c>
+      <c r="EH19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ER</t>
+        </is>
+      </c>
+      <c r="EI19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ER</t>
+        </is>
+      </c>
     </row>
     <row r="20" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="93" t="s">
@@ -34186,6 +34700,26 @@
       <c r="DY20" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_0161</t>
+        </is>
+      </c>
+      <c r="ED20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ES</t>
+        </is>
+      </c>
+      <c r="EE20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ES</t>
+        </is>
+      </c>
+      <c r="EH20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ES</t>
+        </is>
+      </c>
+      <c r="EI20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ES</t>
         </is>
       </c>
     </row>
@@ -34347,6 +34881,26 @@
       <c r="DC21" s="115"/>
       <c r="DD21" s="115"/>
       <c r="DE21" s="115"/>
+      <c r="ED21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TE</t>
+        </is>
+      </c>
+      <c r="EE21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TE</t>
+        </is>
+      </c>
+      <c r="EH21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TE</t>
+        </is>
+      </c>
+      <c r="EI21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TE</t>
+        </is>
+      </c>
     </row>
     <row r="22" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="93" t="s">
@@ -34521,6 +35075,26 @@
           <t xml:space="preserve">LATIN_016B</t>
         </is>
       </c>
+      <c r="ED22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_U</t>
+        </is>
+      </c>
+      <c r="EE22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_U</t>
+        </is>
+      </c>
+      <c r="EH22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_U</t>
+        </is>
+      </c>
+      <c r="EI22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_U</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -34691,6 +35265,26 @@
           <t xml:space="preserve">@</t>
         </is>
       </c>
+      <c r="ED23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_VE</t>
+        </is>
+      </c>
+      <c r="EE23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_VE</t>
+        </is>
+      </c>
+      <c r="EH23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_VE</t>
+        </is>
+      </c>
+      <c r="EI23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_VE</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -34871,6 +35465,26 @@
       <c r="DI24" t="inlineStr">
         <is>
           <t xml:space="preserve">|</t>
+        </is>
+      </c>
+      <c r="ED24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_NJE</t>
+        </is>
+      </c>
+      <c r="EE24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_NJE</t>
+        </is>
+      </c>
+      <c r="EH24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_NJE</t>
+        </is>
+      </c>
+      <c r="EI24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_NJE</t>
         </is>
       </c>
     </row>
@@ -35038,6 +35652,26 @@
       <c r="DE25" s="115" t="s">
         <v>1228</v>
       </c>
+      <c r="ED25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZHE</t>
+        </is>
+      </c>
+      <c r="EE25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZHE</t>
+        </is>
+      </c>
+      <c r="EH25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZHE</t>
+        </is>
+      </c>
+      <c r="EI25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZHE</t>
+        </is>
+      </c>
     </row>
     <row r="26" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="93" t="s">
@@ -35237,6 +35871,26 @@
           <t xml:space="preserve">Z</t>
         </is>
       </c>
+      <c r="ED26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZE</t>
+        </is>
+      </c>
+      <c r="EE26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZE</t>
+        </is>
+      </c>
+      <c r="EH26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZE</t>
+        </is>
+      </c>
+      <c r="EI26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZE</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -35450,6 +36104,26 @@
           <t xml:space="preserve">LATIN_017E</t>
         </is>
       </c>
+      <c r="ED27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DZE</t>
+        </is>
+      </c>
+      <c r="EE27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DZE</t>
+        </is>
+      </c>
+      <c r="EH27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZE</t>
+        </is>
+      </c>
+      <c r="EI27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZE</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -35783,6 +36457,28 @@
         </is>
       </c>
       <c r="DX28">
+        <v>1</v>
+      </c>
+      <c r="ED28">
+        <v>1</v>
+      </c>
+      <c r="EE28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="EF28">
+        <v>1</v>
+      </c>
+      <c r="EH28">
+        <v>1</v>
+      </c>
+      <c r="EI28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="EJ28">
         <v>1</v>
       </c>
     </row>
@@ -36141,6 +36837,28 @@
           <t xml:space="preserve">@</t>
         </is>
       </c>
+      <c r="ED29">
+        <v>2</v>
+      </c>
+      <c r="EE29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"</t>
+        </is>
+      </c>
+      <c r="EF29">
+        <v>2</v>
+      </c>
+      <c r="EH29">
+        <v>2</v>
+      </c>
+      <c r="EI29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"</t>
+        </is>
+      </c>
+      <c r="EJ29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -36499,6 +37217,28 @@
           <t xml:space="preserve">POUND_SIGN</t>
         </is>
       </c>
+      <c r="ED30">
+        <v>3</v>
+      </c>
+      <c r="EE30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="EF30">
+        <v>3</v>
+      </c>
+      <c r="EH30">
+        <v>3</v>
+      </c>
+      <c r="EI30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="EJ30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -36857,6 +37597,28 @@
           <t xml:space="preserve">$</t>
         </is>
       </c>
+      <c r="ED31">
+        <v>4</v>
+      </c>
+      <c r="EE31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="EF31">
+        <v>4</v>
+      </c>
+      <c r="EH31">
+        <v>4</v>
+      </c>
+      <c r="EI31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="EJ31">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -37210,6 +37972,28 @@
       <c r="DX32">
         <v>5</v>
       </c>
+      <c r="ED32">
+        <v>5</v>
+      </c>
+      <c r="EE32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="EF32">
+        <v>5</v>
+      </c>
+      <c r="EH32">
+        <v>5</v>
+      </c>
+      <c r="EI32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="EJ32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -37551,6 +38335,28 @@
       <c r="DX33">
         <v>6</v>
       </c>
+      <c r="ED33">
+        <v>6</v>
+      </c>
+      <c r="EE33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="EF33">
+        <v>6</v>
+      </c>
+      <c r="EH33">
+        <v>6</v>
+      </c>
+      <c r="EI33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="EJ33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -37907,6 +38713,28 @@
           <t xml:space="preserve">{</t>
         </is>
       </c>
+      <c r="ED34">
+        <v>7</v>
+      </c>
+      <c r="EE34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="EF34">
+        <v>7</v>
+      </c>
+      <c r="EH34">
+        <v>7</v>
+      </c>
+      <c r="EI34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="EJ34">
+        <v>7</v>
+      </c>
     </row>
     <row r="35" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="93" t="s">
@@ -38263,6 +39091,28 @@
           <t xml:space="preserve">[</t>
         </is>
       </c>
+      <c r="ED35">
+        <v>8</v>
+      </c>
+      <c r="EE35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="EF35">
+        <v>8</v>
+      </c>
+      <c r="EH35">
+        <v>8</v>
+      </c>
+      <c r="EI35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="EJ35">
+        <v>8</v>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -38617,6 +39467,28 @@
           <t xml:space="preserve">]</t>
         </is>
       </c>
+      <c r="ED36">
+        <v>9</v>
+      </c>
+      <c r="EE36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="EF36">
+        <v>9</v>
+      </c>
+      <c r="EH36">
+        <v>9</v>
+      </c>
+      <c r="EI36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="EJ36">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -38983,6 +39855,36 @@
       <c r="DY37" t="inlineStr">
         <is>
           <t xml:space="preserve">}</t>
+        </is>
+      </c>
+      <c r="ED37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="EE37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="EF37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="EH37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="EI37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="EJ37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
         </is>
       </c>
     </row>
@@ -39895,6 +40797,36 @@
           <t xml:space="preserve">BACKSLASH</t>
         </is>
       </c>
+      <c r="ED43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="EE43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="EF43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="EH43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="EI43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="EJ43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -40234,6 +41166,36 @@
           <t xml:space="preserve">ACUTE_ACCENT</t>
         </is>
       </c>
+      <c r="ED44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="EE44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="EF44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="EH44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="EI44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="EJ44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -40555,6 +41517,26 @@
           <t xml:space="preserve">ACUTE_ACCENT</t>
         </is>
       </c>
+      <c r="ED45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SHA</t>
+        </is>
+      </c>
+      <c r="EE45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SHA</t>
+        </is>
+      </c>
+      <c r="EH45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SHA</t>
+        </is>
+      </c>
+      <c r="EI45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SHA</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -40880,6 +41862,26 @@
       <c r="EB46" t="inlineStr">
         <is>
           <t xml:space="preserve">[</t>
+        </is>
+      </c>
+      <c r="ED46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DJE</t>
+        </is>
+      </c>
+      <c r="EE46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DJE</t>
+        </is>
+      </c>
+      <c r="EH46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_GJE</t>
+        </is>
+      </c>
+      <c r="EI46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_GJE</t>
         </is>
       </c>
     </row>
@@ -41339,6 +42341,26 @@
           <t xml:space="preserve">'</t>
         </is>
       </c>
+      <c r="ED48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZHE</t>
+        </is>
+      </c>
+      <c r="EE48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZHE</t>
+        </is>
+      </c>
+      <c r="EH48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZHE</t>
+        </is>
+      </c>
+      <c r="EI48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZHE</t>
+        </is>
+      </c>
     </row>
     <row r="49" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="93" t="s">
@@ -41637,6 +42659,26 @@
       <c r="EA49" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_00C7</t>
+        </is>
+      </c>
+      <c r="ED49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_CHE</t>
+        </is>
+      </c>
+      <c r="EE49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_CHE</t>
+        </is>
+      </c>
+      <c r="EH49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_CHE</t>
+        </is>
+      </c>
+      <c r="EI49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_CHE</t>
         </is>
       </c>
     </row>
@@ -41946,6 +42988,26 @@
       <c r="EB50" t="inlineStr">
         <is>
           <t xml:space="preserve">~</t>
+        </is>
+      </c>
+      <c r="ED50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TSHE</t>
+        </is>
+      </c>
+      <c r="EE50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TSHE</t>
+        </is>
+      </c>
+      <c r="EH50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_KJE</t>
+        </is>
+      </c>
+      <c r="EI50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_KJE</t>
         </is>
       </c>
     </row>
@@ -43304,6 +44366,36 @@
           <t xml:space="preserve">|</t>
         </is>
       </c>
+      <c r="ED55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="EE55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="EF55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="EH55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="EI55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="EJ55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
     </row>
     <row r="56" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="141" t="s">
@@ -43565,6 +44657,22 @@
       <c r="EC56">
         <v>52</v>
       </c>
+      <c r="EE56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EG56">
+        <v>50</v>
+      </c>
+      <c r="EI56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EK56">
+        <v>50</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -43826,6 +44934,22 @@
       <c r="EC57">
         <v>12</v>
       </c>
+      <c r="EE57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EG57">
+        <v>13</v>
+      </c>
+      <c r="EI57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="EK57">
+        <v>13</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -44075,6 +45199,18 @@
       <c r="EC58">
         <v>52</v>
       </c>
+      <c r="EE58">
+        <v>30</v>
+      </c>
+      <c r="EG58">
+        <v>50</v>
+      </c>
+      <c r="EI58">
+        <v>30</v>
+      </c>
+      <c r="EK58">
+        <v>50</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -44324,6 +45460,18 @@
       <c r="EC59">
         <v>12</v>
       </c>
+      <c r="EE59">
+        <v>0</v>
+      </c>
+      <c r="EG59">
+        <v>13</v>
+      </c>
+      <c r="EI59">
+        <v>0</v>
+      </c>
+      <c r="EK59">
+        <v>13</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -44573,6 +45721,18 @@
       <c r="EC60">
         <v>52</v>
       </c>
+      <c r="EE60">
+        <v>30</v>
+      </c>
+      <c r="EG60">
+        <v>50</v>
+      </c>
+      <c r="EI60">
+        <v>30</v>
+      </c>
+      <c r="EK60">
+        <v>50</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -44821,6 +45981,18 @@
       </c>
       <c r="EC61">
         <v>12</v>
+      </c>
+      <c r="EE61">
+        <v>0</v>
+      </c>
+      <c r="EG61">
+        <v>13</v>
+      </c>
+      <c r="EI61">
+        <v>0</v>
+      </c>
+      <c r="EK61">
+        <v>13</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
polykybd: add Persian (fa-IR) layout + Perso-Arabic font support
Phase 3 (Arabic). Added 13 Perso-Arabic glyphs (Persian pe/che/je/gaf/keheh/
farsi-yeh + Urdu tteh/ddal/rreh/noon-ghunna/heh-doachashmee/heh-goal/yeh-barree)
to named_glyphs and a new _PerArab_ Arabic font variant; regenerated
arabic_fonts.h with the pinned fontconvert (FreeType 2.13.3/HarfBuzz 2.6.7) -
+195 lines, zero changes to existing Arabic glyphs (generate_fonts.py --check
reproduces all committed headers).

  fa-IR Persian (ISIRI 2901 standard)

Urdu glyphs+font are now in place (layout to follow). Persian layout NEEDS a
review pass (shift diacritic layer and Persian-Indic digits intentionally
omitted for now). All existing languages regenerate identically (mk-MK only
gains trailing commas).

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -29658,92 +29658,196 @@
       <c r="E973" s="7"/>
     </row>
     <row r="974" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A974" s="7"/>
-      <c r="B974" s="7"/>
+      <c r="A974" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_PEH</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t xml:space="preserve">67E</t>
+        </is>
+      </c>
       <c r="C974" s="7"/>
       <c r="D974" s="7"/>
       <c r="E974" s="7"/>
     </row>
     <row r="975" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A975" s="7"/>
-      <c r="B975" s="7"/>
+      <c r="A975" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TCHEH</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t xml:space="preserve">686</t>
+        </is>
+      </c>
       <c r="C975" s="7"/>
       <c r="D975" s="7"/>
       <c r="E975" s="7"/>
     </row>
     <row r="976" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A976" s="7"/>
-      <c r="B976" s="7"/>
+      <c r="A976" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEH</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t xml:space="preserve">698</t>
+        </is>
+      </c>
       <c r="C976" s="7"/>
       <c r="D976" s="7"/>
       <c r="E976" s="7"/>
     </row>
     <row r="977" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A977" s="7"/>
-      <c r="B977" s="7"/>
+      <c r="A977" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GAF</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6AF</t>
+        </is>
+      </c>
       <c r="C977" s="7"/>
       <c r="D977" s="7"/>
       <c r="E977" s="7"/>
     </row>
     <row r="978" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A978" s="7"/>
-      <c r="B978" s="7"/>
+      <c r="A978" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KEHEH</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6A9</t>
+        </is>
+      </c>
       <c r="C978" s="7"/>
       <c r="D978" s="7"/>
       <c r="E978" s="7"/>
     </row>
     <row r="979" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A979" s="7"/>
-      <c r="B979" s="7"/>
+      <c r="A979" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FARSI_YEH</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6CC</t>
+        </is>
+      </c>
       <c r="C979" s="7"/>
       <c r="D979" s="7"/>
       <c r="E979" s="7"/>
     </row>
     <row r="980" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A980" s="7"/>
-      <c r="B980" s="7"/>
+      <c r="A980" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TTEH</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t xml:space="preserve">679</t>
+        </is>
+      </c>
       <c r="C980" s="7"/>
       <c r="D980" s="7"/>
       <c r="E980" s="7"/>
     </row>
     <row r="981" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A981" s="7"/>
-      <c r="B981" s="7"/>
+      <c r="A981" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DDAL</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t xml:space="preserve">688</t>
+        </is>
+      </c>
       <c r="C981" s="7"/>
       <c r="D981" s="7"/>
       <c r="E981" s="7"/>
     </row>
     <row r="982" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A982" s="7"/>
-      <c r="B982" s="7"/>
+      <c r="A982" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_RREH</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t xml:space="preserve">691</t>
+        </is>
+      </c>
       <c r="C982" s="7"/>
       <c r="D982" s="7"/>
       <c r="E982" s="7"/>
     </row>
     <row r="983" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A983" s="7"/>
-      <c r="B983" s="7"/>
+      <c r="A983" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON_GHUNNA</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6BA</t>
+        </is>
+      </c>
       <c r="C983" s="7"/>
       <c r="D983" s="7"/>
       <c r="E983" s="7"/>
     </row>
     <row r="984" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A984" s="7"/>
-      <c r="B984" s="7"/>
+      <c r="A984" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_DOACHASHMEE</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6BE</t>
+        </is>
+      </c>
       <c r="C984" s="7"/>
       <c r="D984" s="7"/>
       <c r="E984" s="7"/>
     </row>
     <row r="985" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A985" s="7"/>
-      <c r="B985" s="7"/>
+      <c r="A985" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_GOAL</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6C1</t>
+        </is>
+      </c>
       <c r="C985" s="7"/>
       <c r="D985" s="7"/>
       <c r="E985" s="7"/>
     </row>
     <row r="986" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A986" s="7"/>
-      <c r="B986" s="7"/>
+      <c r="A986" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_BARREE</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6D2</t>
+        </is>
+      </c>
       <c r="C986" s="7"/>
       <c r="D986" s="7"/>
       <c r="E986" s="7"/>
@@ -30732,7 +30836,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:EK79"/>
+  <dimension ref="A1:EO79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -31027,6 +31131,11 @@
           <t xml:space="preserve">mk-MK</t>
         </is>
       </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fa-IR</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -31217,6 +31326,16 @@
       <c r="EI2" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_A</t>
+        </is>
+      </c>
+      <c r="EL2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SHEEN</t>
+        </is>
+      </c>
+      <c r="EN2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SHEEN</t>
         </is>
       </c>
     </row>
@@ -31407,6 +31526,16 @@
           <t xml:space="preserve">CYRILLIC_BE</t>
         </is>
       </c>
+      <c r="EL3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THAL</t>
+        </is>
+      </c>
+      <c r="EN3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THAL</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -31601,6 +31730,21 @@
           <t xml:space="preserve">CYRILLIC_TSE</t>
         </is>
       </c>
+      <c r="EL4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAIN</t>
+        </is>
+      </c>
+      <c r="EM4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEH</t>
+        </is>
+      </c>
+      <c r="EN4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAIN</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -31790,6 +31934,16 @@
           <t xml:space="preserve">CYRILLIC_DE</t>
         </is>
       </c>
+      <c r="EL5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FARSI_YEH</t>
+        </is>
+      </c>
+      <c r="EN5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FARSI_YEH</t>
+        </is>
+      </c>
     </row>
     <row r="6" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="93" t="s">
@@ -32035,6 +32189,16 @@
       <c r="EI6" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_IE</t>
+        </is>
+      </c>
+      <c r="EL6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THEH</t>
+        </is>
+      </c>
+      <c r="EN6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THEH</t>
         </is>
       </c>
     </row>
@@ -32225,6 +32389,16 @@
           <t xml:space="preserve">CYRILLIC_EF</t>
         </is>
       </c>
+      <c r="EL7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_BEH</t>
+        </is>
+      </c>
+      <c r="EN7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_BEH</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -32416,6 +32590,16 @@
           <t xml:space="preserve">CYRILLIC_GHE</t>
         </is>
       </c>
+      <c r="EL8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_LAM</t>
+        </is>
+      </c>
+      <c r="EN8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_LAM</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -32597,6 +32781,16 @@
           <t xml:space="preserve">CYRILLIC_HA</t>
         </is>
       </c>
+      <c r="EL9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ALEF</t>
+        </is>
+      </c>
+      <c r="EN9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ALEF</t>
+        </is>
+      </c>
     </row>
     <row r="10" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="93" t="s">
@@ -32791,6 +32985,16 @@
       <c r="EI10" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_I</t>
+        </is>
+      </c>
+      <c r="EL10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH</t>
+        </is>
+      </c>
+      <c r="EN10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH</t>
         </is>
       </c>
     </row>
@@ -32978,6 +33182,16 @@
           <t xml:space="preserve">CYRILLIC_JE</t>
         </is>
       </c>
+      <c r="EL11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH</t>
+        </is>
+      </c>
+      <c r="EN11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH</t>
+        </is>
+      </c>
     </row>
     <row r="12" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
@@ -33166,6 +33380,16 @@
           <t xml:space="preserve">CYRILLIC_KA</t>
         </is>
       </c>
+      <c r="EL12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON</t>
+        </is>
+      </c>
+      <c r="EN12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -33356,6 +33580,16 @@
           <t xml:space="preserve">CYRILLIC_EL</t>
         </is>
       </c>
+      <c r="EL13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_MEEM</t>
+        </is>
+      </c>
+      <c r="EN13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_MEEM</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -33555,6 +33789,16 @@
       <c r="EI14" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_EM</t>
+        </is>
+      </c>
+      <c r="EL14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_PEH</t>
+        </is>
+      </c>
+      <c r="EN14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_PEH</t>
         </is>
       </c>
     </row>
@@ -33752,6 +33996,16 @@
           <t xml:space="preserve">CYRILLIC_EN</t>
         </is>
       </c>
+      <c r="EL15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAL</t>
+        </is>
+      </c>
+      <c r="EN15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAL</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -33937,6 +34191,16 @@
           <t xml:space="preserve">CYRILLIC_O</t>
         </is>
       </c>
+      <c r="EL16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KHAH</t>
+        </is>
+      </c>
+      <c r="EN16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KHAH</t>
+        </is>
+      </c>
     </row>
     <row r="17" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
@@ -34122,6 +34386,16 @@
           <t xml:space="preserve">CYRILLIC_PE</t>
         </is>
       </c>
+      <c r="EL17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HAH</t>
+        </is>
+      </c>
+      <c r="EN17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HAH</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="93" t="s">
@@ -34334,6 +34608,16 @@
       <c r="EI18" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_LJE</t>
+        </is>
+      </c>
+      <c r="EL18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAD</t>
+        </is>
+      </c>
+      <c r="EN18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAD</t>
         </is>
       </c>
     </row>
@@ -34525,6 +34809,16 @@
           <t xml:space="preserve">CYRILLIC_ER</t>
         </is>
       </c>
+      <c r="EL19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_QAF</t>
+        </is>
+      </c>
+      <c r="EN19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_QAF</t>
+        </is>
+      </c>
     </row>
     <row r="20" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="93" t="s">
@@ -34720,6 +35014,16 @@
       <c r="EI20" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_ES</t>
+        </is>
+      </c>
+      <c r="EL20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEEN</t>
+        </is>
+      </c>
+      <c r="EN20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEEN</t>
         </is>
       </c>
     </row>
@@ -34901,6 +35205,16 @@
           <t xml:space="preserve">CYRILLIC_TE</t>
         </is>
       </c>
+      <c r="EL21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FEH</t>
+        </is>
+      </c>
+      <c r="EN21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FEH</t>
+        </is>
+      </c>
     </row>
     <row r="22" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="93" t="s">
@@ -35095,6 +35409,16 @@
           <t xml:space="preserve">CYRILLIC_U</t>
         </is>
       </c>
+      <c r="EL22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_AIN</t>
+        </is>
+      </c>
+      <c r="EN22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_AIN</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -35285,6 +35609,16 @@
           <t xml:space="preserve">CYRILLIC_VE</t>
         </is>
       </c>
+      <c r="EL23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_REH</t>
+        </is>
+      </c>
+      <c r="EN23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_REH</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -35485,6 +35819,16 @@
       <c r="EI24" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_NJE</t>
+        </is>
+      </c>
+      <c r="EL24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SAD</t>
+        </is>
+      </c>
+      <c r="EN24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SAD</t>
         </is>
       </c>
     </row>
@@ -35672,6 +36016,16 @@
           <t xml:space="preserve">CYRILLIC_DZHE</t>
         </is>
       </c>
+      <c r="EL25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TAH</t>
+        </is>
+      </c>
+      <c r="EN25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TAH</t>
+        </is>
+      </c>
     </row>
     <row r="26" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="93" t="s">
@@ -35891,6 +36245,16 @@
           <t xml:space="preserve">CYRILLIC_DZE</t>
         </is>
       </c>
+      <c r="EL26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GHAIN</t>
+        </is>
+      </c>
+      <c r="EN26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GHAIN</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -36122,6 +36486,16 @@
       <c r="EI27" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_ZE</t>
+        </is>
+      </c>
+      <c r="EL27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAH</t>
+        </is>
+      </c>
+      <c r="EN27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAH</t>
         </is>
       </c>
     </row>
@@ -41537,6 +41911,16 @@
           <t xml:space="preserve">CYRILLIC_SHA</t>
         </is>
       </c>
+      <c r="EL45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEEM</t>
+        </is>
+      </c>
+      <c r="EN45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEEM</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -41882,6 +42266,16 @@
       <c r="EI46" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_GJE</t>
+        </is>
+      </c>
+      <c r="EL46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TCHEH</t>
+        </is>
+      </c>
+      <c r="EN46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TCHEH</t>
         </is>
       </c>
     </row>
@@ -42681,6 +43075,16 @@
           <t xml:space="preserve">CYRILLIC_CHE</t>
         </is>
       </c>
+      <c r="EL49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KEHEH</t>
+        </is>
+      </c>
+      <c r="EN49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KEHEH</t>
+        </is>
+      </c>
     </row>
     <row r="50" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="93" t="s">
@@ -43010,6 +43414,16 @@
           <t xml:space="preserve">CYRILLIC_KJE</t>
         </is>
       </c>
+      <c r="EL50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GAF</t>
+        </is>
+      </c>
+      <c r="EN50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GAF</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -43561,6 +43975,16 @@
       </c>
       <c r="DE52" s="115" t="s">
         <v>1181</v>
+      </c>
+      <c r="EL52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_WAW</t>
+        </is>
+      </c>
+      <c r="EN52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_WAW</t>
+        </is>
       </c>
     </row>
     <row r="53" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -44673,6 +45097,12 @@
       <c r="EK56">
         <v>50</v>
       </c>
+      <c r="EM56">
+        <v>42</v>
+      </c>
+      <c r="EO56">
+        <v>52</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -44950,6 +45380,12 @@
       <c r="EK57">
         <v>13</v>
       </c>
+      <c r="EM57">
+        <v>0</v>
+      </c>
+      <c r="EO57">
+        <v>13</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -45211,6 +45647,12 @@
       <c r="EK58">
         <v>50</v>
       </c>
+      <c r="EM58">
+        <v>27</v>
+      </c>
+      <c r="EO58">
+        <v>52</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -45472,6 +45914,12 @@
       <c r="EK59">
         <v>13</v>
       </c>
+      <c r="EM59">
+        <v>0</v>
+      </c>
+      <c r="EO59">
+        <v>13</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -45733,6 +46181,12 @@
       <c r="EK60">
         <v>50</v>
       </c>
+      <c r="EM60">
+        <v>42</v>
+      </c>
+      <c r="EO60">
+        <v>52</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -45992,6 +46446,12 @@
         <v>0</v>
       </c>
       <c r="EK61">
+        <v>13</v>
+      </c>
+      <c r="EM61">
+        <v>0</v>
+      </c>
+      <c r="EO61">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: fix unterminated char32 string for the double-quote key
The number-row KC_2 shift (and Slovak's ô key) used a raw double quote, which cog
emitted as U""" - an unterminated literal that broke the build. Use the QUOTE
named glyph (U+0022), matching how the existing layouts encode it. Caught by the
first full split72 compile.

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -37155,7 +37155,7 @@
       </c>
       <c r="DG29" t="inlineStr">
         <is>
-          <t xml:space="preserve">"</t>
+          <t xml:space="preserve">QUOTE</t>
         </is>
       </c>
       <c r="DH29">
@@ -37200,7 +37200,7 @@
       </c>
       <c r="DW29" t="inlineStr">
         <is>
-          <t xml:space="preserve">"</t>
+          <t xml:space="preserve">QUOTE</t>
         </is>
       </c>
       <c r="DX29">
@@ -37216,7 +37216,7 @@
       </c>
       <c r="EE29" t="inlineStr">
         <is>
-          <t xml:space="preserve">"</t>
+          <t xml:space="preserve">QUOTE</t>
         </is>
       </c>
       <c r="EF29">
@@ -37227,7 +37227,7 @@
       </c>
       <c r="EI29" t="inlineStr">
         <is>
-          <t xml:space="preserve">"</t>
+          <t xml:space="preserve">QUOTE</t>
         </is>
       </c>
       <c r="EJ29">
@@ -43027,7 +43027,7 @@
       </c>
       <c r="DK49" t="inlineStr">
         <is>
-          <t xml:space="preserve">"</t>
+          <t xml:space="preserve">QUOTE</t>
         </is>
       </c>
       <c r="DL49" t="inlineStr">

</xml_diff>

<commit_message>
polykybd: add Hindi/Marathi/Nepali (Devanagari InScript) + Mongolian
Gap 2 part 1 (40 languages total). New Devanagari font: NotoSansDevanagari source
+ devanagari/_Deva_ range (U+0900-097F) in fonts.yaml + dl-fonts.sh, 83 Devanagari
named glyphs, generated devanagari_fonts.h with the pinned fontconvert (other
headers byte-unchanged; --check passes). InScript layout taken verbatim from the
xkb 'in' deva variant (BIS standard), shared by hi-IN/mr-IN/ne-NP. Mongolian
(mn-MN) from xkb 'mn' (no new glyphs; uses Өө/Үү). Re-cogged ALL language files
(lang_lut.*, keycode_helper.h, hid_com.c, split72 keymap.c) so the four are
selectable on the _LL layer + reported to the host; flags regenerated.
split72:default builds clean (~523 KB).

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -29853,582 +29853,1246 @@
       <c r="E986" s="7"/>
     </row>
     <row r="987" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A987" s="7"/>
-      <c r="B987" s="7"/>
+      <c r="A987" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0901</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t xml:space="preserve">901</t>
+        </is>
+      </c>
       <c r="C987" s="7"/>
       <c r="D987" s="7"/>
       <c r="E987" s="7"/>
     </row>
     <row r="988" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A988" s="7"/>
-      <c r="B988" s="7"/>
+      <c r="A988" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t xml:space="preserve">902</t>
+        </is>
+      </c>
       <c r="C988" s="7"/>
       <c r="D988" s="7"/>
       <c r="E988" s="7"/>
     </row>
     <row r="989" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A989" s="7"/>
-      <c r="B989" s="7"/>
+      <c r="A989" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0903</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t xml:space="preserve">903</t>
+        </is>
+      </c>
       <c r="C989" s="7"/>
       <c r="D989" s="7"/>
       <c r="E989" s="7"/>
     </row>
     <row r="990" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A990" s="7"/>
-      <c r="B990" s="7"/>
+      <c r="A990" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0905</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t xml:space="preserve">905</t>
+        </is>
+      </c>
       <c r="C990" s="7"/>
       <c r="D990" s="7"/>
       <c r="E990" s="7"/>
     </row>
     <row r="991" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A991" s="7"/>
-      <c r="B991" s="7"/>
+      <c r="A991" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0906</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t xml:space="preserve">906</t>
+        </is>
+      </c>
       <c r="C991" s="7"/>
       <c r="D991" s="7"/>
       <c r="E991" s="7"/>
     </row>
     <row r="992" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A992" s="7"/>
-      <c r="B992" s="7"/>
+      <c r="A992" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0907</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t xml:space="preserve">907</t>
+        </is>
+      </c>
       <c r="C992" s="7"/>
       <c r="D992" s="7"/>
       <c r="E992" s="7"/>
     </row>
     <row r="993" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A993" s="7"/>
-      <c r="B993" s="7"/>
+      <c r="A993" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0908</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t xml:space="preserve">908</t>
+        </is>
+      </c>
       <c r="C993" s="7"/>
       <c r="D993" s="7"/>
       <c r="E993" s="7"/>
     </row>
     <row r="994" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A994" s="7"/>
-      <c r="B994" s="7"/>
+      <c r="A994" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0909</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t xml:space="preserve">909</t>
+        </is>
+      </c>
       <c r="C994" s="7"/>
       <c r="D994" s="7"/>
       <c r="E994" s="7"/>
     </row>
     <row r="995" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A995" s="7"/>
-      <c r="B995" s="7"/>
+      <c r="A995" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090A</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90A</t>
+        </is>
+      </c>
       <c r="C995" s="7"/>
       <c r="D995" s="7"/>
       <c r="E995" s="7"/>
     </row>
     <row r="996" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A996" s="7"/>
-      <c r="B996" s="7"/>
+      <c r="A996" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090B</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90B</t>
+        </is>
+      </c>
       <c r="C996" s="7"/>
       <c r="D996" s="7"/>
       <c r="E996" s="7"/>
     </row>
     <row r="997" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A997" s="7"/>
-      <c r="B997" s="7"/>
+      <c r="A997" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090D</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90D</t>
+        </is>
+      </c>
       <c r="C997" s="7"/>
       <c r="D997" s="7"/>
       <c r="E997" s="7"/>
     </row>
     <row r="998" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A998" s="7"/>
-      <c r="B998" s="7"/>
+      <c r="A998" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090E</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90E</t>
+        </is>
+      </c>
       <c r="C998" s="7"/>
       <c r="D998" s="7"/>
       <c r="E998" s="7"/>
     </row>
     <row r="999" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A999" s="7"/>
-      <c r="B999" s="7"/>
+      <c r="A999" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090F</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90F</t>
+        </is>
+      </c>
       <c r="C999" s="7"/>
       <c r="D999" s="7"/>
       <c r="E999" s="7"/>
     </row>
     <row r="1000" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1000" s="7"/>
-      <c r="B1000" s="7"/>
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0910</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t xml:space="preserve">910</t>
+        </is>
+      </c>
       <c r="C1000" s="7"/>
       <c r="D1000" s="7"/>
       <c r="E1000" s="7"/>
     </row>
     <row r="1001" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1001" s="7"/>
-      <c r="B1001" s="7"/>
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0911</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t xml:space="preserve">911</t>
+        </is>
+      </c>
       <c r="C1001" s="7"/>
       <c r="D1001" s="7"/>
       <c r="E1001" s="7"/>
     </row>
     <row r="1002" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1002" s="7"/>
-      <c r="B1002" s="7"/>
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0912</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t xml:space="preserve">912</t>
+        </is>
+      </c>
       <c r="C1002" s="7"/>
       <c r="D1002" s="7"/>
       <c r="E1002" s="7"/>
     </row>
     <row r="1003" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1003" s="7"/>
-      <c r="B1003" s="7"/>
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0913</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t xml:space="preserve">913</t>
+        </is>
+      </c>
       <c r="C1003" s="7"/>
       <c r="D1003" s="7"/>
       <c r="E1003" s="7"/>
     </row>
     <row r="1004" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1004" s="7"/>
-      <c r="B1004" s="7"/>
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0914</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t xml:space="preserve">914</t>
+        </is>
+      </c>
       <c r="C1004" s="7"/>
       <c r="D1004" s="7"/>
       <c r="E1004" s="7"/>
     </row>
     <row r="1005" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1005" s="7"/>
-      <c r="B1005" s="7"/>
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t xml:space="preserve">915</t>
+        </is>
+      </c>
       <c r="C1005" s="7"/>
       <c r="D1005" s="7"/>
       <c r="E1005" s="7"/>
     </row>
     <row r="1006" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1006" s="7"/>
-      <c r="B1006" s="7"/>
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0916</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t xml:space="preserve">916</t>
+        </is>
+      </c>
       <c r="C1006" s="7"/>
       <c r="D1006" s="7"/>
       <c r="E1006" s="7"/>
     </row>
     <row r="1007" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1007" s="7"/>
-      <c r="B1007" s="7"/>
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t xml:space="preserve">917</t>
+        </is>
+      </c>
       <c r="C1007" s="7"/>
       <c r="D1007" s="7"/>
       <c r="E1007" s="7"/>
     </row>
     <row r="1008" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1008" s="7"/>
-      <c r="B1008" s="7"/>
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0918</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t xml:space="preserve">918</t>
+        </is>
+      </c>
       <c r="C1008" s="7"/>
       <c r="D1008" s="7"/>
       <c r="E1008" s="7"/>
     </row>
     <row r="1009" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1009" s="7"/>
-      <c r="B1009" s="7"/>
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0919</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t xml:space="preserve">919</t>
+        </is>
+      </c>
       <c r="C1009" s="7"/>
       <c r="D1009" s="7"/>
       <c r="E1009" s="7"/>
     </row>
     <row r="1010" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1010" s="7"/>
-      <c r="B1010" s="7"/>
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91A</t>
+        </is>
+      </c>
       <c r="C1010" s="7"/>
       <c r="D1010" s="7"/>
       <c r="E1010" s="7"/>
     </row>
     <row r="1011" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1011" s="7"/>
-      <c r="B1011" s="7"/>
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091B</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91B</t>
+        </is>
+      </c>
       <c r="C1011" s="7"/>
       <c r="D1011" s="7"/>
       <c r="E1011" s="7"/>
     </row>
     <row r="1012" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1012" s="7"/>
-      <c r="B1012" s="7"/>
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91C</t>
+        </is>
+      </c>
       <c r="C1012" s="7"/>
       <c r="D1012" s="7"/>
       <c r="E1012" s="7"/>
     </row>
     <row r="1013" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1013" s="7"/>
-      <c r="B1013" s="7"/>
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091D</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91D</t>
+        </is>
+      </c>
       <c r="C1013" s="7"/>
       <c r="D1013" s="7"/>
       <c r="E1013" s="7"/>
     </row>
     <row r="1014" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1014" s="7"/>
-      <c r="B1014" s="7"/>
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091E</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91E</t>
+        </is>
+      </c>
       <c r="C1014" s="7"/>
       <c r="D1014" s="7"/>
       <c r="E1014" s="7"/>
     </row>
     <row r="1015" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1015" s="7"/>
-      <c r="B1015" s="7"/>
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91F</t>
+        </is>
+      </c>
       <c r="C1015" s="7"/>
       <c r="D1015" s="7"/>
       <c r="E1015" s="7"/>
     </row>
     <row r="1016" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1016" s="7"/>
-      <c r="B1016" s="7"/>
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0920</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t xml:space="preserve">920</t>
+        </is>
+      </c>
       <c r="C1016" s="7"/>
       <c r="D1016" s="7"/>
       <c r="E1016" s="7"/>
     </row>
     <row r="1017" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1017" s="7"/>
-      <c r="B1017" s="7"/>
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t xml:space="preserve">921</t>
+        </is>
+      </c>
       <c r="C1017" s="7"/>
       <c r="D1017" s="7"/>
       <c r="E1017" s="7"/>
     </row>
     <row r="1018" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1018" s="7"/>
-      <c r="B1018" s="7"/>
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0922</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t xml:space="preserve">922</t>
+        </is>
+      </c>
       <c r="C1018" s="7"/>
       <c r="D1018" s="7"/>
       <c r="E1018" s="7"/>
     </row>
     <row r="1019" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1019" s="7"/>
-      <c r="B1019" s="7"/>
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0923</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t xml:space="preserve">923</t>
+        </is>
+      </c>
       <c r="C1019" s="7"/>
       <c r="D1019" s="7"/>
       <c r="E1019" s="7"/>
     </row>
     <row r="1020" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1020" s="7"/>
-      <c r="B1020" s="7"/>
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t xml:space="preserve">924</t>
+        </is>
+      </c>
       <c r="C1020" s="7"/>
       <c r="D1020" s="7"/>
       <c r="E1020" s="7"/>
     </row>
     <row r="1021" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1021" s="7"/>
-      <c r="B1021" s="7"/>
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0925</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t xml:space="preserve">925</t>
+        </is>
+      </c>
       <c r="C1021" s="7"/>
       <c r="D1021" s="7"/>
       <c r="E1021" s="7"/>
     </row>
     <row r="1022" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1022" s="7"/>
-      <c r="B1022" s="7"/>
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t xml:space="preserve">926</t>
+        </is>
+      </c>
       <c r="C1022" s="7"/>
       <c r="D1022" s="7"/>
       <c r="E1022" s="7"/>
     </row>
     <row r="1023" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1023" s="7"/>
-      <c r="B1023" s="7"/>
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0927</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t xml:space="preserve">927</t>
+        </is>
+      </c>
       <c r="C1023" s="7"/>
       <c r="D1023" s="7"/>
       <c r="E1023" s="7"/>
     </row>
     <row r="1024" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1024" s="7"/>
-      <c r="B1024" s="7"/>
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t xml:space="preserve">928</t>
+        </is>
+      </c>
       <c r="C1024" s="7"/>
       <c r="D1024" s="7"/>
       <c r="E1024" s="7"/>
     </row>
     <row r="1025" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1025" s="7"/>
-      <c r="B1025" s="7"/>
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0929</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t xml:space="preserve">929</t>
+        </is>
+      </c>
       <c r="C1025" s="7"/>
       <c r="D1025" s="7"/>
       <c r="E1025" s="7"/>
     </row>
     <row r="1026" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1026" s="7"/>
-      <c r="B1026" s="7"/>
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92A</t>
+        </is>
+      </c>
       <c r="C1026" s="7"/>
       <c r="D1026" s="7"/>
       <c r="E1026" s="7"/>
     </row>
     <row r="1027" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1027" s="7"/>
-      <c r="B1027" s="7"/>
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092B</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92B</t>
+        </is>
+      </c>
       <c r="C1027" s="7"/>
       <c r="D1027" s="7"/>
       <c r="E1027" s="7"/>
     </row>
     <row r="1028" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1028" s="7"/>
-      <c r="B1028" s="7"/>
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92C</t>
+        </is>
+      </c>
       <c r="C1028" s="7"/>
       <c r="D1028" s="7"/>
       <c r="E1028" s="7"/>
     </row>
     <row r="1029" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1029" s="7"/>
-      <c r="B1029" s="7"/>
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092D</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92D</t>
+        </is>
+      </c>
       <c r="C1029" s="7"/>
       <c r="D1029" s="7"/>
       <c r="E1029" s="7"/>
     </row>
     <row r="1030" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1030" s="7"/>
-      <c r="B1030" s="7"/>
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92E</t>
+        </is>
+      </c>
       <c r="C1030" s="7"/>
       <c r="D1030" s="7"/>
       <c r="E1030" s="7"/>
     </row>
     <row r="1031" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1031" s="7"/>
-      <c r="B1031" s="7"/>
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92F</t>
+        </is>
+      </c>
       <c r="C1031" s="7"/>
       <c r="D1031" s="7"/>
       <c r="E1031" s="7"/>
     </row>
     <row r="1032" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1032" s="7"/>
-      <c r="B1032" s="7"/>
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t xml:space="preserve">930</t>
+        </is>
+      </c>
       <c r="C1032" s="7"/>
       <c r="D1032" s="7"/>
       <c r="E1032" s="7"/>
     </row>
     <row r="1033" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1033" s="7"/>
-      <c r="B1033" s="7"/>
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0931</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t xml:space="preserve">931</t>
+        </is>
+      </c>
       <c r="C1033" s="7"/>
       <c r="D1033" s="7"/>
       <c r="E1033" s="7"/>
     </row>
     <row r="1034" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1034" s="7"/>
-      <c r="B1034" s="7"/>
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t xml:space="preserve">932</t>
+        </is>
+      </c>
       <c r="C1034" s="7"/>
       <c r="D1034" s="7"/>
       <c r="E1034" s="7"/>
     </row>
     <row r="1035" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1035" s="7"/>
-      <c r="B1035" s="7"/>
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0933</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t xml:space="preserve">933</t>
+        </is>
+      </c>
       <c r="C1035" s="7"/>
       <c r="D1035" s="7"/>
       <c r="E1035" s="7"/>
     </row>
     <row r="1036" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1036" s="7"/>
-      <c r="B1036" s="7"/>
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0934</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t xml:space="preserve">934</t>
+        </is>
+      </c>
       <c r="C1036" s="7"/>
       <c r="D1036" s="7"/>
       <c r="E1036" s="7"/>
     </row>
     <row r="1037" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1037" s="7"/>
-      <c r="B1037" s="7"/>
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t xml:space="preserve">935</t>
+        </is>
+      </c>
       <c r="C1037" s="7"/>
       <c r="D1037" s="7"/>
       <c r="E1037" s="7"/>
     </row>
     <row r="1038" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1038" s="7"/>
-      <c r="B1038" s="7"/>
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0936</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t xml:space="preserve">936</t>
+        </is>
+      </c>
       <c r="C1038" s="7"/>
       <c r="D1038" s="7"/>
       <c r="E1038" s="7"/>
     </row>
     <row r="1039" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1039" s="7"/>
-      <c r="B1039" s="7"/>
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0937</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t xml:space="preserve">937</t>
+        </is>
+      </c>
       <c r="C1039" s="7"/>
       <c r="D1039" s="7"/>
       <c r="E1039" s="7"/>
     </row>
     <row r="1040" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1040" s="7"/>
-      <c r="B1040" s="7"/>
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t xml:space="preserve">938</t>
+        </is>
+      </c>
       <c r="C1040" s="7"/>
       <c r="D1040" s="7"/>
       <c r="E1040" s="7"/>
     </row>
     <row r="1041" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1041" s="7"/>
-      <c r="B1041" s="7"/>
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t xml:space="preserve">939</t>
+        </is>
+      </c>
       <c r="C1041" s="7"/>
       <c r="D1041" s="7"/>
       <c r="E1041" s="7"/>
     </row>
     <row r="1042" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1042" s="7"/>
-      <c r="B1042" s="7"/>
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93C</t>
+        </is>
+      </c>
       <c r="C1042" s="7"/>
       <c r="D1042" s="7"/>
       <c r="E1042" s="7"/>
     </row>
     <row r="1043" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1043" s="7"/>
-      <c r="B1043" s="7"/>
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93E</t>
+        </is>
+      </c>
       <c r="C1043" s="7"/>
       <c r="D1043" s="7"/>
       <c r="E1043" s="7"/>
     </row>
     <row r="1044" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1044" s="7"/>
-      <c r="B1044" s="7"/>
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93F</t>
+        </is>
+      </c>
       <c r="C1044" s="7"/>
       <c r="D1044" s="7"/>
       <c r="E1044" s="7"/>
     </row>
     <row r="1045" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1045" s="7"/>
-      <c r="B1045" s="7"/>
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t xml:space="preserve">940</t>
+        </is>
+      </c>
       <c r="C1045" s="7"/>
       <c r="D1045" s="7"/>
       <c r="E1045" s="7"/>
     </row>
     <row r="1046" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1046" s="7"/>
-      <c r="B1046" s="7"/>
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t xml:space="preserve">941</t>
+        </is>
+      </c>
       <c r="C1046" s="7"/>
       <c r="D1046" s="7"/>
       <c r="E1046" s="7"/>
     </row>
     <row r="1047" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1047" s="7"/>
-      <c r="B1047" s="7"/>
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t xml:space="preserve">942</t>
+        </is>
+      </c>
       <c r="C1047" s="7"/>
       <c r="D1047" s="7"/>
       <c r="E1047" s="7"/>
     </row>
     <row r="1048" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1048" s="7"/>
-      <c r="B1048" s="7"/>
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t xml:space="preserve">943</t>
+        </is>
+      </c>
       <c r="C1048" s="7"/>
       <c r="D1048" s="7"/>
       <c r="E1048" s="7"/>
     </row>
     <row r="1049" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1049" s="7"/>
-      <c r="B1049" s="7"/>
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0945</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t xml:space="preserve">945</t>
+        </is>
+      </c>
       <c r="C1049" s="7"/>
       <c r="D1049" s="7"/>
       <c r="E1049" s="7"/>
     </row>
     <row r="1050" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1050" s="7"/>
-      <c r="B1050" s="7"/>
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t xml:space="preserve">946</t>
+        </is>
+      </c>
       <c r="C1050" s="7"/>
       <c r="D1050" s="7"/>
       <c r="E1050" s="7"/>
     </row>
     <row r="1051" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1051" s="7"/>
-      <c r="B1051" s="7"/>
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t xml:space="preserve">947</t>
+        </is>
+      </c>
       <c r="C1051" s="7"/>
       <c r="D1051" s="7"/>
       <c r="E1051" s="7"/>
     </row>
     <row r="1052" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1052" s="7"/>
-      <c r="B1052" s="7"/>
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t xml:space="preserve">948</t>
+        </is>
+      </c>
       <c r="C1052" s="7"/>
       <c r="D1052" s="7"/>
       <c r="E1052" s="7"/>
     </row>
     <row r="1053" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1053" s="7"/>
-      <c r="B1053" s="7"/>
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94A</t>
+        </is>
+      </c>
       <c r="C1053" s="7"/>
       <c r="D1053" s="7"/>
       <c r="E1053" s="7"/>
     </row>
     <row r="1054" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1054" s="7"/>
-      <c r="B1054" s="7"/>
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94B</t>
+        </is>
+      </c>
       <c r="C1054" s="7"/>
       <c r="D1054" s="7"/>
       <c r="E1054" s="7"/>
     </row>
     <row r="1055" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1055" s="7"/>
-      <c r="B1055" s="7"/>
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94C</t>
+        </is>
+      </c>
       <c r="C1055" s="7"/>
       <c r="D1055" s="7"/>
       <c r="E1055" s="7"/>
     </row>
     <row r="1056" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1056" s="7"/>
-      <c r="B1056" s="7"/>
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94D</t>
+        </is>
+      </c>
       <c r="C1056" s="7"/>
       <c r="D1056" s="7"/>
       <c r="E1056" s="7"/>
     </row>
     <row r="1057" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1057" s="7"/>
-      <c r="B1057" s="7"/>
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_095F</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t xml:space="preserve">95F</t>
+        </is>
+      </c>
       <c r="C1057" s="7"/>
       <c r="D1057" s="7"/>
       <c r="E1057" s="7"/>
     </row>
     <row r="1058" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1058" s="7"/>
-      <c r="B1058" s="7"/>
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0964</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t xml:space="preserve">964</t>
+        </is>
+      </c>
       <c r="C1058" s="7"/>
       <c r="D1058" s="7"/>
       <c r="E1058" s="7"/>
     </row>
     <row r="1059" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1059" s="7"/>
-      <c r="B1059" s="7"/>
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t xml:space="preserve">966</t>
+        </is>
+      </c>
       <c r="C1059" s="7"/>
       <c r="D1059" s="7"/>
       <c r="E1059" s="7"/>
     </row>
     <row r="1060" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1060" s="7"/>
-      <c r="B1060" s="7"/>
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t xml:space="preserve">967</t>
+        </is>
+      </c>
       <c r="C1060" s="7"/>
       <c r="D1060" s="7"/>
       <c r="E1060" s="7"/>
     </row>
     <row r="1061" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1061" s="7"/>
-      <c r="B1061" s="7"/>
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t xml:space="preserve">968</t>
+        </is>
+      </c>
       <c r="C1061" s="7"/>
       <c r="D1061" s="7"/>
       <c r="E1061" s="7"/>
     </row>
     <row r="1062" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1062" s="7"/>
-      <c r="B1062" s="7"/>
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t xml:space="preserve">969</t>
+        </is>
+      </c>
       <c r="C1062" s="7"/>
       <c r="D1062" s="7"/>
       <c r="E1062" s="7"/>
     </row>
     <row r="1063" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1063" s="7"/>
-      <c r="B1063" s="7"/>
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96A</t>
+        </is>
+      </c>
       <c r="C1063" s="7"/>
       <c r="D1063" s="7"/>
       <c r="E1063" s="7"/>
     </row>
     <row r="1064" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1064" s="7"/>
-      <c r="B1064" s="7"/>
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96B</t>
+        </is>
+      </c>
       <c r="C1064" s="7"/>
       <c r="D1064" s="7"/>
       <c r="E1064" s="7"/>
     </row>
     <row r="1065" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1065" s="7"/>
-      <c r="B1065" s="7"/>
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96C</t>
+        </is>
+      </c>
       <c r="C1065" s="7"/>
       <c r="D1065" s="7"/>
       <c r="E1065" s="7"/>
     </row>
     <row r="1066" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1066" s="7"/>
-      <c r="B1066" s="7"/>
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96D</t>
+        </is>
+      </c>
       <c r="C1066" s="7"/>
       <c r="D1066" s="7"/>
       <c r="E1066" s="7"/>
     </row>
     <row r="1067" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1067" s="7"/>
-      <c r="B1067" s="7"/>
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96E</t>
+        </is>
+      </c>
       <c r="C1067" s="7"/>
       <c r="D1067" s="7"/>
       <c r="E1067" s="7"/>
     </row>
     <row r="1068" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1068" s="7"/>
-      <c r="B1068" s="7"/>
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96F</t>
+        </is>
+      </c>
       <c r="C1068" s="7"/>
       <c r="D1068" s="7"/>
       <c r="E1068" s="7"/>
     </row>
     <row r="1069" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1069" s="7"/>
-      <c r="B1069" s="7"/>
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0972</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t xml:space="preserve">972</t>
+        </is>
+      </c>
       <c r="C1069" s="7"/>
       <c r="D1069" s="7"/>
       <c r="E1069" s="7"/>
@@ -30836,7 +31500,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:EO79"/>
+  <dimension ref="A1:FE79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -31136,6 +31800,26 @@
           <t xml:space="preserve">fa-IR</t>
         </is>
       </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hi-IN</t>
+        </is>
+      </c>
+      <c r="ET1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mr-IN</t>
+        </is>
+      </c>
+      <c r="EX1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ne-NP</t>
+        </is>
+      </c>
+      <c r="FB1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mn-MN</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -31336,6 +32020,61 @@
       <c r="EN2" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_SHEEN</t>
+        </is>
+      </c>
+      <c r="EP2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="EQ2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0913</t>
+        </is>
+      </c>
+      <c r="ER2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="ET2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="EU2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0913</t>
+        </is>
+      </c>
+      <c r="EV2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="EX2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="EY2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0913</t>
+        </is>
+      </c>
+      <c r="EZ2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094B</t>
+        </is>
+      </c>
+      <c r="FB2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SHORT_I</t>
+        </is>
+      </c>
+      <c r="FC2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SHORT_I</t>
         </is>
       </c>
     </row>
@@ -31536,6 +32275,61 @@
           <t xml:space="preserve">ARABIC_THAL</t>
         </is>
       </c>
+      <c r="EP3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="EQ3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0934</t>
+        </is>
+      </c>
+      <c r="ER3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="ET3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="EU3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0934</t>
+        </is>
+      </c>
+      <c r="EV3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="EX3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="EY3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0934</t>
+        </is>
+      </c>
+      <c r="EZ3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0935</t>
+        </is>
+      </c>
+      <c r="FB3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EM</t>
+        </is>
+      </c>
+      <c r="FC3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EM</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -31745,6 +32539,61 @@
           <t xml:space="preserve">ARABIC_ZAIN</t>
         </is>
       </c>
+      <c r="EP4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="EQ4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0923</t>
+        </is>
+      </c>
+      <c r="ER4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="ET4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="EU4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0923</t>
+        </is>
+      </c>
+      <c r="EV4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="EX4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="EY4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0923</t>
+        </is>
+      </c>
+      <c r="EZ4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092E</t>
+        </is>
+      </c>
+      <c r="FB4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_IO</t>
+        </is>
+      </c>
+      <c r="FC4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_IO</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -31944,6 +32793,61 @@
           <t xml:space="preserve">ARABIC_FARSI_YEH</t>
         </is>
       </c>
+      <c r="EP5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="EQ5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0905</t>
+        </is>
+      </c>
+      <c r="ER5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="ET5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="EU5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0905</t>
+        </is>
+      </c>
+      <c r="EV5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="EX5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="EY5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0905</t>
+        </is>
+      </c>
+      <c r="EZ5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094D</t>
+        </is>
+      </c>
+      <c r="FB5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_BE</t>
+        </is>
+      </c>
+      <c r="FC5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_BE</t>
+        </is>
+      </c>
     </row>
     <row r="6" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="93" t="s">
@@ -32199,6 +33103,61 @@
       <c r="EN6" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_THEH</t>
+        </is>
+      </c>
+      <c r="EP6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="EQ6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0906</t>
+        </is>
+      </c>
+      <c r="ER6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="ET6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="EU6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0906</t>
+        </is>
+      </c>
+      <c r="EV6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="EX6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="EY6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0906</t>
+        </is>
+      </c>
+      <c r="EZ6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093E</t>
+        </is>
+      </c>
+      <c r="FB6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_U</t>
+        </is>
+      </c>
+      <c r="FC6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_U</t>
         </is>
       </c>
     </row>
@@ -32399,6 +33358,61 @@
           <t xml:space="preserve">ARABIC_BEH</t>
         </is>
       </c>
+      <c r="EP7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="EQ7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0907</t>
+        </is>
+      </c>
+      <c r="ER7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="ET7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="EU7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0907</t>
+        </is>
+      </c>
+      <c r="EV7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="EX7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="EY7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0907</t>
+        </is>
+      </c>
+      <c r="EZ7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093F</t>
+        </is>
+      </c>
+      <c r="FB7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_BARRED_O</t>
+        </is>
+      </c>
+      <c r="FC7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_BARRED_O</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -32600,6 +33614,61 @@
           <t xml:space="preserve">ARABIC_LAM</t>
         </is>
       </c>
+      <c r="EP8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="EQ8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0909</t>
+        </is>
+      </c>
+      <c r="ER8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="ET8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="EU8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0909</t>
+        </is>
+      </c>
+      <c r="EV8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="EX8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="EY8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0909</t>
+        </is>
+      </c>
+      <c r="EZ8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0941</t>
+        </is>
+      </c>
+      <c r="FB8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_A</t>
+        </is>
+      </c>
+      <c r="FC8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_A</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -32791,6 +33860,61 @@
           <t xml:space="preserve">ARABIC_ALEF</t>
         </is>
       </c>
+      <c r="EP9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="EQ9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092B</t>
+        </is>
+      </c>
+      <c r="ER9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="ET9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="EU9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092B</t>
+        </is>
+      </c>
+      <c r="EV9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="EX9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="EY9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092B</t>
+        </is>
+      </c>
+      <c r="EZ9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092A</t>
+        </is>
+      </c>
+      <c r="FB9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_HA</t>
+        </is>
+      </c>
+      <c r="FC9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_HA</t>
+        </is>
+      </c>
     </row>
     <row r="10" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="93" t="s">
@@ -32995,6 +34119,61 @@
       <c r="EN10" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_HEH</t>
+        </is>
+      </c>
+      <c r="EP10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="EQ10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0918</t>
+        </is>
+      </c>
+      <c r="ER10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="ET10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="EU10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0918</t>
+        </is>
+      </c>
+      <c r="EV10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="EX10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="EY10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0918</t>
+        </is>
+      </c>
+      <c r="EZ10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0917</t>
+        </is>
+      </c>
+      <c r="FB10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SHA</t>
+        </is>
+      </c>
+      <c r="FC10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SHA</t>
         </is>
       </c>
     </row>
@@ -33192,6 +34371,61 @@
           <t xml:space="preserve">ARABIC_TEH</t>
         </is>
       </c>
+      <c r="EP11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="EQ11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0931</t>
+        </is>
+      </c>
+      <c r="ER11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="ET11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="EU11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0931</t>
+        </is>
+      </c>
+      <c r="EV11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="EX11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="EY11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0931</t>
+        </is>
+      </c>
+      <c r="EZ11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0930</t>
+        </is>
+      </c>
+      <c r="FB11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ER</t>
+        </is>
+      </c>
+      <c r="FC11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ER</t>
+        </is>
+      </c>
     </row>
     <row r="12" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
@@ -33390,6 +34624,61 @@
           <t xml:space="preserve">ARABIC_NOON</t>
         </is>
       </c>
+      <c r="EP12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="EQ12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0916</t>
+        </is>
+      </c>
+      <c r="ER12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="ET12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="EU12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0916</t>
+        </is>
+      </c>
+      <c r="EV12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="EX12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="EY12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0916</t>
+        </is>
+      </c>
+      <c r="EZ12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0915</t>
+        </is>
+      </c>
+      <c r="FB12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_O</t>
+        </is>
+      </c>
+      <c r="FC12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_O</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -33590,6 +34879,61 @@
           <t xml:space="preserve">ARABIC_MEEM</t>
         </is>
       </c>
+      <c r="EP13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="EQ13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0925</t>
+        </is>
+      </c>
+      <c r="ER13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="ET13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="EU13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0925</t>
+        </is>
+      </c>
+      <c r="EV13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="EX13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="EY13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0925</t>
+        </is>
+      </c>
+      <c r="EZ13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0924</t>
+        </is>
+      </c>
+      <c r="FB13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EL</t>
+        </is>
+      </c>
+      <c r="FC13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EL</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -33799,6 +35143,61 @@
       <c r="EN14" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_PEH</t>
+        </is>
+      </c>
+      <c r="EP14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="EQ14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0936</t>
+        </is>
+      </c>
+      <c r="ER14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="ET14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="EU14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0936</t>
+        </is>
+      </c>
+      <c r="EV14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="EX14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="EY14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0936</t>
+        </is>
+      </c>
+      <c r="EZ14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0938</t>
+        </is>
+      </c>
+      <c r="FB14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TE</t>
+        </is>
+      </c>
+      <c r="FC14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TE</t>
         </is>
       </c>
     </row>
@@ -34006,6 +35405,61 @@
           <t xml:space="preserve">ARABIC_DAL</t>
         </is>
       </c>
+      <c r="EP15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="EQ15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0933</t>
+        </is>
+      </c>
+      <c r="ER15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="ET15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="EU15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0933</t>
+        </is>
+      </c>
+      <c r="EV15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="EX15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="EY15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0933</t>
+        </is>
+      </c>
+      <c r="EZ15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0932</t>
+        </is>
+      </c>
+      <c r="FB15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_I</t>
+        </is>
+      </c>
+      <c r="FC15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_I</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -34201,6 +35655,61 @@
           <t xml:space="preserve">ARABIC_KHAH</t>
         </is>
       </c>
+      <c r="EP16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="EQ16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0927</t>
+        </is>
+      </c>
+      <c r="ER16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="ET16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="EU16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0927</t>
+        </is>
+      </c>
+      <c r="EV16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="EX16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="EY16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0927</t>
+        </is>
+      </c>
+      <c r="EZ16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0926</t>
+        </is>
+      </c>
+      <c r="FB16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_STRAIGHT_U</t>
+        </is>
+      </c>
+      <c r="FC16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_STRAIGHT_U</t>
+        </is>
+      </c>
     </row>
     <row r="17" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
@@ -34396,6 +35905,61 @@
           <t xml:space="preserve">ARABIC_HAH</t>
         </is>
       </c>
+      <c r="EP17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="EQ17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091D</t>
+        </is>
+      </c>
+      <c r="ER17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="ET17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="EU17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091D</t>
+        </is>
+      </c>
+      <c r="EV17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="EX17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="EY17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091D</t>
+        </is>
+      </c>
+      <c r="EZ17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091C</t>
+        </is>
+      </c>
+      <c r="FB17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZE</t>
+        </is>
+      </c>
+      <c r="FC17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZE</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="93" t="s">
@@ -34618,6 +36182,61 @@
       <c r="EN18" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_DAD</t>
+        </is>
+      </c>
+      <c r="EP18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="EQ18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0914</t>
+        </is>
+      </c>
+      <c r="ER18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="ET18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="EU18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0914</t>
+        </is>
+      </c>
+      <c r="EV18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="EX18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="EY18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0914</t>
+        </is>
+      </c>
+      <c r="EZ18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094C</t>
+        </is>
+      </c>
+      <c r="FB18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EF</t>
+        </is>
+      </c>
+      <c r="FC18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EF</t>
         </is>
       </c>
     </row>
@@ -34819,6 +36438,61 @@
           <t xml:space="preserve">ARABIC_QAF</t>
         </is>
       </c>
+      <c r="EP19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="EQ19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0908</t>
+        </is>
+      </c>
+      <c r="ER19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="ET19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="EU19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0908</t>
+        </is>
+      </c>
+      <c r="EV19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="EX19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="EY19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0908</t>
+        </is>
+      </c>
+      <c r="EZ19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0940</t>
+        </is>
+      </c>
+      <c r="FB19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ZHE</t>
+        </is>
+      </c>
+      <c r="FC19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ZHE</t>
+        </is>
+      </c>
     </row>
     <row r="20" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="93" t="s">
@@ -35024,6 +36698,61 @@
       <c r="EN20" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_SEEN</t>
+        </is>
+      </c>
+      <c r="EP20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="EQ20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090F</t>
+        </is>
+      </c>
+      <c r="ER20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="ET20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="EU20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090F</t>
+        </is>
+      </c>
+      <c r="EV20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="EX20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="EY20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090F</t>
+        </is>
+      </c>
+      <c r="EZ20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0947</t>
+        </is>
+      </c>
+      <c r="FB20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_YERU</t>
+        </is>
+      </c>
+      <c r="FC20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_YERU</t>
         </is>
       </c>
     </row>
@@ -35215,6 +36944,61 @@
           <t xml:space="preserve">ARABIC_FEH</t>
         </is>
       </c>
+      <c r="EP21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="EQ21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090A</t>
+        </is>
+      </c>
+      <c r="ER21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="ET21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="EU21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090A</t>
+        </is>
+      </c>
+      <c r="EV21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="EX21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="EY21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090A</t>
+        </is>
+      </c>
+      <c r="EZ21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0942</t>
+        </is>
+      </c>
+      <c r="FB21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_E</t>
+        </is>
+      </c>
+      <c r="FC21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_E</t>
+        </is>
+      </c>
     </row>
     <row r="22" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="93" t="s">
@@ -35419,6 +37203,61 @@
           <t xml:space="preserve">ARABIC_AIN</t>
         </is>
       </c>
+      <c r="EP22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="EQ22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0919</t>
+        </is>
+      </c>
+      <c r="ER22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="ET22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="EU22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0919</t>
+        </is>
+      </c>
+      <c r="EV22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="EX22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="EY22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0919</t>
+        </is>
+      </c>
+      <c r="EZ22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0939</t>
+        </is>
+      </c>
+      <c r="FB22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_GHE</t>
+        </is>
+      </c>
+      <c r="FC22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_GHE</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -35619,6 +37458,61 @@
           <t xml:space="preserve">ARABIC_REH</t>
         </is>
       </c>
+      <c r="EP23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="EQ23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0929</t>
+        </is>
+      </c>
+      <c r="ER23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="ET23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="EU23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0929</t>
+        </is>
+      </c>
+      <c r="EV23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="EX23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="EY23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0929</t>
+        </is>
+      </c>
+      <c r="EZ23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0928</t>
+        </is>
+      </c>
+      <c r="FB23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_ES</t>
+        </is>
+      </c>
+      <c r="FC23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_ES</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -35829,6 +37723,61 @@
       <c r="EN24" t="inlineStr">
         <is>
           <t xml:space="preserve">ARABIC_SAD</t>
+        </is>
+      </c>
+      <c r="EP24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="EQ24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0910</t>
+        </is>
+      </c>
+      <c r="ER24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="ET24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="EU24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0910</t>
+        </is>
+      </c>
+      <c r="EV24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="EX24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="EY24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0910</t>
+        </is>
+      </c>
+      <c r="EZ24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0948</t>
+        </is>
+      </c>
+      <c r="FB24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_TSE</t>
+        </is>
+      </c>
+      <c r="FC24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_TSE</t>
         </is>
       </c>
     </row>
@@ -36026,6 +37975,61 @@
           <t xml:space="preserve">ARABIC_TAH</t>
         </is>
       </c>
+      <c r="EP25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="EQ25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0901</t>
+        </is>
+      </c>
+      <c r="ER25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="ET25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="EU25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0901</t>
+        </is>
+      </c>
+      <c r="EV25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="EX25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="EY25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0901</t>
+        </is>
+      </c>
+      <c r="EZ25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0902</t>
+        </is>
+      </c>
+      <c r="FB25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_CHE</t>
+        </is>
+      </c>
+      <c r="FC25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_CHE</t>
+        </is>
+      </c>
     </row>
     <row r="26" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="93" t="s">
@@ -36255,6 +38259,61 @@
           <t xml:space="preserve">ARABIC_GHAIN</t>
         </is>
       </c>
+      <c r="EP26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="EQ26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092D</t>
+        </is>
+      </c>
+      <c r="ER26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="ET26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="EU26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092D</t>
+        </is>
+      </c>
+      <c r="EV26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="EX26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="EY26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092D</t>
+        </is>
+      </c>
+      <c r="EZ26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092C</t>
+        </is>
+      </c>
+      <c r="FB26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_EN</t>
+        </is>
+      </c>
+      <c r="FC26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_EN</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -36498,6 +38557,61 @@
           <t xml:space="preserve">ARABIC_ZAH</t>
         </is>
       </c>
+      <c r="EP27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="EQ27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090E</t>
+        </is>
+      </c>
+      <c r="ER27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="ET27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="EU27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090E</t>
+        </is>
+      </c>
+      <c r="EV27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="EX27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="EY27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090E</t>
+        </is>
+      </c>
+      <c r="EZ27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0946</t>
+        </is>
+      </c>
+      <c r="FB27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_YA</t>
+        </is>
+      </c>
+      <c r="FC27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_YA</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -36853,6 +38967,62 @@
         </is>
       </c>
       <c r="EJ28">
+        <v>1</v>
+      </c>
+      <c r="EP28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="EQ28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090D</t>
+        </is>
+      </c>
+      <c r="ER28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="ET28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="EU28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090D</t>
+        </is>
+      </c>
+      <c r="EV28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="EX28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="EY28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090D</t>
+        </is>
+      </c>
+      <c r="EZ28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0967</t>
+        </is>
+      </c>
+      <c r="FB28">
+        <v>1</v>
+      </c>
+      <c r="FC28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NUMERO_SIGN</t>
+        </is>
+      </c>
+      <c r="FD28">
         <v>1</v>
       </c>
     </row>
@@ -37233,6 +39403,62 @@
       <c r="EJ29">
         <v>2</v>
       </c>
+      <c r="EP29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="EQ29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0945</t>
+        </is>
+      </c>
+      <c r="ER29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="ET29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="EU29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0945</t>
+        </is>
+      </c>
+      <c r="EV29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="EX29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="EY29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0945</t>
+        </is>
+      </c>
+      <c r="EZ29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0968</t>
+        </is>
+      </c>
+      <c r="FB29">
+        <v>2</v>
+      </c>
+      <c r="FC29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="FD29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -37613,6 +39839,62 @@
       <c r="EJ30">
         <v>3</v>
       </c>
+      <c r="EP30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="EQ30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="ER30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="ET30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="EU30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="EV30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="EX30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="EY30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="EZ30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0969</t>
+        </is>
+      </c>
+      <c r="FB30">
+        <v>3</v>
+      </c>
+      <c r="FC30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QUOTE</t>
+        </is>
+      </c>
+      <c r="FD30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -37993,6 +40275,57 @@
       <c r="EJ31">
         <v>4</v>
       </c>
+      <c r="EP31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="EQ31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="ER31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="ET31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="EU31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="EV31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="EX31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="EY31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="EZ31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096A</t>
+        </is>
+      </c>
+      <c r="FB31">
+        <v>4</v>
+      </c>
+      <c r="FD31">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -38368,6 +40701,62 @@
       <c r="EJ32">
         <v>5</v>
       </c>
+      <c r="EP32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="EQ32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="ER32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="ET32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="EU32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="EV32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="EX32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="EY32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="EZ32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096B</t>
+        </is>
+      </c>
+      <c r="FB32">
+        <v>5</v>
+      </c>
+      <c r="FC32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">:</t>
+        </is>
+      </c>
+      <c r="FD32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -38731,6 +41120,62 @@
       <c r="EJ33">
         <v>6</v>
       </c>
+      <c r="EP33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="EQ33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="ER33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="ET33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="EU33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="EV33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="EX33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="EY33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="EZ33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096C</t>
+        </is>
+      </c>
+      <c r="FB33">
+        <v>6</v>
+      </c>
+      <c r="FC33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="FD33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -39107,6 +41552,62 @@
         </is>
       </c>
       <c r="EJ34">
+        <v>7</v>
+      </c>
+      <c r="EP34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="EQ34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="ER34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="ET34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="EU34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="EV34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="EX34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="EY34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&amp;</t>
+        </is>
+      </c>
+      <c r="EZ34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096D</t>
+        </is>
+      </c>
+      <c r="FB34">
+        <v>7</v>
+      </c>
+      <c r="FC34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_</t>
+        </is>
+      </c>
+      <c r="FD34">
         <v>7</v>
       </c>
     </row>
@@ -39487,6 +41988,62 @@
       <c r="EJ35">
         <v>8</v>
       </c>
+      <c r="EP35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="EQ35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="ER35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="ET35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="EU35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="EV35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="EX35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="EY35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="EZ35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096E</t>
+        </is>
+      </c>
+      <c r="FB35">
+        <v>8</v>
+      </c>
+      <c r="FC35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="FD35">
+        <v>8</v>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -39863,6 +42420,62 @@
       <c r="EJ36">
         <v>9</v>
       </c>
+      <c r="EP36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="EQ36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="ER36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="ET36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="EU36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="EV36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="EX36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="EY36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="EZ36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_096F</t>
+        </is>
+      </c>
+      <c r="FB36">
+        <v>9</v>
+      </c>
+      <c r="FC36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="FD36">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -40257,6 +42870,66 @@
         </is>
       </c>
       <c r="EJ37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="EP37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="EQ37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="ER37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="ET37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="EU37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="EV37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="EX37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="EY37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="EZ37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0966</t>
+        </is>
+      </c>
+      <c r="FB37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="FC37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="FD37" t="inlineStr">
         <is>
           <t xml:space="preserve">ZERO</t>
         </is>
@@ -41201,6 +43874,61 @@
           <t xml:space="preserve">'</t>
         </is>
       </c>
+      <c r="EP43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="EQ43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0903</t>
+        </is>
+      </c>
+      <c r="ER43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="ET43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="EU43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0903</t>
+        </is>
+      </c>
+      <c r="EV43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="EX43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="EY43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0903</t>
+        </is>
+      </c>
+      <c r="EZ43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="FB43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_IE</t>
+        </is>
+      </c>
+      <c r="FC43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_IE</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -41570,6 +44298,61 @@
           <t xml:space="preserve">+</t>
         </is>
       </c>
+      <c r="EP44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="EQ44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090B</t>
+        </is>
+      </c>
+      <c r="ER44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="ET44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="EU44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090B</t>
+        </is>
+      </c>
+      <c r="EV44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="EX44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="EY44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_090B</t>
+        </is>
+      </c>
+      <c r="EZ44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0943</t>
+        </is>
+      </c>
+      <c r="FB44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SHCHA</t>
+        </is>
+      </c>
+      <c r="FC44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SHCHA</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -41921,6 +44704,61 @@
           <t xml:space="preserve">ARABIC_JEEM</t>
         </is>
       </c>
+      <c r="EP45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="EQ45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0922</t>
+        </is>
+      </c>
+      <c r="ER45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="ET45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="EU45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0922</t>
+        </is>
+      </c>
+      <c r="EV45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="EX45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="EY45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0922</t>
+        </is>
+      </c>
+      <c r="EZ45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0921</t>
+        </is>
+      </c>
+      <c r="FB45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_KA</t>
+        </is>
+      </c>
+      <c r="FC45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_KA</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -42278,6 +45116,61 @@
           <t xml:space="preserve">ARABIC_TCHEH</t>
         </is>
       </c>
+      <c r="EP46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="EQ46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091E</t>
+        </is>
+      </c>
+      <c r="ER46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="ET46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="EU46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091E</t>
+        </is>
+      </c>
+      <c r="EV46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="EX46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="EY46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091E</t>
+        </is>
+      </c>
+      <c r="EZ46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_093C</t>
+        </is>
+      </c>
+      <c r="FB46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_HARD_SIGN</t>
+        </is>
+      </c>
+      <c r="FC46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_HARD_SIGN</t>
+        </is>
+      </c>
     </row>
     <row r="47" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="93" t="s">
@@ -42558,6 +45451,21 @@
       <c r="EB47" t="inlineStr">
         <is>
           <t xml:space="preserve">]</t>
+        </is>
+      </c>
+      <c r="FB47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="FC47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|</t>
+        </is>
+      </c>
+      <c r="FD47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
         </is>
       </c>
     </row>
@@ -43085,6 +45993,61 @@
           <t xml:space="preserve">ARABIC_KEHEH</t>
         </is>
       </c>
+      <c r="EP49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="EQ49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091B</t>
+        </is>
+      </c>
+      <c r="ER49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="ET49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="EU49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091B</t>
+        </is>
+      </c>
+      <c r="EV49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="EX49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="EY49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091B</t>
+        </is>
+      </c>
+      <c r="EZ49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091A</t>
+        </is>
+      </c>
+      <c r="FB49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_DE</t>
+        </is>
+      </c>
+      <c r="FC49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_DE</t>
+        </is>
+      </c>
     </row>
     <row r="50" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="93" t="s">
@@ -43424,6 +46387,61 @@
           <t xml:space="preserve">ARABIC_GAF</t>
         </is>
       </c>
+      <c r="EP50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="EQ50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0920</t>
+        </is>
+      </c>
+      <c r="ER50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="ET50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="EU50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0920</t>
+        </is>
+      </c>
+      <c r="EV50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="EX50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="EY50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0920</t>
+        </is>
+      </c>
+      <c r="EZ50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_091F</t>
+        </is>
+      </c>
+      <c r="FB50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_PE</t>
+        </is>
+      </c>
+      <c r="FC50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_PE</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -43719,6 +46737,66 @@
       <c r="DL51" t="inlineStr">
         <is>
           <t xml:space="preserve">;</t>
+        </is>
+      </c>
+      <c r="EP51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="EQ51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0912</t>
+        </is>
+      </c>
+      <c r="ER51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="ET51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="EU51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0912</t>
+        </is>
+      </c>
+      <c r="EV51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="EX51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="EY51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0912</t>
+        </is>
+      </c>
+      <c r="EZ51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_094A</t>
+        </is>
+      </c>
+      <c r="FB51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="FC51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="FD51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
         </is>
       </c>
     </row>
@@ -43986,6 +47064,61 @@
           <t xml:space="preserve">ARABIC_WAW</t>
         </is>
       </c>
+      <c r="EP52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="EQ52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0937</t>
+        </is>
+      </c>
+      <c r="ER52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="ET52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="EU52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0937</t>
+        </is>
+      </c>
+      <c r="EV52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="EX52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="EY52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0937</t>
+        </is>
+      </c>
+      <c r="EZ52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">,</t>
+        </is>
+      </c>
+      <c r="FB52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_SOFT_SIGN</t>
+        </is>
+      </c>
+      <c r="FC52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SOFT_SIGN</t>
+        </is>
+      </c>
     </row>
     <row r="53" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="93" t="s">
@@ -44245,6 +47378,61 @@
       <c r="DE53" s="115" t="s">
         <v>1223</v>
       </c>
+      <c r="EP53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="EQ53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0964</t>
+        </is>
+      </c>
+      <c r="ER53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="ET53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="EU53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0964</t>
+        </is>
+      </c>
+      <c r="EV53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="EX53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="EY53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_0964</t>
+        </is>
+      </c>
+      <c r="EZ53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.</t>
+        </is>
+      </c>
+      <c r="FB53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_VE</t>
+        </is>
+      </c>
+      <c r="FC53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_VE</t>
+        </is>
+      </c>
     </row>
     <row r="54" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="93" t="s">
@@ -44509,6 +47697,61 @@
       </c>
       <c r="DE54" s="115" t="s">
         <v>1272</v>
+      </c>
+      <c r="EP54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="EQ54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_095F</t>
+        </is>
+      </c>
+      <c r="ER54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="ET54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="EU54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_095F</t>
+        </is>
+      </c>
+      <c r="EV54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="EX54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="EY54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_095F</t>
+        </is>
+      </c>
+      <c r="EZ54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEVANAGARI_092F</t>
+        </is>
+      </c>
+      <c r="FB54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_SM_YU</t>
+        </is>
+      </c>
+      <c r="FC54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CYRILLIC_YU</t>
+        </is>
       </c>
     </row>
     <row r="55" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -44820,6 +48063,21 @@
           <t xml:space="preserve">&lt;</t>
         </is>
       </c>
+      <c r="FB55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="FC55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="FD55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
     </row>
     <row r="56" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="141" t="s">
@@ -45103,6 +48361,32 @@
       <c r="EO56">
         <v>52</v>
       </c>
+      <c r="EQ56">
+        <v>40</v>
+      </c>
+      <c r="ES56">
+        <v>52</v>
+      </c>
+      <c r="EU56">
+        <v>40</v>
+      </c>
+      <c r="EW56">
+        <v>52</v>
+      </c>
+      <c r="EY56">
+        <v>40</v>
+      </c>
+      <c r="FA56">
+        <v>52</v>
+      </c>
+      <c r="FC56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="FE56">
+        <v>50</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -45386,6 +48670,32 @@
       <c r="EO57">
         <v>13</v>
       </c>
+      <c r="EQ57">
+        <v>0</v>
+      </c>
+      <c r="ES57">
+        <v>13</v>
+      </c>
+      <c r="EU57">
+        <v>0</v>
+      </c>
+      <c r="EW57">
+        <v>13</v>
+      </c>
+      <c r="EY57">
+        <v>0</v>
+      </c>
+      <c r="FA57">
+        <v>13</v>
+      </c>
+      <c r="FC57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
+      <c r="FE57">
+        <v>13</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -45653,6 +48963,30 @@
       <c r="EO58">
         <v>52</v>
       </c>
+      <c r="EQ58">
+        <v>28</v>
+      </c>
+      <c r="ES58">
+        <v>52</v>
+      </c>
+      <c r="EU58">
+        <v>28</v>
+      </c>
+      <c r="EW58">
+        <v>52</v>
+      </c>
+      <c r="EY58">
+        <v>28</v>
+      </c>
+      <c r="FA58">
+        <v>52</v>
+      </c>
+      <c r="FC58">
+        <v>30</v>
+      </c>
+      <c r="FE58">
+        <v>50</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -45920,6 +49254,30 @@
       <c r="EO59">
         <v>13</v>
       </c>
+      <c r="EQ59">
+        <v>0</v>
+      </c>
+      <c r="ES59">
+        <v>13</v>
+      </c>
+      <c r="EU59">
+        <v>0</v>
+      </c>
+      <c r="EW59">
+        <v>13</v>
+      </c>
+      <c r="EY59">
+        <v>0</v>
+      </c>
+      <c r="FA59">
+        <v>13</v>
+      </c>
+      <c r="FC59">
+        <v>0</v>
+      </c>
+      <c r="FE59">
+        <v>13</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -46187,6 +49545,30 @@
       <c r="EO60">
         <v>52</v>
       </c>
+      <c r="EQ60">
+        <v>40</v>
+      </c>
+      <c r="ES60">
+        <v>52</v>
+      </c>
+      <c r="EU60">
+        <v>40</v>
+      </c>
+      <c r="EW60">
+        <v>52</v>
+      </c>
+      <c r="EY60">
+        <v>40</v>
+      </c>
+      <c r="FA60">
+        <v>52</v>
+      </c>
+      <c r="FC60">
+        <v>30</v>
+      </c>
+      <c r="FE60">
+        <v>50</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -46452,6 +49834,30 @@
         <v>0</v>
       </c>
       <c r="EO61">
+        <v>13</v>
+      </c>
+      <c r="EQ61">
+        <v>0</v>
+      </c>
+      <c r="ES61">
+        <v>13</v>
+      </c>
+      <c r="EU61">
+        <v>0</v>
+      </c>
+      <c r="EW61">
+        <v>13</v>
+      </c>
+      <c r="EY61">
+        <v>0</v>
+      </c>
+      <c r="FA61">
+        <v>13</v>
+      </c>
+      <c r="FC61">
+        <v>0</v>
+      </c>
+      <c r="FE61">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: add Urdu (ur-PK) - language set complete (41 languages)
Final gap-2 language. Added 4 more Perso-Arabic glyphs (heh-goal-hamza,
teh-marbuta-goal, yeh-barree-hamza, arabic full-stop) and extended the _PerArab_
font range; regenerated arabic_fonts.h with the pinned fontconvert. Urdu layout
is the official NLA standard taken from xkb pk/urd-nla. Re-cogged all language
files so ur-PK is selectable on the _LL layer; flag added. Builds clean.

Completes the requested set: 27 original + 14 new (hr sk lt lv et pt-BR, sr-RS
mk, fa, hi mr ne, mn, ur). Non-Latin/complex layouts built from the published
standards (xkb) and flagged for hardware review.

https://claude.ai/code/session_01U69j8s2Phaxg2troJeBT1K
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -31098,29 +31098,61 @@
       <c r="E1069" s="7"/>
     </row>
     <row r="1070" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1070" s="7"/>
-      <c r="B1070" s="7"/>
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_GOAL_HAMZA</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6C2</t>
+        </is>
+      </c>
       <c r="C1070" s="7"/>
       <c r="D1070" s="7"/>
       <c r="E1070" s="7"/>
     </row>
     <row r="1071" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1071" s="7"/>
-      <c r="B1071" s="7"/>
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH_MARBUTA_GOAL</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6C3</t>
+        </is>
+      </c>
       <c r="C1071" s="7"/>
       <c r="D1071" s="7"/>
       <c r="E1071" s="7"/>
     </row>
     <row r="1072" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1072" s="7"/>
-      <c r="B1072" s="7"/>
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_BARREE_HAMZA</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6D3</t>
+        </is>
+      </c>
       <c r="C1072" s="7"/>
       <c r="D1072" s="7"/>
       <c r="E1072" s="7"/>
     </row>
     <row r="1073" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1073" s="7"/>
-      <c r="B1073" s="7"/>
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FULL_STOP</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6D4</t>
+        </is>
+      </c>
       <c r="C1073" s="7"/>
       <c r="D1073" s="7"/>
       <c r="E1073" s="7"/>
@@ -31500,7 +31532,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:FE79"/>
+  <dimension ref="A1:FI79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -31820,6 +31852,11 @@
           <t xml:space="preserve">mn-MN</t>
         </is>
       </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ur-PK</t>
+        </is>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -32075,6 +32112,21 @@
       <c r="FC2" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_SHORT_I</t>
+        </is>
+      </c>
+      <c r="FF2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_MEEM</t>
+        </is>
+      </c>
+      <c r="FG2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEH</t>
+        </is>
+      </c>
+      <c r="FH2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_MEEM</t>
         </is>
       </c>
     </row>
@@ -32330,6 +32382,21 @@
           <t xml:space="preserve">CYRILLIC_EM</t>
         </is>
       </c>
+      <c r="FF3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SHEEN</t>
+        </is>
+      </c>
+      <c r="FG3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_WAW_HAMZA_A</t>
+        </is>
+      </c>
+      <c r="FH3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SHEEN</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -32594,6 +32661,21 @@
           <t xml:space="preserve">CYRILLIC_IO</t>
         </is>
       </c>
+      <c r="FF4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_BARREE</t>
+        </is>
+      </c>
+      <c r="FG4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_BARREE_HAMZA</t>
+        </is>
+      </c>
+      <c r="FH4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_BARREE</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -32848,6 +32930,21 @@
           <t xml:space="preserve">CYRILLIC_BE</t>
         </is>
       </c>
+      <c r="FF5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_REH</t>
+        </is>
+      </c>
+      <c r="FG5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_RREH</t>
+        </is>
+      </c>
+      <c r="FH5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_REH</t>
+        </is>
+      </c>
     </row>
     <row r="6" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="93" t="s">
@@ -33158,6 +33255,21 @@
       <c r="FC6" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_U</t>
+        </is>
+      </c>
+      <c r="FF6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_DOACHASHMEE</t>
+        </is>
+      </c>
+      <c r="FG6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THAL</t>
+        </is>
+      </c>
+      <c r="FH6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_DOACHASHMEE</t>
         </is>
       </c>
     </row>
@@ -33413,6 +33525,21 @@
           <t xml:space="preserve">CYRILLIC_BARRED_O</t>
         </is>
       </c>
+      <c r="FF7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON</t>
+        </is>
+      </c>
+      <c r="FG7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON_GHUNNA</t>
+        </is>
+      </c>
+      <c r="FH7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_NOON</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -33669,6 +33796,21 @@
           <t xml:space="preserve">CYRILLIC_A</t>
         </is>
       </c>
+      <c r="FF8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_LAM</t>
+        </is>
+      </c>
+      <c r="FG8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_GOAL_HAMZA</t>
+        </is>
+      </c>
+      <c r="FH8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_LAM</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -33915,6 +34057,21 @@
           <t xml:space="preserve">CYRILLIC_HA</t>
         </is>
       </c>
+      <c r="FF9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_GOAL</t>
+        </is>
+      </c>
+      <c r="FG9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HAMZA</t>
+        </is>
+      </c>
+      <c r="FH9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HEH_GOAL</t>
+        </is>
+      </c>
     </row>
     <row r="10" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="93" t="s">
@@ -34174,6 +34331,21 @@
       <c r="FC10" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_SHA</t>
+        </is>
+      </c>
+      <c r="FF10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_BEH</t>
+        </is>
+      </c>
+      <c r="FG10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TATWEEL</t>
+        </is>
+      </c>
+      <c r="FH10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_BEH</t>
         </is>
       </c>
     </row>
@@ -34426,6 +34598,21 @@
           <t xml:space="preserve">CYRILLIC_ER</t>
         </is>
       </c>
+      <c r="FF11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ALEF</t>
+        </is>
+      </c>
+      <c r="FG11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ALEF_MADDA_A</t>
+        </is>
+      </c>
+      <c r="FH11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ALEF</t>
+        </is>
+      </c>
     </row>
     <row r="12" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
@@ -34679,6 +34866,21 @@
           <t xml:space="preserve">CYRILLIC_O</t>
         </is>
       </c>
+      <c r="FF12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KEHEH</t>
+        </is>
+      </c>
+      <c r="FG12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GAF</t>
+        </is>
+      </c>
+      <c r="FH12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KEHEH</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -34934,6 +35136,21 @@
           <t xml:space="preserve">CYRILLIC_EL</t>
         </is>
       </c>
+      <c r="FF13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FARSI_YEH</t>
+        </is>
+      </c>
+      <c r="FG13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH</t>
+        </is>
+      </c>
+      <c r="FH13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FARSI_YEH</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -35198,6 +35415,16 @@
       <c r="FC14" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_TE</t>
+        </is>
+      </c>
+      <c r="FF14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_AIN</t>
+        </is>
+      </c>
+      <c r="FH14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_AIN</t>
         </is>
       </c>
     </row>
@@ -35460,6 +35687,21 @@
           <t xml:space="preserve">CYRILLIC_I</t>
         </is>
       </c>
+      <c r="FF15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GHAIN</t>
+        </is>
+      </c>
+      <c r="FG15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_YEH_HAMZA_A</t>
+        </is>
+      </c>
+      <c r="FH15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_GHAIN</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -35710,6 +35952,21 @@
           <t xml:space="preserve">CYRILLIC_STRAIGHT_U</t>
         </is>
       </c>
+      <c r="FF16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEEM</t>
+        </is>
+      </c>
+      <c r="FG16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TCHEH</t>
+        </is>
+      </c>
+      <c r="FH16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_JEEM</t>
+        </is>
+      </c>
     </row>
     <row r="17" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
@@ -35960,6 +36217,21 @@
           <t xml:space="preserve">CYRILLIC_ZE</t>
         </is>
       </c>
+      <c r="FF17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HAH</t>
+        </is>
+      </c>
+      <c r="FG17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_KHAH</t>
+        </is>
+      </c>
+      <c r="FH17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_HAH</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="93" t="s">
@@ -36237,6 +36509,21 @@
       <c r="FC18" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_EF</t>
+        </is>
+      </c>
+      <c r="FF18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TAH</t>
+        </is>
+      </c>
+      <c r="FG18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAH</t>
+        </is>
+      </c>
+      <c r="FH18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TAH</t>
         </is>
       </c>
     </row>
@@ -36493,6 +36780,21 @@
           <t xml:space="preserve">CYRILLIC_ZHE</t>
         </is>
       </c>
+      <c r="FF19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAL</t>
+        </is>
+      </c>
+      <c r="FG19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DDAL</t>
+        </is>
+      </c>
+      <c r="FH19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAL</t>
+        </is>
+      </c>
     </row>
     <row r="20" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="93" t="s">
@@ -36753,6 +37055,21 @@
       <c r="FC20" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_YERU</t>
+        </is>
+      </c>
+      <c r="FF20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_WAW</t>
+        </is>
+      </c>
+      <c r="FG20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_ZAIN</t>
+        </is>
+      </c>
+      <c r="FH20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_WAW</t>
         </is>
       </c>
     </row>
@@ -36999,6 +37316,21 @@
           <t xml:space="preserve">CYRILLIC_E</t>
         </is>
       </c>
+      <c r="FF21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TTEH</t>
+        </is>
+      </c>
+      <c r="FG21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_THEH</t>
+        </is>
+      </c>
+      <c r="FH21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TTEH</t>
+        </is>
+      </c>
     </row>
     <row r="22" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="93" t="s">
@@ -37258,6 +37590,21 @@
           <t xml:space="preserve">CYRILLIC_GHE</t>
         </is>
       </c>
+      <c r="FF22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH</t>
+        </is>
+      </c>
+      <c r="FG22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH_MARBUTA_GOAL</t>
+        </is>
+      </c>
+      <c r="FH22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_TEH</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -37513,6 +37860,16 @@
           <t xml:space="preserve">CYRILLIC_ES</t>
         </is>
       </c>
+      <c r="FF23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEEN</t>
+        </is>
+      </c>
+      <c r="FH23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEEN</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -37778,6 +38135,21 @@
       <c r="FC24" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_TSE</t>
+        </is>
+      </c>
+      <c r="FF24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SAD</t>
+        </is>
+      </c>
+      <c r="FG24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_DAD</t>
+        </is>
+      </c>
+      <c r="FH24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SAD</t>
         </is>
       </c>
     </row>
@@ -38030,6 +38402,16 @@
           <t xml:space="preserve">CYRILLIC_CHE</t>
         </is>
       </c>
+      <c r="FF25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FEH</t>
+        </is>
+      </c>
+      <c r="FH25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FEH</t>
+        </is>
+      </c>
     </row>
     <row r="26" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="93" t="s">
@@ -38314,6 +38696,21 @@
           <t xml:space="preserve">CYRILLIC_EN</t>
         </is>
       </c>
+      <c r="FF26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_PEH</t>
+        </is>
+      </c>
+      <c r="FG26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SHADDA</t>
+        </is>
+      </c>
+      <c r="FH26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_PEH</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -38612,6 +39009,16 @@
           <t xml:space="preserve">CYRILLIC_YA</t>
         </is>
       </c>
+      <c r="FF27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_QAF</t>
+        </is>
+      </c>
+      <c r="FH27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_QAF</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -39023,6 +39430,17 @@
         </is>
       </c>
       <c r="FD28">
+        <v>1</v>
+      </c>
+      <c r="FF28">
+        <v>1</v>
+      </c>
+      <c r="FG28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="FH28">
         <v>1</v>
       </c>
     </row>
@@ -39459,6 +39877,17 @@
       <c r="FD29">
         <v>2</v>
       </c>
+      <c r="FF29">
+        <v>2</v>
+      </c>
+      <c r="FG29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@</t>
+        </is>
+      </c>
+      <c r="FH29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -39895,6 +40324,17 @@
       <c r="FD30">
         <v>3</v>
       </c>
+      <c r="FF30">
+        <v>3</v>
+      </c>
+      <c r="FG30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="FH30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -40326,6 +40766,17 @@
       <c r="FD31">
         <v>4</v>
       </c>
+      <c r="FF31">
+        <v>4</v>
+      </c>
+      <c r="FG31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="FH31">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -40757,6 +41208,12 @@
       <c r="FD32">
         <v>5</v>
       </c>
+      <c r="FF32">
+        <v>5</v>
+      </c>
+      <c r="FH32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -41176,6 +41633,17 @@
       <c r="FD33">
         <v>6</v>
       </c>
+      <c r="FF33">
+        <v>6</v>
+      </c>
+      <c r="FG33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">^</t>
+        </is>
+      </c>
+      <c r="FH33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -41608,6 +42076,12 @@
         </is>
       </c>
       <c r="FD34">
+        <v>7</v>
+      </c>
+      <c r="FF34">
+        <v>7</v>
+      </c>
+      <c r="FH34">
         <v>7</v>
       </c>
     </row>
@@ -42044,6 +42518,12 @@
       <c r="FD35">
         <v>8</v>
       </c>
+      <c r="FF35">
+        <v>8</v>
+      </c>
+      <c r="FH35">
+        <v>8</v>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -42476,6 +42956,17 @@
       <c r="FD36">
         <v>9</v>
       </c>
+      <c r="FF36">
+        <v>9</v>
+      </c>
+      <c r="FG36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="FH36">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -42930,6 +43421,21 @@
         </is>
       </c>
       <c r="FD37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="FF37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
+        </is>
+      </c>
+      <c r="FG37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="FH37" t="inlineStr">
         <is>
           <t xml:space="preserve">ZERO</t>
         </is>
@@ -43929,6 +44435,21 @@
           <t xml:space="preserve">CYRILLIC_IE</t>
         </is>
       </c>
+      <c r="FF43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="FG43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">_</t>
+        </is>
+      </c>
+      <c r="FH43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -44353,6 +44874,21 @@
           <t xml:space="preserve">CYRILLIC_SHCHA</t>
         </is>
       </c>
+      <c r="FF44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="FG44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="FH44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -44759,6 +45295,21 @@
           <t xml:space="preserve">CYRILLIC_KA</t>
         </is>
       </c>
+      <c r="FF45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
+      <c r="FG45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">}</t>
+        </is>
+      </c>
+      <c r="FH45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -45171,6 +45722,21 @@
           <t xml:space="preserve">CYRILLIC_HARD_SIGN</t>
         </is>
       </c>
+      <c r="FF46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
+      <c r="FG46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{</t>
+        </is>
+      </c>
+      <c r="FH46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
     </row>
     <row r="47" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="93" t="s">
@@ -45466,6 +46032,21 @@
       <c r="FD47" t="inlineStr">
         <is>
           <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="FF47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BACKSLASH</t>
+        </is>
+      </c>
+      <c r="FG47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">|</t>
+        </is>
+      </c>
+      <c r="FH47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BACKSLASH</t>
         </is>
       </c>
     </row>
@@ -46048,6 +46629,21 @@
           <t xml:space="preserve">CYRILLIC_DE</t>
         </is>
       </c>
+      <c r="FF49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEMICOLON</t>
+        </is>
+      </c>
+      <c r="FG49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">:</t>
+        </is>
+      </c>
+      <c r="FH49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_SEMICOLON</t>
+        </is>
+      </c>
     </row>
     <row r="50" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="93" t="s">
@@ -46442,6 +47038,21 @@
           <t xml:space="preserve">CYRILLIC_PE</t>
         </is>
       </c>
+      <c r="FF50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="FG50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QUOTE</t>
+        </is>
+      </c>
+      <c r="FH50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -46797,6 +47408,21 @@
       <c r="FD51" t="inlineStr">
         <is>
           <t xml:space="preserve">=</t>
+        </is>
+      </c>
+      <c r="FF51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
+        </is>
+      </c>
+      <c r="FG51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~</t>
+        </is>
+      </c>
+      <c r="FH51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`</t>
         </is>
       </c>
     </row>
@@ -47119,6 +47745,21 @@
           <t xml:space="preserve">CYRILLIC_SOFT_SIGN</t>
         </is>
       </c>
+      <c r="FF52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_COMMA</t>
+        </is>
+      </c>
+      <c r="FG52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;</t>
+        </is>
+      </c>
+      <c r="FH52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_COMMA</t>
+        </is>
+      </c>
     </row>
     <row r="53" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="93" t="s">
@@ -47433,6 +48074,21 @@
           <t xml:space="preserve">CYRILLIC_VE</t>
         </is>
       </c>
+      <c r="FF53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FULL_STOP</t>
+        </is>
+      </c>
+      <c r="FG53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;</t>
+        </is>
+      </c>
+      <c r="FH53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_FULL_STOP</t>
+        </is>
+      </c>
     </row>
     <row r="54" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="93" t="s">
@@ -47751,6 +48407,21 @@
       <c r="FC54" t="inlineStr">
         <is>
           <t xml:space="preserve">CYRILLIC_YU</t>
+        </is>
+      </c>
+      <c r="FF54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="FG54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARABIC_QMARK</t>
+        </is>
+      </c>
+      <c r="FH54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
         </is>
       </c>
     </row>
@@ -48387,6 +49058,12 @@
       <c r="FE56">
         <v>50</v>
       </c>
+      <c r="FG56">
+        <v>42</v>
+      </c>
+      <c r="FI56">
+        <v>52</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -48696,6 +49373,12 @@
       <c r="FE57">
         <v>13</v>
       </c>
+      <c r="FG57">
+        <v>0</v>
+      </c>
+      <c r="FI57">
+        <v>13</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -48987,6 +49670,12 @@
       <c r="FE58">
         <v>50</v>
       </c>
+      <c r="FG58">
+        <v>27</v>
+      </c>
+      <c r="FI58">
+        <v>52</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -49278,6 +49967,12 @@
       <c r="FE59">
         <v>13</v>
       </c>
+      <c r="FG59">
+        <v>0</v>
+      </c>
+      <c r="FI59">
+        <v>13</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -49569,6 +50264,12 @@
       <c r="FE60">
         <v>50</v>
       </c>
+      <c r="FG60">
+        <v>42</v>
+      </c>
+      <c r="FI60">
+        <v>52</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -49858,6 +50559,12 @@
         <v>0</v>
       </c>
       <c r="FE61">
+        <v>13</v>
+      </c>
+      <c r="FG61">
+        <v>0</v>
+      </c>
+      <c r="FI61">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: round-2 language-layer feedback (ka-GE size, ta-IN, Enter key)
- ka-GE: reduced Georgian font 18 -> 17 pt (kept the +3 px down-nudge).
- ta-IN: hid the letter shift-preview ({letter.voffset} SHIFT = HIDE) so keys
  like Q render only the base Tamil glyph (the InScript shift glyph was too big
  to fit alongside), and moved all glyph types down 3 px (letter/num/sym voffset
  SMALL = 3) to stop the top clipping.
- _LL layer: the left half's bottom-row outer slot is KC_ENTER on the base
  layer, so it is now left blank (KC_NO) instead of holding a language. Bottom
  rows redistributed (left row5 = 5 langs + Enter hole, right row5 = the rest);
  all 57 layouts still placed.

Only georgian_fonts.h regenerates (+ gfx_used_fonts.h name). Builds clean.

Note: the Vietnamese vn(basic) / TCVN layout has no digits on the number row
(it is all Vietnamese vowels + tone marks), so there is nothing to display for
digits there - they come from the keyboard's Num layer or an OS group switch.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -61401,8 +61401,13 @@
       <c r="GO57">
         <v>13</v>
       </c>
-      <c r="GQ57">
-        <v>0</v>
+      <c r="GP57">
+        <v>3</v>
+      </c>
+      <c r="GQ57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
       </c>
       <c r="GS57">
         <v>13</v>
@@ -62190,6 +62195,9 @@
       <c r="GO59">
         <v>13</v>
       </c>
+      <c r="GP59">
+        <v>3</v>
+      </c>
       <c r="GQ59">
         <v>0</v>
       </c>
@@ -62963,6 +62971,9 @@
       </c>
       <c r="GO61">
         <v>13</v>
+      </c>
+      <c r="GP61">
+        <v>3</v>
       </c>
       <c r="GQ61">
         <v>0</v>

</xml_diff>

<commit_message>
polykybd: vi-VN show digit hints on the number row (AltGr slot)
The Vietnamese TCVN layout puts Vietnamese vowels / tone marks on the number
row, so the digits 1-0 aren't otherwise visible. Add the digit as the AltGr
preview hint on KC_1..KC_0 of the vi-VN column (num.* AltGr offsets already
position it). It's a visual hint only - the digit is actually typed via the
keyboard's Num layer / an OS group switch, not AltGr on this layout.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -47718,6 +47718,9 @@
           <t xml:space="preserve">LATIN_0102</t>
         </is>
       </c>
+      <c r="HU28">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="93" t="s">
@@ -48341,6 +48344,9 @@
           <t xml:space="preserve">LATIN_00C2</t>
         </is>
       </c>
+      <c r="HU29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -48991,6 +48997,9 @@
           <t xml:space="preserve">LATIN_00CA</t>
         </is>
       </c>
+      <c r="HU30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -49631,6 +49640,9 @@
           <t xml:space="preserve">LATIN_00D4</t>
         </is>
       </c>
+      <c r="HU31">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -50217,6 +50229,9 @@
           <t xml:space="preserve">VIET_DC_0300</t>
         </is>
       </c>
+      <c r="HU32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -50844,6 +50859,9 @@
           <t xml:space="preserve">VIET_DC_0309</t>
         </is>
       </c>
+      <c r="HU33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -51459,6 +51477,9 @@
         <is>
           <t xml:space="preserve">VIET_DC_0303</t>
         </is>
+      </c>
+      <c r="HU34">
+        <v>7</v>
       </c>
     </row>
     <row r="35" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -52065,6 +52086,9 @@
           <t xml:space="preserve">VIET_DC_0301</t>
         </is>
       </c>
+      <c r="HU35">
+        <v>8</v>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -52668,6 +52692,9 @@
           <t xml:space="preserve">VIET_DC_0323</t>
         </is>
       </c>
+      <c r="HU36">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -53299,6 +53326,11 @@
       <c r="HS37" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_0110</t>
+        </is>
+      </c>
+      <c r="HU37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: round-3 feedback (right Enter, ta-IN previews, th-TH digits, hy-AM)
- _LL: also blank the right-half bottom-row inner slot - it is KC_ENTER on the
  2nd default layer (_L1), the mirror of the left Enter we already skip. Bottom
  rows redistributed; all 57 layouts still placed.
- ta-IN: restored the letter shift-preview ({letter.voffset} SHIFT back to 0;
  kept the +3 px down-nudge). Most Tamil keys show both glyphs again; the
  firmware's existing clear/clamp/stagger handles the few wide composites
  per-key ("if space allows"). Hiding all of them was too aggressive.
- th-TH: added Arabic digit hints 1-0 on the number row AltGr slot, same as
  vi-VN (Kedmanee has no Arabic digits on the base/shift layers).
- hy-AM: like ka-GE, reduced the Armenian font 18 -> 17 pt and moved all glyphs
  down 3 px (letter/num/sym voffset SMALL) to stop top clipping.

Only armenian_fonts.h regenerates. Verified each via tools/oled_preview.py;
split72:default builds clean.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -47658,6 +47658,9 @@
           <t xml:space="preserve">THAI_0E45</t>
         </is>
       </c>
+      <c r="GG28">
+        <v>1</v>
+      </c>
       <c r="GH28" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09E7</t>
@@ -48262,6 +48265,9 @@
           <t xml:space="preserve">/</t>
         </is>
       </c>
+      <c r="GG29">
+        <v>2</v>
+      </c>
       <c r="GH29" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09E8</t>
@@ -48906,6 +48912,9 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
+      <c r="GG30">
+        <v>3</v>
+      </c>
       <c r="GH30" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09E9</t>
@@ -49549,6 +49558,9 @@
           <t xml:space="preserve">THAI_0E20</t>
         </is>
       </c>
+      <c r="GG31">
+        <v>4</v>
+      </c>
       <c r="GH31" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09EA</t>
@@ -50144,6 +50156,9 @@
           <t xml:space="preserve">THAI_0E16</t>
         </is>
       </c>
+      <c r="GG32">
+        <v>5</v>
+      </c>
       <c r="GH32" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09EB</t>
@@ -50763,6 +50778,9 @@
           <t xml:space="preserve">THAI_DC_0E38</t>
         </is>
       </c>
+      <c r="GG33">
+        <v>6</v>
+      </c>
       <c r="GH33" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09EC</t>
@@ -51381,6 +51399,9 @@
         <is>
           <t xml:space="preserve">THAI_DC_0E36</t>
         </is>
+      </c>
+      <c r="GG34">
+        <v>7</v>
       </c>
       <c r="GH34" t="inlineStr">
         <is>
@@ -52001,6 +52022,9 @@
           <t xml:space="preserve">THAI_0E04</t>
         </is>
       </c>
+      <c r="GG35">
+        <v>8</v>
+      </c>
       <c r="GH35" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09EE</t>
@@ -52607,6 +52631,9 @@
           <t xml:space="preserve">THAI_0E15</t>
         </is>
       </c>
+      <c r="GG36">
+        <v>9</v>
+      </c>
       <c r="GH36" t="inlineStr">
         <is>
           <t xml:space="preserve">BENGALI_09EF</t>
@@ -53251,6 +53278,11 @@
       <c r="GF37" t="inlineStr">
         <is>
           <t xml:space="preserve">THAI_0E08</t>
+        </is>
+      </c>
+      <c r="GG37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
         </is>
       </c>
       <c r="GH37" t="inlineStr">
@@ -61436,10 +61468,8 @@
       <c r="GP57">
         <v>3</v>
       </c>
-      <c r="GQ57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HIDE</t>
-        </is>
+      <c r="GQ57">
+        <v>0</v>
       </c>
       <c r="GS57">
         <v>13</v>
@@ -61462,6 +61492,9 @@
       </c>
       <c r="HA57">
         <v>12</v>
+      </c>
+      <c r="HB57">
+        <v>3</v>
       </c>
       <c r="HC57" t="inlineStr">
         <is>
@@ -62248,6 +62281,9 @@
       <c r="HA59">
         <v>12</v>
       </c>
+      <c r="HB59">
+        <v>3</v>
+      </c>
       <c r="HC59">
         <v>0</v>
       </c>
@@ -63024,6 +63060,9 @@
       </c>
       <c r="HA61">
         <v>12</v>
+      </c>
+      <c r="HB61">
+        <v>3</v>
       </c>
       <c r="HC61">
         <v>0</v>

</xml_diff>

<commit_message>
polykybd: hy-AM - reduce Armenian font to 16 pt + add number-row digit hints
- Armenian font 17 -> 16 pt (the typewriter layout's tall caps were still a
  touch high at 17).
- Added Arabic digit hints 1-0 on the number-row AltGr slot, like vi-VN/th-TH:
  the Armenian typewriter layout puts letters on the number row, so the digits
  aren't otherwise shown.

Only armenian_fonts.h regenerates. Verified via tools/oled_preview.py; builds clean.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -47711,6 +47711,9 @@
           <t xml:space="preserve">ARMENIAN_0556</t>
         </is>
       </c>
+      <c r="HE28">
+        <v>1</v>
+      </c>
       <c r="HR28" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_0103</t>
@@ -48318,6 +48321,9 @@
           <t xml:space="preserve">ARMENIAN_0541</t>
         </is>
       </c>
+      <c r="HE29">
+        <v>2</v>
+      </c>
       <c r="HJ29">
         <v>2</v>
       </c>
@@ -48985,6 +48991,9 @@
           <t xml:space="preserve">ARMENIAN_058A</t>
         </is>
       </c>
+      <c r="HE30">
+        <v>3</v>
+      </c>
       <c r="HJ30">
         <v>3</v>
       </c>
@@ -49631,6 +49640,9 @@
           <t xml:space="preserve">COMMA</t>
         </is>
       </c>
+      <c r="HE31">
+        <v>4</v>
+      </c>
       <c r="HJ31">
         <v>4</v>
       </c>
@@ -50229,6 +50241,9 @@
           <t xml:space="preserve">ARMENIAN_0589</t>
         </is>
       </c>
+      <c r="HE32">
+        <v>5</v>
+      </c>
       <c r="HR32" t="inlineStr">
         <is>
           <t xml:space="preserve">VIET_DC_0300</t>
@@ -50851,6 +50866,9 @@
           <t xml:space="preserve">ARMENIAN_055E</t>
         </is>
       </c>
+      <c r="HE33">
+        <v>6</v>
+      </c>
       <c r="HJ33">
         <v>6</v>
       </c>
@@ -51472,6 +51490,9 @@
         <is>
           <t xml:space="preserve">ARMENIAN_2024</t>
         </is>
+      </c>
+      <c r="HE34">
+        <v>7</v>
       </c>
       <c r="HJ34">
         <v>7</v>
@@ -52095,6 +52116,9 @@
           <t xml:space="preserve">ARMENIAN_055B</t>
         </is>
       </c>
+      <c r="HE35">
+        <v>8</v>
+      </c>
       <c r="HR35" t="inlineStr">
         <is>
           <t xml:space="preserve">VIET_DC_0301</t>
@@ -52704,6 +52728,9 @@
           <t xml:space="preserve">)</t>
         </is>
       </c>
+      <c r="HE36">
+        <v>9</v>
+      </c>
       <c r="HR36" t="inlineStr">
         <is>
           <t xml:space="preserve">VIET_DC_0323</t>
@@ -53348,6 +53375,11 @@
       <c r="HC37" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0555</t>
+        </is>
+      </c>
+      <c r="HE37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
         </is>
       </c>
       <c r="HR37" t="inlineStr">

</xml_diff>

<commit_message>
polykybd: fix _LL country-sort layout + drop ta-IN overlap previews
- _LL layer (keymap.c cog): assign the country-sorted language list
  row-by-row ACROSS both halves instead of filling the whole left half
  first. Reading the keyboard left->right, top->bottom now follows the
  sorted sequence contiguously (row1 am..dk, row2 ee..in, ... row5
  sa..vn) instead of jumping from the left block to the right block.
- ta-IN: clear the SHIFT glyph for KC_A, KC_Q and KC_GRAVE so their
  wide dotted-circle vowel-sign composites no longer overlap with a
  shift preview. The base glyph is kept; only these three keys lose the
  second glyph (the rest of the layer keeps both).
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -37915,7 +37915,7 @@
       </c>
       <c r="GQ2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMIL_0B93</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="GR2" t="inlineStr">
@@ -43767,7 +43767,7 @@
       </c>
       <c r="GQ18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMIL_0B94</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="GR18" t="inlineStr">
@@ -58869,7 +58869,7 @@
       </c>
       <c r="GQ51" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMIL_0B92</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="GR51" t="inlineStr">

</xml_diff>

<commit_message>
polykybd: add zh-HK (Hong Kong, Cangjie) language
Adds LANG_ZHHK / KCL_ZHHK as the 58th language (enum index 57), the
rank-12 gap from the market analysis. No new fonts or named glyphs were
needed: the Cangjie radical legends (Kangxi-radical block U+2F00-2FD5
plus 中/廿/難) already ship, because the existing zh-CN column is itself a
Cangjie radical layout. zh-HK mirrors that column with its own HK flag
and the zh-HK locale.

- lang_lut.xlsx: append zh-HK key_lut column (copy of zh-CN's Cangjie
  mapping) + LCID 3076 in _patch_xlsx.py's informational map.
- Re-cogged lang_lut.{h,c}, keycode_helper.h, hid_com.c, keymap.c
  (enum, KCL, languages list, sorted _LL placement, to_static_text,
  post_process_record_user) - the _LL layer now holds all 58, still
  country-sorted (hk slots between el-GR and hr-HR).
- flag_fonts.h: regenerated, 58 flags (adds the HK regional-indicator pair).
- LANGUAGE_MARKET_ANALYSIS.md: record zh-HK shipped.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -37149,7 +37149,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:HU79"/>
+  <dimension ref="A1:HY79"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="21.56"/>
@@ -37581,6 +37581,14 @@
           <t xml:space="preserve">vi-VN</t>
         </is>
       </c>
+      <c r="HV1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">zh-HK</t>
+        </is>
+      </c>
+      <c r="HY1">
+        <v>3076</v>
+      </c>
     </row>
     <row r="2" s="92" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="64" t="s">
@@ -37951,6 +37959,21 @@
       <c r="HC2" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_054B</t>
+        </is>
+      </c>
+      <c r="HV2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_SUN</t>
+        </is>
+      </c>
+      <c r="HW2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a</t>
+        </is>
+      </c>
+      <c r="HX2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_SUN</t>
         </is>
       </c>
     </row>
@@ -38296,6 +38319,21 @@
           <t xml:space="preserve">ARMENIAN_0536</t>
         </is>
       </c>
+      <c r="HV3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOON</t>
+        </is>
+      </c>
+      <c r="HW3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b</t>
+        </is>
+      </c>
+      <c r="HX3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOON</t>
+        </is>
+      </c>
     </row>
     <row r="4" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="93" t="s">
@@ -38670,6 +38708,21 @@
           <t xml:space="preserve">ARMENIAN_0549</t>
         </is>
       </c>
+      <c r="HV4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_GOLD</t>
+        </is>
+      </c>
+      <c r="HW4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c</t>
+        </is>
+      </c>
+      <c r="HX4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_GOLD</t>
+        </is>
+      </c>
     </row>
     <row r="5" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="93" t="s">
@@ -39029,6 +39082,21 @@
           <t xml:space="preserve">ARMENIAN_0533</t>
         </is>
       </c>
+      <c r="HV5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_TREE</t>
+        </is>
+      </c>
+      <c r="HW5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d</t>
+        </is>
+      </c>
+      <c r="HX5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_TREE</t>
+        </is>
+      </c>
     </row>
     <row r="6" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="93" t="s">
@@ -39489,6 +39557,21 @@
       <c r="HC6" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0532</t>
+        </is>
+      </c>
+      <c r="HV6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_WATER</t>
+        </is>
+      </c>
+      <c r="HW6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e</t>
+        </is>
+      </c>
+      <c r="HX6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_WATER</t>
         </is>
       </c>
     </row>
@@ -39849,6 +39932,21 @@
           <t xml:space="preserve">ARMENIAN_0535</t>
         </is>
       </c>
+      <c r="HV7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_FIRE</t>
+        </is>
+      </c>
+      <c r="HW7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f</t>
+        </is>
+      </c>
+      <c r="HX7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_FIRE</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="93" t="s">
@@ -40210,6 +40308,21 @@
           <t xml:space="preserve">ARMENIAN_0531</t>
         </is>
       </c>
+      <c r="HV8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_EARTH</t>
+        </is>
+      </c>
+      <c r="HW8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g</t>
+        </is>
+      </c>
+      <c r="HX8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_EARTH</t>
+        </is>
+      </c>
     </row>
     <row r="9" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="93" t="s">
@@ -40556,6 +40669,21 @@
           <t xml:space="preserve">ARMENIAN_0546</t>
         </is>
       </c>
+      <c r="HV9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BAMBOO</t>
+        </is>
+      </c>
+      <c r="HW9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="HX9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BAMBOO</t>
+        </is>
+      </c>
     </row>
     <row r="10" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="93" t="s">
@@ -40915,6 +41043,21 @@
       <c r="HK10" t="inlineStr">
         <is>
           <t xml:space="preserve">I_WITH_DOT</t>
+        </is>
+      </c>
+      <c r="HV10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HALBERD</t>
+        </is>
+      </c>
+      <c r="HW10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i</t>
+        </is>
+      </c>
+      <c r="HX10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HALBERD</t>
         </is>
       </c>
     </row>
@@ -41272,6 +41415,21 @@
           <t xml:space="preserve">ARMENIAN_053B</t>
         </is>
       </c>
+      <c r="HV11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_TEN</t>
+        </is>
+      </c>
+      <c r="HW11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">j</t>
+        </is>
+      </c>
+      <c r="HX11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_TEN</t>
+        </is>
+      </c>
     </row>
     <row r="12" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
@@ -41625,6 +41783,21 @@
           <t xml:space="preserve">ARMENIAN_054F</t>
         </is>
       </c>
+      <c r="HV12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BIG</t>
+        </is>
+      </c>
+      <c r="HW12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k</t>
+        </is>
+      </c>
+      <c r="HX12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BIG</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="93" t="s">
@@ -41980,6 +42153,21 @@
           <t xml:space="preserve">ARMENIAN_0540</t>
         </is>
       </c>
+      <c r="HV13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_4E2D</t>
+        </is>
+      </c>
+      <c r="HW13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">l</t>
+        </is>
+      </c>
+      <c r="HX13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_4E2D</t>
+        </is>
+      </c>
     </row>
     <row r="14" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="93" t="s">
@@ -42359,6 +42547,21 @@
       <c r="HC14" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0554</t>
+        </is>
+      </c>
+      <c r="HV14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_ONE</t>
+        </is>
+      </c>
+      <c r="HW14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m</t>
+        </is>
+      </c>
+      <c r="HX14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_ONE</t>
         </is>
       </c>
     </row>
@@ -42721,6 +42924,21 @@
           <t xml:space="preserve">ARMENIAN_053C</t>
         </is>
       </c>
+      <c r="HV15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BOW</t>
+        </is>
+      </c>
+      <c r="HW15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n</t>
+        </is>
+      </c>
+      <c r="HX15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_BOW</t>
+        </is>
+      </c>
     </row>
     <row r="16" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="93" t="s">
@@ -43061,6 +43279,21 @@
           <t xml:space="preserve">ARMENIAN_0538</t>
         </is>
       </c>
+      <c r="HV16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MAN</t>
+        </is>
+      </c>
+      <c r="HW16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">o</t>
+        </is>
+      </c>
+      <c r="HX16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MAN</t>
+        </is>
+      </c>
     </row>
     <row r="17" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
@@ -43411,6 +43644,21 @@
           <t xml:space="preserve">ARMENIAN_0539</t>
         </is>
       </c>
+      <c r="HV17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HEART</t>
+        </is>
+      </c>
+      <c r="HW17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p</t>
+        </is>
+      </c>
+      <c r="HX17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HEART</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="93" t="s">
@@ -43803,6 +44051,21 @@
       <c r="HC18" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0543</t>
+        </is>
+      </c>
+      <c r="HV18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HAND</t>
+        </is>
+      </c>
+      <c r="HW18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">q</t>
+        </is>
+      </c>
+      <c r="HX18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_HAND</t>
         </is>
       </c>
     </row>
@@ -44169,6 +44432,21 @@
           <t xml:space="preserve">ARMENIAN_054D</t>
         </is>
       </c>
+      <c r="HV19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOUTH</t>
+        </is>
+      </c>
+      <c r="HW19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r</t>
+        </is>
+      </c>
+      <c r="HX19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="20" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="93" t="s">
@@ -44539,6 +44817,21 @@
       <c r="HC20" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_054E</t>
+        </is>
+      </c>
+      <c r="HV20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_CORPSE</t>
+        </is>
+      </c>
+      <c r="HW20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="HX20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_CORPSE</t>
         </is>
       </c>
     </row>
@@ -44895,6 +45188,21 @@
           <t xml:space="preserve">ARMENIAN_0544</t>
         </is>
       </c>
+      <c r="HV21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_5EFF</t>
+        </is>
+      </c>
+      <c r="HW21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t</t>
+        </is>
+      </c>
+      <c r="HX21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_5EFF</t>
+        </is>
+      </c>
     </row>
     <row r="22" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="93" t="s">
@@ -45259,6 +45567,21 @@
           <t xml:space="preserve">ARMENIAN_0552</t>
         </is>
       </c>
+      <c r="HV22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOUNTAIN</t>
+        </is>
+      </c>
+      <c r="HW22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">u</t>
+        </is>
+      </c>
+      <c r="HX22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_MOUNTAIN</t>
+        </is>
+      </c>
     </row>
     <row r="23" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="93" t="s">
@@ -45604,6 +45927,21 @@
           <t xml:space="preserve">ARMENIAN_0545</t>
         </is>
       </c>
+      <c r="HV23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_WOMAN</t>
+        </is>
+      </c>
+      <c r="HW23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v</t>
+        </is>
+      </c>
+      <c r="HX23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_WOMAN</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="93" t="s">
@@ -45999,6 +46337,21 @@
       <c r="HK24" t="inlineStr">
         <is>
           <t xml:space="preserve">UMLAUT_U</t>
+        </is>
+      </c>
+      <c r="HV24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_FIELD</t>
+        </is>
+      </c>
+      <c r="HW24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">w</t>
+        </is>
+      </c>
+      <c r="HX24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_FIELD</t>
         </is>
       </c>
     </row>
@@ -46346,6 +46699,21 @@
           <t xml:space="preserve">ARMENIAN_0534</t>
         </is>
       </c>
+      <c r="HV25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_96E3</t>
+        </is>
+      </c>
+      <c r="HW25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="HX25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_96E3</t>
+        </is>
+      </c>
     </row>
     <row r="26" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="93" t="s">
@@ -46730,6 +47098,21 @@
           <t xml:space="preserve">ARMENIAN_0548</t>
         </is>
       </c>
+      <c r="HV26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_DIVINATION</t>
+        </is>
+      </c>
+      <c r="HW26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y</t>
+        </is>
+      </c>
+      <c r="HX26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_DIVINATION</t>
+        </is>
+      </c>
     </row>
     <row r="27" s="116" customFormat="true" ht="15.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="93" t="s">
@@ -47138,6 +47521,21 @@
           <t xml:space="preserve">ARMENIAN_053A</t>
         </is>
       </c>
+      <c r="HV27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Z</t>
+        </is>
+      </c>
+      <c r="HW27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z</t>
+        </is>
+      </c>
+      <c r="HX27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z</t>
+        </is>
+      </c>
     </row>
     <row r="28" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="93" t="s">
@@ -47725,6 +48123,17 @@
         </is>
       </c>
       <c r="HU28">
+        <v>1</v>
+      </c>
+      <c r="HV28">
+        <v>1</v>
+      </c>
+      <c r="HW28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">!</t>
+        </is>
+      </c>
+      <c r="HX28">
         <v>1</v>
       </c>
     </row>
@@ -48359,6 +48768,17 @@
       <c r="HU29">
         <v>2</v>
       </c>
+      <c r="HV29">
+        <v>2</v>
+      </c>
+      <c r="HW29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIDDLE_DOT</t>
+        </is>
+      </c>
+      <c r="HX29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="93" t="s">
@@ -49018,6 +49438,17 @@
       <c r="HU30">
         <v>3</v>
       </c>
+      <c r="HV30">
+        <v>3</v>
+      </c>
+      <c r="HW30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LANGLE_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="93" t="s">
@@ -49667,6 +50098,17 @@
       <c r="HU31">
         <v>4</v>
       </c>
+      <c r="HV31">
+        <v>4</v>
+      </c>
+      <c r="HW31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YEN_SIGN</t>
+        </is>
+      </c>
+      <c r="HX31">
+        <v>4</v>
+      </c>
     </row>
     <row r="32" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="93" t="s">
@@ -50262,6 +50704,17 @@
       <c r="HU32">
         <v>5</v>
       </c>
+      <c r="HV32">
+        <v>5</v>
+      </c>
+      <c r="HW32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RANGLE_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="93" t="s">
@@ -50898,6 +51351,17 @@
       <c r="HU33">
         <v>6</v>
       </c>
+      <c r="HV33">
+        <v>6</v>
+      </c>
+      <c r="HW33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LWCORNER_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX33">
+        <v>6</v>
+      </c>
     </row>
     <row r="34" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="93" t="s">
@@ -51521,6 +51985,17 @@
         </is>
       </c>
       <c r="HU34">
+        <v>7</v>
+      </c>
+      <c r="HV34">
+        <v>7</v>
+      </c>
+      <c r="HW34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RWCORNER_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX34">
         <v>7</v>
       </c>
     </row>
@@ -52137,6 +52612,17 @@
       <c r="HU35">
         <v>8</v>
       </c>
+      <c r="HV35">
+        <v>8</v>
+      </c>
+      <c r="HW35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">u". . ."</t>
+        </is>
+      </c>
+      <c r="HX35">
+        <v>8</v>
+      </c>
     </row>
     <row r="36" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="93" t="s">
@@ -52749,6 +53235,17 @@
       <c r="HU36">
         <v>9</v>
       </c>
+      <c r="HV36">
+        <v>9</v>
+      </c>
+      <c r="HW36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(</t>
+        </is>
+      </c>
+      <c r="HX36">
+        <v>9</v>
+      </c>
     </row>
     <row r="37" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="93" t="s">
@@ -53396,6 +53893,17 @@
         <is>
           <t xml:space="preserve">ZERO</t>
         </is>
+      </c>
+      <c r="HV37">
+        <v>0</v>
+      </c>
+      <c r="HW37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">)</t>
+        </is>
+      </c>
+      <c r="HX37">
+        <v>0</v>
       </c>
     </row>
     <row r="38" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -54577,6 +55085,21 @@
           <t xml:space="preserve">UMLAUT_O</t>
         </is>
       </c>
+      <c r="HV43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICON_LEFT</t>
+        </is>
+      </c>
+      <c r="HW43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCORNER_BRKT</t>
+        </is>
+      </c>
+      <c r="HX43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICON_LEFT</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="93" t="s">
@@ -55171,6 +55694,21 @@
           <t xml:space="preserve">DONG_SIGN</t>
         </is>
       </c>
+      <c r="HV44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICON_RIGHT</t>
+        </is>
+      </c>
+      <c r="HW44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RCORNER_BRKT</t>
+        </is>
+      </c>
+      <c r="HX44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICON_RIGHT</t>
+        </is>
+      </c>
     </row>
     <row r="45" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="93" t="s">
@@ -55752,6 +56290,21 @@
           <t xml:space="preserve">LATIN_01AF</t>
         </is>
       </c>
+      <c r="HV45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
+      <c r="HW45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LLENTICULAR_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="93" t="s">
@@ -56354,6 +56907,21 @@
           <t xml:space="preserve">LATIN_01A0</t>
         </is>
       </c>
+      <c r="HV46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
+      <c r="HW46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RLENTICULAR_BRACKET</t>
+        </is>
+      </c>
+      <c r="HX46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">]</t>
+        </is>
+      </c>
     </row>
     <row r="47" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="93" t="s">
@@ -56864,6 +57432,21 @@
       <c r="HP47" t="inlineStr">
         <is>
           <t xml:space="preserve">+</t>
+        </is>
+      </c>
+      <c r="HV47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_IDEOG_COMMA</t>
+        </is>
+      </c>
+      <c r="HW47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_ONE</t>
+        </is>
+      </c>
+      <c r="HX47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_IDEOG_COMMA</t>
         </is>
       </c>
     </row>
@@ -57216,6 +57799,21 @@
           <t xml:space="preserve">+</t>
         </is>
       </c>
+      <c r="HV48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+      <c r="HW48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~</t>
+        </is>
+      </c>
+      <c r="HX48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
     </row>
     <row r="49" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="93" t="s">
@@ -57769,6 +58367,21 @@
       <c r="HO49" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_00C6</t>
+        </is>
+      </c>
+      <c r="HV49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">;</t>
+        </is>
+      </c>
+      <c r="HW49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">:</t>
+        </is>
+      </c>
+      <c r="HX49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">;</t>
         </is>
       </c>
     </row>
@@ -58365,6 +58978,21 @@
           <t xml:space="preserve">ACUTE_ACCENT</t>
         </is>
       </c>
+      <c r="HV50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
+      <c r="HW50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QUOTE</t>
+        </is>
+      </c>
+      <c r="HX50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'</t>
+        </is>
+      </c>
     </row>
     <row r="51" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="93" t="s">
@@ -58905,6 +59533,21 @@
       <c r="HP51" t="inlineStr">
         <is>
           <t xml:space="preserve">MOD_RING</t>
+        </is>
+      </c>
+      <c r="HV51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRAVE_ACCENT</t>
+        </is>
+      </c>
+      <c r="HW51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~</t>
+        </is>
+      </c>
+      <c r="HX51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRAVE_ACCENT</t>
         </is>
       </c>
     </row>
@@ -59362,6 +60005,21 @@
           <t xml:space="preserve">C_WITH_CEDILLA</t>
         </is>
       </c>
+      <c r="HV52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COMMA</t>
+        </is>
+      </c>
+      <c r="HW52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LANGLE_BRACKET_DBL</t>
+        </is>
+      </c>
+      <c r="HX52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COMMA</t>
+        </is>
+      </c>
     </row>
     <row r="53" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="93" t="s">
@@ -59796,6 +60454,16 @@
           <t xml:space="preserve">S_WITH_CEDILLA</t>
         </is>
       </c>
+      <c r="HV53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_IDEOG_FSTOP</t>
+        </is>
+      </c>
+      <c r="HW53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RANGLE_BRACKET_DBL</t>
+        </is>
+      </c>
     </row>
     <row r="54" s="116" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="93" t="s">
@@ -60254,6 +60922,21 @@
       <c r="HO54" t="inlineStr">
         <is>
           <t xml:space="preserve">LATIN_00DE</t>
+        </is>
+      </c>
+      <c r="HV54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
+        </is>
+      </c>
+      <c r="HW54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">?</t>
+        </is>
+      </c>
+      <c r="HX54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/</t>
         </is>
       </c>
     </row>
@@ -60691,6 +61374,21 @@
           <t xml:space="preserve">?</t>
         </is>
       </c>
+      <c r="HV55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_IDEOG_COMMA</t>
+        </is>
+      </c>
+      <c r="HW55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KANGXI_RADICAL_ONE</t>
+        </is>
+      </c>
+      <c r="HX55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_IDEOG_COMMA</t>
+        </is>
+      </c>
     </row>
     <row r="56" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="141" t="s">
@@ -61121,6 +61819,9 @@
       <c r="HU56">
         <v>50</v>
       </c>
+      <c r="HW56">
+        <v>42</v>
+      </c>
     </row>
     <row r="57" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="141" t="s">
@@ -61560,6 +62261,9 @@
       <c r="HU57">
         <v>13</v>
       </c>
+      <c r="HW57">
+        <v>10</v>
+      </c>
     </row>
     <row r="58" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="141" t="s">
@@ -61947,6 +62651,9 @@
       <c r="HU58">
         <v>50</v>
       </c>
+      <c r="HW58">
+        <v>34</v>
+      </c>
     </row>
     <row r="59" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="141" t="s">
@@ -62340,6 +63047,9 @@
       <c r="HU59">
         <v>13</v>
       </c>
+      <c r="HW59">
+        <v>10</v>
+      </c>
     </row>
     <row r="60" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="141" t="s">
@@ -62727,6 +63437,9 @@
       <c r="HU60">
         <v>50</v>
       </c>
+      <c r="HW60">
+        <v>34</v>
+      </c>
     </row>
     <row r="61" s="172" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="141" t="s">
@@ -63119,6 +63832,9 @@
       </c>
       <c r="HU61">
         <v>13</v>
+      </c>
+      <c r="HW61">
+        <v>10</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
polykybd: complete Cangjie set - add Z = 重 (U+91CD) to zh-CN/zh-HK
The Cangjie Z key was the only radical left as the Latin 'Z'. Add the
重 ideograph (U+91CD) as a single-codepoint NotoSansJP font (_Cjk91cd_,
matching the existing 中/廿/難 entries) and a CJK_91CD named glyph, then
map KC_Z base+caps to it for both the zh-CN and zh-HK Cangjie columns
(the Latin 'z' stays as the shift preview). Only jp_fonts.h and the
ALL_FONTS table change in the generated output.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -6068,7 +6068,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1563"/>
+  <dimension ref="A1:I1564"/>
   <sheetFormatPr defaultColWidth="12.5234375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="39.25"/>
@@ -37127,6 +37127,18 @@
       <c r="B1563" t="inlineStr">
         <is>
           <t xml:space="preserve">E1A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1564" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_91CD</t>
+        </is>
+      </c>
+      <c r="B1564" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91CD</t>
         </is>
       </c>
     </row>
@@ -47240,14 +47252,18 @@
       <c r="BS27" s="110"/>
       <c r="BT27" s="110"/>
       <c r="BU27" s="110"/>
-      <c r="BV27" s="83" t="s">
-        <v>1220</v>
+      <c r="BV27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_91CD</t>
+        </is>
       </c>
       <c r="BW27" s="84" t="s">
         <v>1219</v>
       </c>
-      <c r="BX27" s="83" t="s">
-        <v>1219</v>
+      <c r="BX27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CJK_91CD</t>
+        </is>
       </c>
       <c r="BY27" s="84"/>
       <c r="BZ27" s="111"/>
@@ -47523,7 +47539,7 @@
       </c>
       <c r="HV27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z</t>
+          <t xml:space="preserve">CJK_91CD</t>
         </is>
       </c>
       <c r="HW27" t="inlineStr">
@@ -47533,7 +47549,7 @@
       </c>
       <c r="HX27" t="inlineStr">
         <is>
-          <t xml:space="preserve">z</t>
+          <t xml:space="preserve">CJK_91CD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
polykybd: re-point zh-CN to Pinyin (plain US-QWERTY fold)
Mainland Chinese is typed with a Pinyin IME on a plain US-QWERTY board
(no Han glyphs on the keycaps), so empty zh-CN's key_lut column - it now
folds onto en-US like id-ID. The Cangjie radical legends now live solely
on zh-HK (Zhuyin on zh-TW), matching real-world keyboards. zh-CN stays a
selectable language (enum entry + flag); only its keycaps changed, so the
layout count stays 58. Host fold cn=us added separately in PolyKybdHost.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -37722,16 +37722,6 @@
       <c r="BS2" s="82"/>
       <c r="BT2" s="82"/>
       <c r="BU2" s="82"/>
-      <c r="BV2" s="83" t="s">
-        <v>767</v>
-      </c>
-      <c r="BW2" s="84" t="s">
-        <v>1130</v>
-      </c>
-      <c r="BX2" s="83" t="s">
-        <v>767</v>
-      </c>
-      <c r="BY2" s="83"/>
       <c r="BZ2" s="85"/>
       <c r="CA2" s="85"/>
       <c r="CB2" s="85"/>
@@ -38103,16 +38093,6 @@
       <c r="BS3" s="110"/>
       <c r="BT3" s="110"/>
       <c r="BU3" s="110"/>
-      <c r="BV3" s="83" t="s">
-        <v>769</v>
-      </c>
-      <c r="BW3" s="84" t="s">
-        <v>1135</v>
-      </c>
-      <c r="BX3" s="83" t="s">
-        <v>769</v>
-      </c>
-      <c r="BY3" s="84"/>
       <c r="BZ3" s="111"/>
       <c r="CA3" s="111"/>
       <c r="CB3" s="111"/>
@@ -38465,16 +38445,6 @@
       <c r="BU4" s="124" t="s">
         <v>62</v>
       </c>
-      <c r="BV4" s="83" t="s">
-        <v>781</v>
-      </c>
-      <c r="BW4" s="84" t="s">
-        <v>1139</v>
-      </c>
-      <c r="BX4" s="83" t="s">
-        <v>781</v>
-      </c>
-      <c r="BY4" s="84"/>
       <c r="BZ4" s="111"/>
       <c r="CA4" s="111"/>
       <c r="CB4" s="125" t="s">
@@ -38856,16 +38826,6 @@
       <c r="BU5" s="110" t="s">
         <v>1146</v>
       </c>
-      <c r="BV5" s="83" t="s">
-        <v>771</v>
-      </c>
-      <c r="BW5" s="84" t="s">
-        <v>1143</v>
-      </c>
-      <c r="BX5" s="83" t="s">
-        <v>771</v>
-      </c>
-      <c r="BY5" s="84"/>
       <c r="BZ5" s="111"/>
       <c r="CA5" s="111"/>
       <c r="CB5" s="111"/>
@@ -39246,16 +39206,6 @@
       <c r="BU6" s="110" t="s">
         <v>682</v>
       </c>
-      <c r="BV6" s="83" t="s">
-        <v>773</v>
-      </c>
-      <c r="BW6" s="84" t="s">
-        <v>1148</v>
-      </c>
-      <c r="BX6" s="83" t="s">
-        <v>773</v>
-      </c>
-      <c r="BY6" s="84"/>
       <c r="BZ6" s="111"/>
       <c r="CA6" s="111"/>
       <c r="CB6" s="111" t="s">
@@ -39701,16 +39651,6 @@
       <c r="BS7" s="110"/>
       <c r="BT7" s="110"/>
       <c r="BU7" s="110"/>
-      <c r="BV7" s="83" t="s">
-        <v>775</v>
-      </c>
-      <c r="BW7" s="84" t="s">
-        <v>1152</v>
-      </c>
-      <c r="BX7" s="83" t="s">
-        <v>775</v>
-      </c>
-      <c r="BY7" s="84"/>
       <c r="BZ7" s="111"/>
       <c r="CA7" s="111"/>
       <c r="CB7" s="111"/>
@@ -40070,16 +40010,6 @@
       <c r="BS8" s="110"/>
       <c r="BT8" s="110"/>
       <c r="BU8" s="110"/>
-      <c r="BV8" s="83" t="s">
-        <v>749</v>
-      </c>
-      <c r="BW8" s="84" t="s">
-        <v>1156</v>
-      </c>
-      <c r="BX8" s="83" t="s">
-        <v>749</v>
-      </c>
-      <c r="BY8" s="84"/>
       <c r="BZ8" s="111"/>
       <c r="CA8" s="111"/>
       <c r="CB8" s="111"/>
@@ -40450,16 +40380,6 @@
       <c r="BS9" s="110"/>
       <c r="BT9" s="110"/>
       <c r="BU9" s="110"/>
-      <c r="BV9" s="83" t="s">
-        <v>779</v>
-      </c>
-      <c r="BW9" s="84" t="s">
-        <v>1159</v>
-      </c>
-      <c r="BX9" s="83" t="s">
-        <v>779</v>
-      </c>
-      <c r="BY9" s="84"/>
       <c r="BZ9" s="111"/>
       <c r="CA9" s="111"/>
       <c r="CB9" s="111"/>
@@ -40817,16 +40737,6 @@
       <c r="BS10" s="110"/>
       <c r="BT10" s="110"/>
       <c r="BU10" s="110"/>
-      <c r="BV10" s="83" t="s">
-        <v>763</v>
-      </c>
-      <c r="BW10" s="84" t="s">
-        <v>1162</v>
-      </c>
-      <c r="BX10" s="83" t="s">
-        <v>763</v>
-      </c>
-      <c r="BY10" s="84"/>
       <c r="BZ10" s="111"/>
       <c r="CA10" s="111"/>
       <c r="CB10" s="111"/>
@@ -41187,16 +41097,6 @@
       <c r="BS11" s="110"/>
       <c r="BT11" s="110"/>
       <c r="BU11" s="110"/>
-      <c r="BV11" s="83" t="s">
-        <v>743</v>
-      </c>
-      <c r="BW11" s="84" t="s">
-        <v>1165</v>
-      </c>
-      <c r="BX11" s="83" t="s">
-        <v>743</v>
-      </c>
-      <c r="BY11" s="84"/>
       <c r="BZ11" s="111"/>
       <c r="CA11" s="111"/>
       <c r="CB11" s="111"/>
@@ -41557,16 +41457,6 @@
       <c r="BS12" s="110"/>
       <c r="BT12" s="110"/>
       <c r="BU12" s="110"/>
-      <c r="BV12" s="83" t="s">
-        <v>751</v>
-      </c>
-      <c r="BW12" s="84" t="s">
-        <v>1168</v>
-      </c>
-      <c r="BX12" s="83" t="s">
-        <v>751</v>
-      </c>
-      <c r="BY12" s="84"/>
       <c r="BZ12" s="111"/>
       <c r="CA12" s="111"/>
       <c r="CB12" s="111"/>
@@ -41927,16 +41817,6 @@
       <c r="BU13" s="110" t="s">
         <v>1174</v>
       </c>
-      <c r="BV13" s="129" t="s">
-        <v>938</v>
-      </c>
-      <c r="BW13" s="84" t="s">
-        <v>1172</v>
-      </c>
-      <c r="BX13" s="129" t="s">
-        <v>938</v>
-      </c>
-      <c r="BY13" s="84"/>
       <c r="BZ13" s="111"/>
       <c r="CA13" s="111"/>
       <c r="CB13" s="111"/>
@@ -42303,16 +42183,6 @@
       <c r="BS14" s="110"/>
       <c r="BT14" s="110"/>
       <c r="BU14" s="110"/>
-      <c r="BV14" s="83" t="s">
-        <v>739</v>
-      </c>
-      <c r="BW14" s="84" t="s">
-        <v>1176</v>
-      </c>
-      <c r="BX14" s="83" t="s">
-        <v>739</v>
-      </c>
-      <c r="BY14" s="84"/>
       <c r="BZ14" s="111"/>
       <c r="CA14" s="111"/>
       <c r="CB14" s="111"/>
@@ -42693,16 +42563,6 @@
       <c r="BS15" s="110"/>
       <c r="BT15" s="110"/>
       <c r="BU15" s="110"/>
-      <c r="BV15" s="83" t="s">
-        <v>759</v>
-      </c>
-      <c r="BW15" s="84" t="s">
-        <v>1183</v>
-      </c>
-      <c r="BX15" s="83" t="s">
-        <v>759</v>
-      </c>
-      <c r="BY15" s="84"/>
       <c r="BZ15" s="111"/>
       <c r="CA15" s="111"/>
       <c r="CB15" s="111"/>
@@ -43068,16 +42928,6 @@
       <c r="BS16" s="110"/>
       <c r="BT16" s="110"/>
       <c r="BU16" s="110"/>
-      <c r="BV16" s="83" t="s">
-        <v>741</v>
-      </c>
-      <c r="BW16" s="84" t="s">
-        <v>1187</v>
-      </c>
-      <c r="BX16" s="83" t="s">
-        <v>741</v>
-      </c>
-      <c r="BY16" s="84"/>
       <c r="BZ16" s="111"/>
       <c r="CA16" s="111"/>
       <c r="CB16" s="111"/>
@@ -43425,16 +43275,6 @@
       <c r="BU17" s="124" t="s">
         <v>57</v>
       </c>
-      <c r="BV17" s="83" t="s">
-        <v>761</v>
-      </c>
-      <c r="BW17" s="84" t="s">
-        <v>1190</v>
-      </c>
-      <c r="BX17" s="83" t="s">
-        <v>761</v>
-      </c>
-      <c r="BY17" s="84"/>
       <c r="BZ17" s="111"/>
       <c r="CA17" s="111"/>
       <c r="CB17" s="111"/>
@@ -43800,16 +43640,6 @@
       <c r="BS18" s="110"/>
       <c r="BT18" s="110"/>
       <c r="BU18" s="110"/>
-      <c r="BV18" s="83" t="s">
-        <v>765</v>
-      </c>
-      <c r="BW18" s="84" t="s">
-        <v>1132</v>
-      </c>
-      <c r="BX18" s="83" t="s">
-        <v>765</v>
-      </c>
-      <c r="BY18" s="84"/>
       <c r="BZ18" s="111"/>
       <c r="CA18" s="111"/>
       <c r="CB18" s="111"/>
@@ -44201,16 +44031,6 @@
       <c r="BS19" s="110"/>
       <c r="BT19" s="110"/>
       <c r="BU19" s="110"/>
-      <c r="BV19" s="83" t="s">
-        <v>747</v>
-      </c>
-      <c r="BW19" s="84" t="s">
-        <v>1201</v>
-      </c>
-      <c r="BX19" s="83" t="s">
-        <v>747</v>
-      </c>
-      <c r="BY19" s="84"/>
       <c r="BZ19" s="111"/>
       <c r="CA19" s="111"/>
       <c r="CB19" s="111"/>
@@ -44576,16 +44396,6 @@
       <c r="BU20" s="124" t="s">
         <v>135</v>
       </c>
-      <c r="BV20" s="83" t="s">
-        <v>755</v>
-      </c>
-      <c r="BW20" s="84" t="s">
-        <v>1205</v>
-      </c>
-      <c r="BX20" s="83" t="s">
-        <v>755</v>
-      </c>
-      <c r="BY20" s="84"/>
       <c r="BZ20" s="111"/>
       <c r="CA20" s="111"/>
       <c r="CB20" s="111"/>
@@ -44959,16 +44769,6 @@
       <c r="BS21" s="110"/>
       <c r="BT21" s="110"/>
       <c r="BU21" s="110"/>
-      <c r="BV21" s="129" t="s">
-        <v>941</v>
-      </c>
-      <c r="BW21" s="84" t="s">
-        <v>1209</v>
-      </c>
-      <c r="BX21" s="129" t="s">
-        <v>941</v>
-      </c>
-      <c r="BY21" s="84"/>
       <c r="BZ21" s="111"/>
       <c r="CA21" s="111"/>
       <c r="CB21" s="111"/>
@@ -45334,16 +45134,6 @@
       <c r="BS22" s="110"/>
       <c r="BT22" s="110"/>
       <c r="BU22" s="110"/>
-      <c r="BV22" s="83" t="s">
-        <v>757</v>
-      </c>
-      <c r="BW22" s="84" t="s">
-        <v>1211</v>
-      </c>
-      <c r="BX22" s="83" t="s">
-        <v>757</v>
-      </c>
-      <c r="BY22" s="84"/>
       <c r="BZ22" s="111"/>
       <c r="CA22" s="111"/>
       <c r="CB22" s="111"/>
@@ -45711,16 +45501,6 @@
       <c r="BS23" s="110"/>
       <c r="BT23" s="110"/>
       <c r="BU23" s="110"/>
-      <c r="BV23" s="83" t="s">
-        <v>753</v>
-      </c>
-      <c r="BW23" s="84" t="s">
-        <v>1214</v>
-      </c>
-      <c r="BX23" s="83" t="s">
-        <v>753</v>
-      </c>
-      <c r="BY23" s="84"/>
       <c r="BZ23" s="111"/>
       <c r="CA23" s="111"/>
       <c r="CB23" s="111"/>
@@ -46079,16 +45859,6 @@
       <c r="BS24" s="110"/>
       <c r="BT24" s="110"/>
       <c r="BU24" s="110"/>
-      <c r="BV24" s="83" t="s">
-        <v>777</v>
-      </c>
-      <c r="BW24" s="84" t="s">
-        <v>1217</v>
-      </c>
-      <c r="BX24" s="83" t="s">
-        <v>777</v>
-      </c>
-      <c r="BY24" s="84"/>
       <c r="BZ24" s="111"/>
       <c r="CA24" s="111"/>
       <c r="CB24" s="111"/>
@@ -46481,16 +46251,6 @@
       <c r="BS25" s="110"/>
       <c r="BT25" s="110"/>
       <c r="BU25" s="110"/>
-      <c r="BV25" s="129" t="s">
-        <v>944</v>
-      </c>
-      <c r="BW25" s="84" t="s">
-        <v>1226</v>
-      </c>
-      <c r="BX25" s="129" t="s">
-        <v>944</v>
-      </c>
-      <c r="BY25" s="84"/>
       <c r="BZ25" s="111"/>
       <c r="CA25" s="111"/>
       <c r="CB25" s="111"/>
@@ -46851,16 +46611,6 @@
       <c r="BS26" s="110"/>
       <c r="BT26" s="110"/>
       <c r="BU26" s="110"/>
-      <c r="BV26" s="83" t="s">
-        <v>745</v>
-      </c>
-      <c r="BW26" s="84" t="s">
-        <v>1230</v>
-      </c>
-      <c r="BX26" s="83" t="s">
-        <v>745</v>
-      </c>
-      <c r="BY26" s="84"/>
       <c r="BZ26" s="111"/>
       <c r="CA26" s="111"/>
       <c r="CB26" s="111"/>
@@ -47252,20 +47002,6 @@
       <c r="BS27" s="110"/>
       <c r="BT27" s="110"/>
       <c r="BU27" s="110"/>
-      <c r="BV27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CJK_91CD</t>
-        </is>
-      </c>
-      <c r="BW27" s="84" t="s">
-        <v>1219</v>
-      </c>
-      <c r="BX27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CJK_91CD</t>
-        </is>
-      </c>
-      <c r="BY27" s="84"/>
       <c r="BZ27" s="111"/>
       <c r="CA27" s="111"/>
       <c r="CB27" s="111"/>
@@ -47735,16 +47471,6 @@
       <c r="BU28" s="110" t="s">
         <v>198</v>
       </c>
-      <c r="BV28" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="BW28" s="84" t="s">
-        <v>1236</v>
-      </c>
-      <c r="BX28" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY28" s="84"/>
       <c r="BZ28" s="111" t="n">
         <v>1</v>
       </c>
@@ -48343,16 +48069,6 @@
       <c r="BU29" s="110" t="s">
         <v>1241</v>
       </c>
-      <c r="BV29" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="BW29" s="131" t="s">
-        <v>86</v>
-      </c>
-      <c r="BX29" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="BY29" s="84"/>
       <c r="BZ29" s="111" t="n">
         <v>2</v>
       </c>
@@ -48988,16 +48704,6 @@
       <c r="BU30" s="110" t="s">
         <v>1245</v>
       </c>
-      <c r="BV30" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW30" s="131" t="s">
-        <v>785</v>
-      </c>
-      <c r="BX30" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="BY30" s="84"/>
       <c r="BZ30" s="111" t="n">
         <v>3</v>
       </c>
@@ -49658,16 +49364,6 @@
       <c r="BU31" s="110" t="s">
         <v>190</v>
       </c>
-      <c r="BV31" s="84" t="n">
-        <v>4</v>
-      </c>
-      <c r="BW31" s="131" t="s">
-        <v>53</v>
-      </c>
-      <c r="BX31" s="84" t="n">
-        <v>4</v>
-      </c>
-      <c r="BY31" s="84"/>
       <c r="BZ31" s="132" t="s">
         <v>1252</v>
       </c>
@@ -50318,16 +50014,6 @@
       <c r="BU32" s="110" t="s">
         <v>194</v>
       </c>
-      <c r="BV32" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="BW32" s="131" t="s">
-        <v>787</v>
-      </c>
-      <c r="BX32" s="84" t="n">
-        <v>5</v>
-      </c>
-      <c r="BY32" s="84"/>
       <c r="BZ32" s="132" t="s">
         <v>1259</v>
       </c>
@@ -50920,16 +50606,6 @@
       <c r="BU33" s="124" t="s">
         <v>196</v>
       </c>
-      <c r="BV33" s="84" t="n">
-        <v>6</v>
-      </c>
-      <c r="BW33" s="131" t="s">
-        <v>797</v>
-      </c>
-      <c r="BX33" s="84" t="n">
-        <v>6</v>
-      </c>
-      <c r="BY33" s="84"/>
       <c r="BZ33" s="111" t="n">
         <v>6</v>
       </c>
@@ -51569,16 +51245,6 @@
       <c r="BU34" s="110" t="s">
         <v>1268</v>
       </c>
-      <c r="BV34" s="84" t="n">
-        <v>7</v>
-      </c>
-      <c r="BW34" s="131" t="s">
-        <v>799</v>
-      </c>
-      <c r="BX34" s="84" t="n">
-        <v>7</v>
-      </c>
-      <c r="BY34" s="84"/>
       <c r="BZ34" s="111" t="n">
         <v>7</v>
       </c>
@@ -52205,16 +51871,6 @@
       <c r="BU35" s="124" t="s">
         <v>192</v>
       </c>
-      <c r="BV35" s="84" t="n">
-        <v>8</v>
-      </c>
-      <c r="BW35" s="84" t="s">
-        <v>1273</v>
-      </c>
-      <c r="BX35" s="84" t="n">
-        <v>8</v>
-      </c>
-      <c r="BY35" s="84"/>
       <c r="BZ35" s="111" t="n">
         <v>8</v>
       </c>
@@ -52830,16 +52486,6 @@
       <c r="BU36" s="124" t="s">
         <v>80</v>
       </c>
-      <c r="BV36" s="84" t="n">
-        <v>9</v>
-      </c>
-      <c r="BW36" s="84" t="s">
-        <v>1257</v>
-      </c>
-      <c r="BX36" s="84" t="n">
-        <v>9</v>
-      </c>
-      <c r="BY36" s="84"/>
       <c r="BZ36" s="111" t="n">
         <v>9</v>
       </c>
@@ -53453,16 +53099,6 @@
       <c r="BU37" s="124" t="s">
         <v>200</v>
       </c>
-      <c r="BV37" s="84" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW37" s="84" t="s">
-        <v>1276</v>
-      </c>
-      <c r="BX37" s="84" t="n">
-        <v>0</v>
-      </c>
-      <c r="BY37" s="84"/>
       <c r="BZ37" s="111" t="s">
         <v>12</v>
       </c>
@@ -54000,10 +53636,6 @@
       <c r="BS38" s="110"/>
       <c r="BT38" s="110"/>
       <c r="BU38" s="110"/>
-      <c r="BV38" s="84"/>
-      <c r="BW38" s="84"/>
-      <c r="BX38" s="84"/>
-      <c r="BY38" s="84"/>
       <c r="BZ38" s="111"/>
       <c r="CA38" s="111"/>
       <c r="CB38" s="111"/>
@@ -54115,10 +53747,6 @@
       <c r="BS39" s="110"/>
       <c r="BT39" s="110"/>
       <c r="BU39" s="110"/>
-      <c r="BV39" s="84"/>
-      <c r="BW39" s="84"/>
-      <c r="BX39" s="84"/>
-      <c r="BY39" s="84"/>
       <c r="BZ39" s="111"/>
       <c r="CA39" s="111"/>
       <c r="CB39" s="111"/>
@@ -54230,10 +53858,6 @@
       <c r="BS40" s="110"/>
       <c r="BT40" s="110"/>
       <c r="BU40" s="110"/>
-      <c r="BV40" s="84"/>
-      <c r="BW40" s="84"/>
-      <c r="BX40" s="84"/>
-      <c r="BY40" s="84"/>
       <c r="BZ40" s="111"/>
       <c r="CA40" s="111"/>
       <c r="CB40" s="111"/>
@@ -54345,10 +53969,6 @@
       <c r="BS41" s="110"/>
       <c r="BT41" s="110"/>
       <c r="BU41" s="110"/>
-      <c r="BV41" s="84"/>
-      <c r="BW41" s="84"/>
-      <c r="BX41" s="84"/>
-      <c r="BY41" s="84"/>
       <c r="BZ41" s="111"/>
       <c r="CA41" s="111"/>
       <c r="CB41" s="111"/>
@@ -54460,10 +54080,6 @@
       <c r="BS42" s="110"/>
       <c r="BT42" s="110"/>
       <c r="BU42" s="110"/>
-      <c r="BV42" s="84"/>
-      <c r="BW42" s="84"/>
-      <c r="BX42" s="84"/>
-      <c r="BY42" s="84"/>
       <c r="BZ42" s="111"/>
       <c r="CA42" s="111"/>
       <c r="CB42" s="111"/>
@@ -54659,16 +54275,6 @@
       <c r="BU43" s="124" t="s">
         <v>1291</v>
       </c>
-      <c r="BV43" s="84" t="s">
-        <v>22</v>
-      </c>
-      <c r="BW43" s="131" t="s">
-        <v>793</v>
-      </c>
-      <c r="BX43" s="84" t="s">
-        <v>22</v>
-      </c>
-      <c r="BY43" s="84"/>
       <c r="BZ43" s="111" t="s">
         <v>1173</v>
       </c>
@@ -55293,16 +54899,6 @@
       <c r="BU44" s="110" t="s">
         <v>1294</v>
       </c>
-      <c r="BV44" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="BW44" s="84" t="s">
-        <v>795</v>
-      </c>
-      <c r="BX44" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="BY44" s="84"/>
       <c r="BZ44" s="125" t="s">
         <v>72</v>
       </c>
@@ -55900,16 +55496,6 @@
       <c r="BU45" s="110" t="s">
         <v>1302</v>
       </c>
-      <c r="BV45" s="84" t="s">
-        <v>1154</v>
-      </c>
-      <c r="BW45" s="84" t="s">
-        <v>801</v>
-      </c>
-      <c r="BX45" s="84" t="s">
-        <v>1154</v>
-      </c>
-      <c r="BY45" s="84"/>
       <c r="BZ45" s="125" t="s">
         <v>59</v>
       </c>
@@ -56496,16 +56082,6 @@
       <c r="BU46" s="110" t="s">
         <v>1310</v>
       </c>
-      <c r="BV46" s="84" t="s">
-        <v>1145</v>
-      </c>
-      <c r="BW46" s="84" t="s">
-        <v>803</v>
-      </c>
-      <c r="BX46" s="84" t="s">
-        <v>1145</v>
-      </c>
-      <c r="BY46" s="131"/>
       <c r="BZ46" s="111" t="s">
         <v>1272</v>
       </c>
@@ -57109,16 +56685,6 @@
       <c r="BU47" s="124" t="s">
         <v>1320</v>
       </c>
-      <c r="BV47" s="84" t="s">
-        <v>783</v>
-      </c>
-      <c r="BW47" s="84" t="s">
-        <v>739</v>
-      </c>
-      <c r="BX47" s="84" t="s">
-        <v>783</v>
-      </c>
-      <c r="BY47" s="131"/>
       <c r="BZ47" s="111" t="s">
         <v>1181</v>
       </c>
@@ -57552,16 +57118,6 @@
       <c r="BS48" s="110"/>
       <c r="BT48" s="110"/>
       <c r="BU48" s="110"/>
-      <c r="BV48" s="84" t="s">
-        <v>1228</v>
-      </c>
-      <c r="BW48" s="84" t="s">
-        <v>1234</v>
-      </c>
-      <c r="BX48" s="84" t="s">
-        <v>1228</v>
-      </c>
-      <c r="BY48" s="84"/>
       <c r="BZ48" s="111"/>
       <c r="CA48" s="111"/>
       <c r="CB48" s="111"/>
@@ -57993,16 +57549,6 @@
       <c r="BU49" s="110" t="s">
         <v>1326</v>
       </c>
-      <c r="BV49" s="84" t="s">
-        <v>1197</v>
-      </c>
-      <c r="BW49" s="84" t="s">
-        <v>1198</v>
-      </c>
-      <c r="BX49" s="84" t="s">
-        <v>1197</v>
-      </c>
-      <c r="BY49" s="84"/>
       <c r="BZ49" s="111" t="s">
         <v>1237</v>
       </c>
@@ -58567,16 +58113,6 @@
       <c r="BU50" s="110" t="s">
         <v>1336</v>
       </c>
-      <c r="BV50" s="84" t="s">
-        <v>1222</v>
-      </c>
-      <c r="BW50" s="84" t="s">
-        <v>8</v>
-      </c>
-      <c r="BX50" s="84" t="s">
-        <v>1222</v>
-      </c>
-      <c r="BY50" s="84"/>
       <c r="BZ50" s="111" t="s">
         <v>1268</v>
       </c>
@@ -59184,16 +58720,6 @@
       <c r="BU51" s="110" t="s">
         <v>1344</v>
       </c>
-      <c r="BV51" s="84" t="s">
-        <v>18</v>
-      </c>
-      <c r="BW51" s="84" t="s">
-        <v>1234</v>
-      </c>
-      <c r="BX51" s="84" t="s">
-        <v>18</v>
-      </c>
-      <c r="BY51" s="131"/>
       <c r="BZ51" s="111" t="s">
         <v>1195</v>
       </c>
@@ -59733,16 +59259,6 @@
       <c r="BU52" s="110" t="s">
         <v>1347</v>
       </c>
-      <c r="BV52" s="84" t="s">
-        <v>10</v>
-      </c>
-      <c r="BW52" s="84" t="s">
-        <v>789</v>
-      </c>
-      <c r="BX52" s="84" t="s">
-        <v>10</v>
-      </c>
-      <c r="BY52" s="84"/>
       <c r="BZ52" s="111" t="s">
         <v>1179</v>
       </c>
@@ -60203,14 +59719,6 @@
       <c r="BU53" s="110" t="s">
         <v>1349</v>
       </c>
-      <c r="BV53" s="84" t="s">
-        <v>784</v>
-      </c>
-      <c r="BW53" s="84" t="s">
-        <v>791</v>
-      </c>
-      <c r="BX53" s="84"/>
-      <c r="BY53" s="84"/>
       <c r="BZ53" s="111" t="s">
         <v>1267</v>
       </c>
@@ -60655,16 +60163,6 @@
         <v>1173</v>
       </c>
       <c r="BU54" s="110"/>
-      <c r="BV54" s="84" t="s">
-        <v>1173</v>
-      </c>
-      <c r="BW54" s="84" t="s">
-        <v>1180</v>
-      </c>
-      <c r="BX54" s="84" t="s">
-        <v>1173</v>
-      </c>
-      <c r="BY54" s="84"/>
       <c r="BZ54" s="111" t="s">
         <v>1262</v>
       </c>
@@ -61082,16 +60580,6 @@
         <v>16</v>
       </c>
       <c r="BU55" s="162"/>
-      <c r="BV55" s="131" t="s">
-        <v>783</v>
-      </c>
-      <c r="BW55" s="131" t="s">
-        <v>739</v>
-      </c>
-      <c r="BX55" s="131" t="s">
-        <v>783</v>
-      </c>
-      <c r="BY55" s="163"/>
       <c r="BZ55" s="164" t="s">
         <v>1145</v>
       </c>
@@ -61548,12 +61036,6 @@
       <c r="BU56" s="162" t="n">
         <v>48</v>
       </c>
-      <c r="BV56" s="163"/>
-      <c r="BW56" s="163" t="n">
-        <v>42</v>
-      </c>
-      <c r="BX56" s="163"/>
-      <c r="BY56" s="163"/>
       <c r="BZ56" s="164"/>
       <c r="CA56" s="164" t="s">
         <v>1354</v>
@@ -61981,12 +61463,6 @@
       <c r="BU57" s="162" t="n">
         <v>12</v>
       </c>
-      <c r="BV57" s="163"/>
-      <c r="BW57" s="163" t="n">
-        <v>10</v>
-      </c>
-      <c r="BX57" s="163"/>
-      <c r="BY57" s="163"/>
       <c r="BZ57" s="164"/>
       <c r="CA57" s="164" t="s">
         <v>1354</v>
@@ -62423,12 +61899,6 @@
       <c r="BU58" s="162" t="n">
         <v>50</v>
       </c>
-      <c r="BV58" s="163"/>
-      <c r="BW58" s="163" t="n">
-        <v>34</v>
-      </c>
-      <c r="BX58" s="163"/>
-      <c r="BY58" s="163"/>
       <c r="BZ58" s="164"/>
       <c r="CA58" s="164" t="n">
         <v>28</v>
@@ -62813,12 +62283,6 @@
       <c r="BU59" s="162" t="n">
         <v>12</v>
       </c>
-      <c r="BV59" s="163"/>
-      <c r="BW59" s="163" t="n">
-        <v>10</v>
-      </c>
-      <c r="BX59" s="163"/>
-      <c r="BY59" s="163"/>
       <c r="BZ59" s="164"/>
       <c r="CA59" s="164" t="n">
         <v>0</v>
@@ -63209,12 +62673,6 @@
       <c r="BU60" s="162" t="n">
         <v>48</v>
       </c>
-      <c r="BV60" s="163"/>
-      <c r="BW60" s="163" t="n">
-        <v>34</v>
-      </c>
-      <c r="BX60" s="163"/>
-      <c r="BY60" s="163"/>
       <c r="BZ60" s="164"/>
       <c r="CA60" s="164" t="n">
         <v>28</v>
@@ -63599,12 +63057,6 @@
       <c r="BU61" s="162" t="n">
         <v>12</v>
       </c>
-      <c r="BV61" s="163"/>
-      <c r="BW61" s="163" t="n">
-        <v>10</v>
-      </c>
-      <c r="BX61" s="163"/>
-      <c r="BY61" s="163"/>
       <c r="BZ61" s="164"/>
       <c r="CA61" s="164" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
polykybd: fix zh-CN fold rendering + add zh-TW number hints
zh-CN/id-ID: emptying the column for the en-US fold also wiped the
settings rows, but get_setting() has no en-US fallback (only glyphs do),
so the letter shift-preview was drawn at offset 0 - right on top of the
base. Copy en-US's settings verbatim (letter hoff/voff SHIFT=HIDE,
num/sym hoff SHIFT=35) so the fold renders pixel-identical to en-US:
lowercase-only letters, offset !/@/# previews on the number/symbol row.

zh-TW: the number keys had the AltGr digit-hint position configured
(num hoff/voff ALTGR=50/12) but no AltGr glyph, so no digit showed.
Populate KC_1..KC_0 ALTGR with 1..9 + ZERO (same as th-TH/vi-VN), so the
Bopomofo number row now shows the digit in the corner.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -47841,6 +47841,9 @@
           <t xml:space="preserve">ZHUYIN_3105</t>
         </is>
       </c>
+      <c r="GW28">
+        <v>1</v>
+      </c>
       <c r="HB28" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0586</t>
@@ -48452,6 +48455,9 @@
           <t xml:space="preserve">ZHUYIN_3109</t>
         </is>
       </c>
+      <c r="GW29">
+        <v>2</v>
+      </c>
       <c r="HB29" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0571</t>
@@ -49118,6 +49124,9 @@
           <t xml:space="preserve">ZHUYIN_02C7</t>
         </is>
       </c>
+      <c r="GW30">
+        <v>3</v>
+      </c>
       <c r="HB30" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_058A</t>
@@ -49768,6 +49777,9 @@
           <t xml:space="preserve">ZHUYIN_02CB</t>
         </is>
       </c>
+      <c r="GW31">
+        <v>4</v>
+      </c>
       <c r="HB31" t="inlineStr">
         <is>
           <t xml:space="preserve">COMMA</t>
@@ -50370,6 +50382,9 @@
           <t xml:space="preserve">ZHUYIN_3113</t>
         </is>
       </c>
+      <c r="GW32">
+        <v>5</v>
+      </c>
       <c r="HB32" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_0589</t>
@@ -50996,6 +51011,9 @@
           <t xml:space="preserve">ZHUYIN_02CA</t>
         </is>
       </c>
+      <c r="GW33">
+        <v>6</v>
+      </c>
       <c r="HB33" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_055E</t>
@@ -51621,6 +51639,9 @@
         <is>
           <t xml:space="preserve">ZHUYIN_02D9</t>
         </is>
+      </c>
+      <c r="GW34">
+        <v>7</v>
       </c>
       <c r="HB34" t="inlineStr">
         <is>
@@ -52248,6 +52269,9 @@
           <t xml:space="preserve">ZHUYIN_311A</t>
         </is>
       </c>
+      <c r="GW35">
+        <v>8</v>
+      </c>
       <c r="HB35" t="inlineStr">
         <is>
           <t xml:space="preserve">ARMENIAN_055B</t>
@@ -52861,6 +52885,9 @@
           <t xml:space="preserve">ZHUYIN_311E</t>
         </is>
       </c>
+      <c r="GW36">
+        <v>9</v>
+      </c>
       <c r="HB36" t="inlineStr">
         <is>
           <t xml:space="preserve">)</t>
@@ -53514,6 +53541,11 @@
       <c r="GV37" t="inlineStr">
         <is>
           <t xml:space="preserve">ZHUYIN_3122</t>
+        </is>
+      </c>
+      <c r="GW37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZERO</t>
         </is>
       </c>
       <c r="HB37" t="inlineStr">
@@ -61036,6 +61068,11 @@
       <c r="BU56" s="162" t="n">
         <v>48</v>
       </c>
+      <c r="BW56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
       <c r="BZ56" s="164"/>
       <c r="CA56" s="164" t="s">
         <v>1354</v>
@@ -61292,6 +61329,11 @@
       </c>
       <c r="HE56">
         <v>50</v>
+      </c>
+      <c r="HG56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
       </c>
       <c r="HK56" t="inlineStr">
         <is>
@@ -61463,6 +61505,11 @@
       <c r="BU57" s="162" t="n">
         <v>12</v>
       </c>
+      <c r="BW57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
+      </c>
       <c r="BZ57" s="164"/>
       <c r="CA57" s="164" t="s">
         <v>1354</v>
@@ -61728,6 +61775,11 @@
       </c>
       <c r="HE57">
         <v>12</v>
+      </c>
+      <c r="HG57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIDE</t>
+        </is>
       </c>
       <c r="HK57" t="inlineStr">
         <is>
@@ -61899,6 +61951,9 @@
       <c r="BU58" s="162" t="n">
         <v>50</v>
       </c>
+      <c r="BW58">
+        <v>35</v>
+      </c>
       <c r="BZ58" s="164"/>
       <c r="CA58" s="164" t="n">
         <v>28</v>
@@ -62118,6 +62173,9 @@
       </c>
       <c r="HE58">
         <v>50</v>
+      </c>
+      <c r="HG58">
+        <v>35</v>
       </c>
       <c r="HK58">
         <v>28</v>
@@ -62283,6 +62341,9 @@
       <c r="BU59" s="162" t="n">
         <v>12</v>
       </c>
+      <c r="BW59">
+        <v>0</v>
+      </c>
       <c r="BZ59" s="164"/>
       <c r="CA59" s="164" t="n">
         <v>0</v>
@@ -62508,6 +62569,9 @@
       </c>
       <c r="HE59">
         <v>12</v>
+      </c>
+      <c r="HG59">
+        <v>0</v>
       </c>
       <c r="HK59">
         <v>0</v>
@@ -62673,6 +62737,9 @@
       <c r="BU60" s="162" t="n">
         <v>48</v>
       </c>
+      <c r="BW60">
+        <v>35</v>
+      </c>
       <c r="BZ60" s="164"/>
       <c r="CA60" s="164" t="n">
         <v>28</v>
@@ -62892,6 +62959,9 @@
       </c>
       <c r="HE60">
         <v>50</v>
+      </c>
+      <c r="HG60">
+        <v>35</v>
       </c>
       <c r="HK60">
         <v>28</v>
@@ -63057,6 +63127,9 @@
       <c r="BU61" s="162" t="n">
         <v>12</v>
       </c>
+      <c r="BW61">
+        <v>0</v>
+      </c>
       <c r="BZ61" s="164"/>
       <c r="CA61" s="164" t="n">
         <v>0</v>
@@ -63282,6 +63355,9 @@
       </c>
       <c r="HE61">
         <v>12</v>
+      </c>
+      <c r="HG61">
+        <v>0</v>
       </c>
       <c r="HK61">
         <v>0</v>

</xml_diff>

<commit_message>
polykybd: zh-TW - shrink Bopomofo font to 16pt + nudge glyphs down
Some Bopomofo glyphs clipped at the top of the keycap. Reduce the
bopomofo category font 18->16 pt (fonts.yaml) and set zh-TW's base
voffset (letter/num/sym SMALL) to +3 so the glyphs sit lower. The
number-row digit hints (num.voff ALTGR) are unaffected. Only
bopomofo_fonts.h + the ALL_FONTS table change in generated output.
</commit_message>
<xml_diff>
--- a/keyboards/handwired/polykybd/lang/lang_lut.xlsx
+++ b/keyboards/handwired/polykybd/lang/lang_lut.xlsx
@@ -61746,6 +61746,9 @@
       <c r="GS57">
         <v>13</v>
       </c>
+      <c r="GT57">
+        <v>3</v>
+      </c>
       <c r="GU57" t="inlineStr">
         <is>
           <t xml:space="preserve">HIDE</t>
@@ -62549,6 +62552,9 @@
       <c r="GS59">
         <v>13</v>
       </c>
+      <c r="GT59">
+        <v>3</v>
+      </c>
       <c r="GU59">
         <v>0</v>
       </c>
@@ -63334,6 +63340,9 @@
       </c>
       <c r="GS61">
         <v>13</v>
+      </c>
+      <c r="GT61">
+        <v>3</v>
       </c>
       <c r="GU61">
         <v>0</v>

</xml_diff>